<commit_message>
feat: release expanded exercise catalog and tracking
</commit_message>
<xml_diff>
--- a/tools/source_data/baza_cwiczen_316.xlsx
+++ b/tools/source_data/baza_cwiczen_316.xlsx
@@ -813,7 +813,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="24" customHeight="1" s="39">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -965,7 +964,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="24" customHeight="1" s="39">
       <c r="A22" s="4" t="inlineStr">
         <is>
@@ -1165,7 +1163,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40" ht="24" customHeight="1" s="39">
       <c r="A40" s="4" t="inlineStr">
         <is>
@@ -1269,7 +1266,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50" ht="24" customHeight="1" s="39">
       <c r="A50" s="4" t="inlineStr">
         <is>
@@ -1340,7 +1336,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58" ht="24" customHeight="1" s="39">
       <c r="A58" s="4" t="inlineStr">
         <is>
@@ -1384,7 +1379,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63" ht="24" customHeight="1" s="39">
       <c r="A63" s="4" t="inlineStr">
         <is>
@@ -1476,7 +1470,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72" ht="24" customHeight="1" s="39">
       <c r="A72" s="4" t="inlineStr">
         <is>
@@ -1688,7 +1681,6 @@
         </is>
       </c>
     </row>
-    <row r="90"/>
     <row r="91" ht="24" customHeight="1" s="39">
       <c r="A91" s="12" t="inlineStr">
         <is>
@@ -1792,7 +1784,6 @@
         </is>
       </c>
     </row>
-    <row r="100"/>
     <row r="101" ht="24" customHeight="1" s="39">
       <c r="A101" s="4" t="inlineStr">
         <is>
@@ -1932,7 +1923,6 @@
         </is>
       </c>
     </row>
-    <row r="113"/>
     <row r="114" ht="24" customHeight="1" s="39">
       <c r="A114" s="4" t="inlineStr">
         <is>
@@ -8445,7 +8435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P317"/>
+  <dimension ref="A1:P364"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.8515625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.00390625" customWidth="1" style="39" min="1" max="1"/>
@@ -33820,6 +33810,3766 @@
       <c r="P317" s="34" t="inlineStr">
         <is>
           <t>Athlean-X</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="19" t="n">
+        <v>317</v>
+      </c>
+      <c r="B318" s="19" t="inlineStr">
+        <is>
+          <t>Martwy ciąg z sandbagiem za uchwyty</t>
+        </is>
+      </c>
+      <c r="C318" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag deadlift</t>
+        </is>
+      </c>
+      <c r="D318" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Tył uda</t>
+        </is>
+      </c>
+      <c r="E318" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Brzuch, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F318" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G318" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H318" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I318" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J318" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K318" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L318" s="19" t="inlineStr">
+        <is>
+          <t>Ustaw worek blisko goleni i chwyć symetryczne uchwyty; Cofnij biodra, napnij brzuch i wstań, prowadząc worek blisko nóg; Odstaw go przez zgięcie bioder bez garbienia; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M318" s="19" t="inlineStr">
+        <is>
+          <t>Szarpanie z podłogi; Zaokrąglanie lędźwi; Odchylanie się w końcowej pozycji</t>
+        </is>
+      </c>
+      <c r="N318" s="19" t="inlineStr">
+        <is>
+          <t>Zwiększ ciężar dopiero po serii równych powtórzeń</t>
+        </is>
+      </c>
+      <c r="O318" s="19" t="inlineStr">
+        <is>
+          <t>Zmniejsz wypełnienie i ćwicz krótsze serie</t>
+        </is>
+      </c>
+      <c r="P318" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/the-ultimate-sandbag-deadlift-challenge/</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="19" t="n">
+        <v>318</v>
+      </c>
+      <c r="B319" s="19" t="inlineStr">
+        <is>
+          <t>Przysiad z sandbagiem trzymanym z przodu</t>
+        </is>
+      </c>
+      <c r="C319" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag front hold squat</t>
+        </is>
+      </c>
+      <c r="D319" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E319" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Biceps</t>
+        </is>
+      </c>
+      <c r="F319" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G319" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H319" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I319" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J319" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K319" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L319" s="19" t="inlineStr">
+        <is>
+          <t>Oprzyj worek poziomo przed klatką na przedramionach; Zejdź między biodra, utrzymując całe stopy na podłożu; Wstań bez wypychania żeber do przodu; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M319" s="19" t="inlineStr">
+        <is>
+          <t>Zapadanie kolan do środka; Opadanie łokci i tułowia; Odrywanie pięt</t>
+        </is>
+      </c>
+      <c r="N319" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż pauzę na dole bez utraty ustawienia</t>
+        </is>
+      </c>
+      <c r="O319" s="19" t="inlineStr">
+        <is>
+          <t>Płytszy przysiad z lżejszym workiem</t>
+        </is>
+      </c>
+      <c r="P319" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/top-10-ultimate-sandbag-training-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="19" t="n">
+        <v>319</v>
+      </c>
+      <c r="B320" s="19" t="inlineStr">
+        <is>
+          <t>Przysiad z sandbagiem objętym pionowo</t>
+        </is>
+      </c>
+      <c r="C320" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag bear hug squat</t>
+        </is>
+      </c>
+      <c r="D320" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E320" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="F320" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G320" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H320" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I320" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J320" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K320" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L320" s="19" t="inlineStr">
+        <is>
+          <t>Obejmij pionowo ustawiony worek, przyciągając go do tułowia; Usiądź między biodra i prowadź kolana w kierunku palców; Utrzymuj spokojny wydech podczas wstawania; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M320" s="19" t="inlineStr">
+        <is>
+          <t>Worek odsunięty od ciała; Garbienie górnych pleców; Wstrzymywanie oddechu przez całą serię</t>
+        </is>
+      </c>
+      <c r="N320" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo pogłębiaj przysiad z zachowaniem stabilnych stóp</t>
+        </is>
+      </c>
+      <c r="O320" s="19" t="inlineStr">
+        <is>
+          <t>Lżejszy worek i mniejsza głębokość</t>
+        </is>
+      </c>
+      <c r="P320" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/top-10-ultimate-sandbag-training-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="19" t="n">
+        <v>320</v>
+      </c>
+      <c r="B321" s="19" t="inlineStr">
+        <is>
+          <t>Przysiad z sandbagiem na jednym barku</t>
+        </is>
+      </c>
+      <c r="C321" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag shoulder squat</t>
+        </is>
+      </c>
+      <c r="D321" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E321" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Barki</t>
+        </is>
+      </c>
+      <c r="F321" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G321" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H321" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I321" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J321" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K321" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L321" s="19" t="inlineStr">
+        <is>
+          <t>Ułóż worek na jednym barku i asekuruj dłońmi; Wykonaj przysiad z tułowiem pośrodku między stopami; Po serii bezpiecznie odłóż worek i zmień bark; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M321" s="19" t="inlineStr">
+        <is>
+          <t>Przechylanie tułowia pod ciężarem; Zsuwanie worka na szyję; Skręt kolan</t>
+        </is>
+      </c>
+      <c r="N321" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj pauzę na dole przy równym rozłożeniu nacisku stóp</t>
+        </is>
+      </c>
+      <c r="O321" s="19" t="inlineStr">
+        <is>
+          <t>Mniejszy ciężar lub przysiad z workiem z przodu</t>
+        </is>
+      </c>
+      <c r="P321" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/10-ultimate-sandbag-exercises-that-are-musts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="19" t="n">
+        <v>321</v>
+      </c>
+      <c r="B322" s="19" t="inlineStr">
+        <is>
+          <t>Skłon biodrowy z sandbagiem przed klatką</t>
+        </is>
+      </c>
+      <c r="C322" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag front loaded good morning</t>
+        </is>
+      </c>
+      <c r="D322" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E322" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Brzuch</t>
+        </is>
+      </c>
+      <c r="F322" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G322" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H322" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I322" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J322" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K322" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L322" s="19" t="inlineStr">
+        <is>
+          <t>Trzymaj worek przy klatce na przedramionach; Z miękkimi kolanami cofnij biodra, wydłużając tył ud; Wróć przez wyprost bioder bez odchylania lędźwi; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M322" s="19" t="inlineStr">
+        <is>
+          <t>Zamiana ruchu w przysiad; Zaokrąglanie grzbietu; Odsuwanie worka od klatki</t>
+        </is>
+      </c>
+      <c r="N322" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż fazę opuszczania do trzech sekund</t>
+        </is>
+      </c>
+      <c r="O322" s="19" t="inlineStr">
+        <is>
+          <t>Lżejszy worek i krótszy skłon</t>
+        </is>
+      </c>
+      <c r="P322" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/top-10-ultimate-sandbag-training-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="19" t="n">
+        <v>322</v>
+      </c>
+      <c r="B323" s="19" t="inlineStr">
+        <is>
+          <t>Wiosłowanie sandbagiem w opadzie</t>
+        </is>
+      </c>
+      <c r="C323" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag bent-over row</t>
+        </is>
+      </c>
+      <c r="D323" s="19" t="inlineStr">
+        <is>
+          <t>Plecy</t>
+        </is>
+      </c>
+      <c r="E323" s="19" t="inlineStr">
+        <is>
+          <t>Biceps, Barki, Brzuch, Tył uda, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F323" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G323" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H323" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I323" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J323" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K323" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L323" s="19" t="inlineStr">
+        <is>
+          <t>Chwyć parę uchwytów i cofnij biodra do stabilnego opadu; Przyciągnij worek ku górnej części brzucha, nie unosząc tułowia; Opuść go powoli, zachowując długą szyję; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M323" s="19" t="inlineStr">
+        <is>
+          <t>Podrzucanie ciężaru tułowiem; Unoszenie barków do uszu; Zgarbione lędźwie</t>
+        </is>
+      </c>
+      <c r="N323" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj sekundę zatrzymania przy brzuchu</t>
+        </is>
+      </c>
+      <c r="O323" s="19" t="inlineStr">
+        <is>
+          <t>Zmniejsz ciężar i skróć serię</t>
+        </is>
+      </c>
+      <c r="P323" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/10-ultimate-sandbag-exercises-that-are-musts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="19" t="n">
+        <v>323</v>
+      </c>
+      <c r="B324" s="19" t="inlineStr">
+        <is>
+          <t>Dynamiczne podciągnięcie sandbaga do klatki</t>
+        </is>
+      </c>
+      <c r="C324" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag high pull</t>
+        </is>
+      </c>
+      <c r="D324" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Tył uda</t>
+        </is>
+      </c>
+      <c r="E324" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Barki, Brzuch, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F324" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G324" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H324" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I324" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J324" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K324" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L324" s="19" t="inlineStr">
+        <is>
+          <t>Rozpocznij z workiem przed goleniami w zgięciu bioder; Wyprostuj biodra dynamicznie i poprowadź łokcie w górę, nie ciągnąc samymi rękami; Kontroluj powrót worka blisko ciała; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M324" s="19" t="inlineStr">
+        <is>
+          <t>Szarpnięcie lędźwiami; Ruch ramion przed wyprostem bioder; Worek daleko od ciała</t>
+        </is>
+      </c>
+      <c r="N324" s="19" t="inlineStr">
+        <is>
+          <t>Przejdź do zarzutu po opanowaniu powtarzalnego toru</t>
+        </is>
+      </c>
+      <c r="O324" s="19" t="inlineStr">
+        <is>
+          <t>Lżejszy worek i spokojny martwy ciąg</t>
+        </is>
+      </c>
+      <c r="P324" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/top-10-ultimate-sandbag-training-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="19" t="n">
+        <v>324</v>
+      </c>
+      <c r="B325" s="19" t="inlineStr">
+        <is>
+          <t>Zarzut sandbaga na przedramiona</t>
+        </is>
+      </c>
+      <c r="C325" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag clean to fists</t>
+        </is>
+      </c>
+      <c r="D325" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Tył uda</t>
+        </is>
+      </c>
+      <c r="E325" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Biceps, Brzuch, Barki</t>
+        </is>
+      </c>
+      <c r="F325" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G325" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H325" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I325" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J325" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K325" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L325" s="19" t="inlineStr">
+        <is>
+          <t>Chwyć równoległe uchwyty i ustaw worek przy goleniach; Nadaj mu pęd biodrami i szybko podprowadź łokcie pod worek; Przyjmij ciężar na przedramionach bez uderzenia w klatkę; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M325" s="19" t="inlineStr">
+        <is>
+          <t>Ciągnięcie wyłącznie bicepsem; Uderzanie workiem o nadgarstki; Przeprost pleców przy chwycie</t>
+        </is>
+      </c>
+      <c r="N325" s="19" t="inlineStr">
+        <is>
+          <t>Po stabilnym przyjęciu dodaj osobne wyciskanie</t>
+        </is>
+      </c>
+      <c r="O325" s="19" t="inlineStr">
+        <is>
+          <t>Ćwicz high pull z mniejszym wypełnieniem</t>
+        </is>
+      </c>
+      <c r="P325" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/top-10-ultimate-sandbag-training-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="19" t="n">
+        <v>325</v>
+      </c>
+      <c r="B326" s="19" t="inlineStr">
+        <is>
+          <t>Wyciskanie sandbaga nad głowę</t>
+        </is>
+      </c>
+      <c r="C326" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag overhead press</t>
+        </is>
+      </c>
+      <c r="D326" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Triceps</t>
+        </is>
+      </c>
+      <c r="E326" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Pośladki</t>
+        </is>
+      </c>
+      <c r="F326" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G326" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H326" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I326" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J326" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K326" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L326" s="19" t="inlineStr">
+        <is>
+          <t>Zarzuć lekki worek raz i ustabilizuj go przed klatką; Wyciśnij pionowo bez wybicia z nóg i bez wypychania żeber; Opuść do pozycji wyjściowej, nie odginając nadgarstków; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M326" s="19" t="inlineStr">
+        <is>
+          <t>Przeprost lędźwi; Nierówny chwyt; Opuszczanie worka na głowę</t>
+        </is>
+      </c>
+      <c r="N326" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż kontrolowane opuszczanie</t>
+        </is>
+      </c>
+      <c r="O326" s="19" t="inlineStr">
+        <is>
+          <t>Zmniejsz wypełnienie lub ogranicz zakres do bezbolesnego</t>
+        </is>
+      </c>
+      <c r="P326" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/9-ultimate-sandbag-exercises-that-make-functional-strength-better/</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="19" t="n">
+        <v>326</v>
+      </c>
+      <c r="B327" s="19" t="inlineStr">
+        <is>
+          <t>Zarzut i wyciskanie sandbaga</t>
+        </is>
+      </c>
+      <c r="C327" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag clean and press</t>
+        </is>
+      </c>
+      <c r="D327" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Tył uda, Barki, Triceps</t>
+        </is>
+      </c>
+      <c r="E327" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Przód uda</t>
+        </is>
+      </c>
+      <c r="F327" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G327" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H327" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I327" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J327" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K327" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L327" s="19" t="inlineStr">
+        <is>
+          <t>W każdym powtórzeniu rozpocznij workiem przy goleniach; Zarzuć z bioder, ustabilizuj tułów i dopiero wtedy wyciśnij; Opuść do klatki, następnie bezpiecznie na podłoże; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M327" s="19" t="inlineStr">
+        <is>
+          <t>Wyciskanie przed ustabilizowaniem zarzutu; Wyginanie pleców; Niekontrolowany upadek worka</t>
+        </is>
+      </c>
+      <c r="N327" s="19" t="inlineStr">
+        <is>
+          <t>Łącz powtórzenia bez utraty jakości przyjęcia</t>
+        </is>
+      </c>
+      <c r="O327" s="19" t="inlineStr">
+        <is>
+          <t>Trenuj oddzielnie lżejszy zarzut i wyciskanie</t>
+        </is>
+      </c>
+      <c r="P327" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/10-ultimate-sandbag-exercises-that-are-musts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="19" t="n">
+        <v>327</v>
+      </c>
+      <c r="B328" s="19" t="inlineStr">
+        <is>
+          <t>Zakrok z przeniesieniem sandbaga przy przedniej nodze</t>
+        </is>
+      </c>
+      <c r="C328" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag MAX lunge</t>
+        </is>
+      </c>
+      <c r="D328" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E328" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Tył uda, Plecy</t>
+        </is>
+      </c>
+      <c r="F328" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G328" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H328" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I328" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J328" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K328" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L328" s="19" t="inlineStr">
+        <is>
+          <t>Trzymaj worek za uchwyty przed biodrami; Cofnij jedną nogę, prowadząc worek na zewnątrz kolana nogi przedniej; Wróć naciskiem przedniej stopy, kontrolując obrót tułowia; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M328" s="19" t="inlineStr">
+        <is>
+          <t>Skręcanie obciążonego kolana; Zbyt obszerny zamach; Utrata równowagi przy powrocie</t>
+        </is>
+      </c>
+      <c r="N328" s="19" t="inlineStr">
+        <is>
+          <t>Łącz kolejne powtórzenia płynnie, nie zwiększając zamachu</t>
+        </is>
+      </c>
+      <c r="O328" s="19" t="inlineStr">
+        <is>
+          <t>Zakrok bez rotacji z lżejszym workiem</t>
+        </is>
+      </c>
+      <c r="P328" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/10-ultimate-sandbag-exercises-that-are-musts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="19" t="n">
+        <v>328</v>
+      </c>
+      <c r="B329" s="19" t="inlineStr">
+        <is>
+          <t>Przenoszenie sandbaga ruchem szuflowania</t>
+        </is>
+      </c>
+      <c r="C329" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag shoveling</t>
+        </is>
+      </c>
+      <c r="D329" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Brzuch</t>
+        </is>
+      </c>
+      <c r="E329" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Plecy, Barki, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F329" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G329" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H329" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I329" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J329" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K329" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L329" s="19" t="inlineStr">
+        <is>
+          <t>Trzymaj worek za uchwyty przed sobą i obróć stopy wraz z biodrami w bok; Cofnij biodro, prowadząc worek przy zewnętrznej stronie kolana; Wyprostuj biodro i przenieś ciężar ku drugiej stronie bez skręcania samych lędźwi; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M329" s="19" t="inlineStr">
+        <is>
+          <t>Stopy przyklejone podczas obrotu; Skręt tylko w pasie; Utrata kontroli hamowania</t>
+        </is>
+      </c>
+      <c r="N329" s="19" t="inlineStr">
+        <is>
+          <t>Zwiększ płynność przejścia między stronami</t>
+        </is>
+      </c>
+      <c r="O329" s="19" t="inlineStr">
+        <is>
+          <t>Lżejszy worek i mały, powolny łuk</t>
+        </is>
+      </c>
+      <c r="P329" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/10-ultimate-sandbag-exercises-that-are-musts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="19" t="n">
+        <v>329</v>
+      </c>
+      <c r="B330" s="19" t="inlineStr">
+        <is>
+          <t>Obwodzenie sandbaga wokół tułowia w klęku</t>
+        </is>
+      </c>
+      <c r="C330" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag around the world</t>
+        </is>
+      </c>
+      <c r="D330" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E330" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Plecy, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F330" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G330" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H330" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I330" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J330" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K330" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L330" s="19" t="inlineStr">
+        <is>
+          <t>Uklęknij wysoko, napinając lekko pośladki; Przeprowadź lekki worek wokół górnej części tułowia jak przy zakładaniu kurtki; Utrzymuj miednicę nad kolanami i wróć tą samą kontrolowaną drogą; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M330" s="19" t="inlineStr">
+        <is>
+          <t>Siadanie na piętach; Przeprost lędźwi; Zbyt ciężki worek przy głowie</t>
+        </is>
+      </c>
+      <c r="N330" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż czas płynnego ruchu bez zwiększania ciężaru</t>
+        </is>
+      </c>
+      <c r="O330" s="19" t="inlineStr">
+        <is>
+          <t>Mały łuk z bardzo lekkim workiem</t>
+        </is>
+      </c>
+      <c r="P330" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/10-ultimate-sandbag-exercises-that-are-musts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="19" t="n">
+        <v>330</v>
+      </c>
+      <c r="B331" s="19" t="inlineStr">
+        <is>
+          <t>Przeciąganie sandbaga pod tułowiem w desce</t>
+        </is>
+      </c>
+      <c r="C331" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag plank lateral drag</t>
+        </is>
+      </c>
+      <c r="D331" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E331" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Plecy, Pośladki, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F331" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G331" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H331" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I331" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J331" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K331" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L331" s="19" t="inlineStr">
+        <is>
+          <t>Ustaw szeroko stopy w podporze, a lekki worek obok dłoni; Sięgnij przeciwną ręką po uchwyt i wolno przeciągnij worek pod klatką; Utrzymuj biodra równolegle do podłogi, potem zmień rękę; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M331" s="19" t="inlineStr">
+        <is>
+          <t>Obracanie miednicy; Zadzieranie bioder; Szarpanie ciężaru</t>
+        </is>
+      </c>
+      <c r="N331" s="19" t="inlineStr">
+        <is>
+          <t>Zwęż rozstaw stóp dopiero przy pełnej kontroli</t>
+        </is>
+      </c>
+      <c r="O331" s="19" t="inlineStr">
+        <is>
+          <t>Oprzyj kolana i mocno zmniejsz wypełnienie</t>
+        </is>
+      </c>
+      <c r="P331" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/top-10-ultimate-sandbag-training-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="19" t="n">
+        <v>331</v>
+      </c>
+      <c r="B332" s="19" t="inlineStr">
+        <is>
+          <t>Most biodrowy z napięciem sandbaga nad klatką</t>
+        </is>
+      </c>
+      <c r="C332" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag tension hip bridge</t>
+        </is>
+      </c>
+      <c r="D332" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Tył uda</t>
+        </is>
+      </c>
+      <c r="E332" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Barki</t>
+        </is>
+      </c>
+      <c r="F332" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G332" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H332" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I332" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J332" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K332" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L332" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się, ustaw stopy blisko pionu pod kolanami i chwyć zewnętrzne uchwyty lekkiego worka; Utrzymuj worek nad dolną klatką, delikatnie rozciągając uchwyty na boki; Unieś biodra naciskiem stóp, nie przenosząc worka na biodra; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M332" s="19" t="inlineStr">
+        <is>
+          <t>Przeprost w lędźwiach; Luźny chwyt nad klatką; Rozjeżdżanie kolan</t>
+        </is>
+      </c>
+      <c r="N332" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj pauzę u góry przy stałym napięciu uchwytów</t>
+        </is>
+      </c>
+      <c r="O332" s="19" t="inlineStr">
+        <is>
+          <t>Lżejszy worek i niższe uniesienie bioder</t>
+        </is>
+      </c>
+      <c r="P332" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/10-ultimate-sandbag-exercises-that-are-musts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="19" t="n">
+        <v>332</v>
+      </c>
+      <c r="B333" s="19" t="inlineStr">
+        <is>
+          <t>Wyciskanie sandbaga łukiem w półklęku</t>
+        </is>
+      </c>
+      <c r="C333" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag half-kneeling arc press</t>
+        </is>
+      </c>
+      <c r="D333" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Triceps</t>
+        </is>
+      </c>
+      <c r="E333" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Pośladki</t>
+        </is>
+      </c>
+      <c r="F333" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G333" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H333" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I333" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J333" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K333" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L333" s="19" t="inlineStr">
+        <is>
+          <t>Przyjmij stabilny półklęk i ułóż lekki worek przy jednym barku; Oburącz wyciśnij go łukiem ponad głową i powoli opuść ku drugiemu barkowi; Oprzyj ciężar na nogach, nie pochylając tułowia na boki; Sprawdź uchwyty i zamknięcia wkładów, nie rzucaj workiem; Dobierz ciężar do techniki — posiadane 20 kg nie jest obciążeniem obowiązkowym</t>
+        </is>
+      </c>
+      <c r="M333" s="19" t="inlineStr">
+        <is>
+          <t>Zbyt niski łuk nad głową; Kołysanie miednicą; Za duży ciężar</t>
+        </is>
+      </c>
+      <c r="N333" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż opuszczanie po drugiej stronie</t>
+        </is>
+      </c>
+      <c r="O333" s="19" t="inlineStr">
+        <is>
+          <t>Bardzo lekki worek i stabilny klęk obunóż</t>
+        </is>
+      </c>
+      <c r="P333" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/10-ultimate-sandbag-exercises-that-are-musts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="19" t="n">
+        <v>333</v>
+      </c>
+      <c r="B334" s="19" t="inlineStr">
+        <is>
+          <t>Przetaczanie kółka w przód z kolan</t>
+        </is>
+      </c>
+      <c r="C334" s="19" t="inlineStr">
+        <is>
+          <t>Kneeling ab wheel rollout</t>
+        </is>
+      </c>
+      <c r="D334" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E334" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Barki, Pośladki</t>
+        </is>
+      </c>
+      <c r="F334" s="19" t="inlineStr">
+        <is>
+          <t>Kółko do brzucha</t>
+        </is>
+      </c>
+      <c r="G334" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H334" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I334" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J334" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10</t>
+        </is>
+      </c>
+      <c r="K334" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L334" s="19" t="inlineStr">
+        <is>
+          <t>Oprzyj kolana na macie i chwyć oba uchwyty; Podwiń lekko miednicę i przetaczaj kółko po prostej tylko tak daleko, jak utrzymujesz napięty brzuch; Wróć bez siadania biodrami na pięty, kółko nie pomaga w powrocie</t>
+        </is>
+      </c>
+      <c r="M334" s="19" t="inlineStr">
+        <is>
+          <t>Opadanie lędźwi; Wyjazd poza kontrolowany zakres; Szarpanie ramionami</t>
+        </is>
+      </c>
+      <c r="N334" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw wydłużaj zakres, rollout ze stania dopiero jako zaawansowany cel po pełnej kontroli z kolan</t>
+        </is>
+      </c>
+      <c r="O334" s="19" t="inlineStr">
+        <is>
+          <t>Krótki zakres ograniczony ścianą, bez uderzania kółkiem</t>
+        </is>
+      </c>
+      <c r="P334" s="19" t="inlineStr">
+        <is>
+          <t>https://theworkoutdigest.com/ab-wheel-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="19" t="n">
+        <v>334</v>
+      </c>
+      <c r="B335" s="19" t="inlineStr">
+        <is>
+          <t>Przetaczanie kółka po skosie z kolan</t>
+        </is>
+      </c>
+      <c r="C335" s="19" t="inlineStr">
+        <is>
+          <t>Kneeling ab wheel V rollout</t>
+        </is>
+      </c>
+      <c r="D335" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E335" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Barki, Pośladki</t>
+        </is>
+      </c>
+      <c r="F335" s="19" t="inlineStr">
+        <is>
+          <t>Kółko do brzucha</t>
+        </is>
+      </c>
+      <c r="G335" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H335" s="19" t="inlineStr">
+        <is>
+          <t>Zaawansowany</t>
+        </is>
+      </c>
+      <c r="I335" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J335" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K335" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L335" s="19" t="inlineStr">
+        <is>
+          <t>Z klęku skieruj kółko lekko po skosie w lewo, trzymając oba uchwyty; Utrzymuj długi tułów bez zapadania lędźwi; Wróć do środka i wykonaj osobne powtórzenie w prawo, nie próbuj ostro skręcać podwójnej rolki pod obciążeniem</t>
+        </is>
+      </c>
+      <c r="M335" s="19" t="inlineStr">
+        <is>
+          <t>Skręt samych lędźwi; Nagła zmiana kierunku w końcu ruchu; Zbyt daleki wyjazd</t>
+        </is>
+      </c>
+      <c r="N335" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo wydłuż tor po skosie bez pogłębiania skrętu</t>
+        </is>
+      </c>
+      <c r="O335" s="19" t="inlineStr">
+        <is>
+          <t>Bardzo krótki skos lub rollout po prostej</t>
+        </is>
+      </c>
+      <c r="P335" s="19" t="inlineStr">
+        <is>
+          <t>https://theworkoutdigest.com/ab-wheel-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="19" t="n">
+        <v>335</v>
+      </c>
+      <c r="B336" s="19" t="inlineStr">
+        <is>
+          <t>Deska z dłońmi na kółku</t>
+        </is>
+      </c>
+      <c r="C336" s="19" t="inlineStr">
+        <is>
+          <t>Ab wheel plank</t>
+        </is>
+      </c>
+      <c r="D336" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E336" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Klatka piersiowa, Pośladki</t>
+        </is>
+      </c>
+      <c r="F336" s="19" t="inlineStr">
+        <is>
+          <t>Kółko do brzucha</t>
+        </is>
+      </c>
+      <c r="G336" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H336" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I336" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J336" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K336" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L336" s="19" t="inlineStr">
+        <is>
+          <t>Chwyć oba uchwyty i ustaw barki nad osią kółka; Wyprostuj nogi do podporu na palcach, napnij brzuch i pośladki; Utrzymuj rolkę nieruchomo i oddychaj, nie odkładaj stóp na kółko</t>
+        </is>
+      </c>
+      <c r="M336" s="19" t="inlineStr">
+        <is>
+          <t>Odjeżdżanie rolki; Zapadanie bioder; Wstrzymanie oddechu</t>
+        </is>
+      </c>
+      <c r="N336" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż utrzymanie przy niezmienionym ustawieniu</t>
+        </is>
+      </c>
+      <c r="O336" s="19" t="inlineStr">
+        <is>
+          <t>Podeprzyj kolana na macie</t>
+        </is>
+      </c>
+      <c r="P336" s="19" t="inlineStr">
+        <is>
+          <t>https://barbend.com/ab-wheel-workouts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="19" t="n">
+        <v>336</v>
+      </c>
+      <c r="B337" s="19" t="inlineStr">
+        <is>
+          <t>Wojownik I</t>
+        </is>
+      </c>
+      <c r="C337" s="19" t="inlineStr">
+        <is>
+          <t>Warrior I — Virabhadrasana I</t>
+        </is>
+      </c>
+      <c r="D337" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E337" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Zginacze bioder, Brzuch, Barki, Plecy</t>
+        </is>
+      </c>
+      <c r="F337" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G337" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H337" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I337" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J337" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K337" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L337" s="19" t="inlineStr">
+        <is>
+          <t>Ustaw jedną nogę z przodu, a tylną stopę lekko skośnie; Zegnij przednie kolano w kierunku palców i unieś ramiona; Wydłuż tułów bez wymuszania ustawienia bioder; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M337" s="19" t="inlineStr">
+        <is>
+          <t>Kolano zapadające do środka; Przeprost lędźwi; Zbyt wąskie ustawienie stóp</t>
+        </is>
+      </c>
+      <c r="N337" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż utrzymanie bez utraty oddechu</t>
+        </is>
+      </c>
+      <c r="O337" s="19" t="inlineStr">
+        <is>
+          <t>Skróć wykrok i trzymaj dłonie na biodrach</t>
+        </is>
+      </c>
+      <c r="P337" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/warrior-i-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="19" t="n">
+        <v>337</v>
+      </c>
+      <c r="B338" s="19" t="inlineStr">
+        <is>
+          <t>Wojownik II</t>
+        </is>
+      </c>
+      <c r="C338" s="19" t="inlineStr">
+        <is>
+          <t>Warrior II — Virabhadrasana II</t>
+        </is>
+      </c>
+      <c r="D338" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki, Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="E338" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Barki, Łydki</t>
+        </is>
+      </c>
+      <c r="F338" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G338" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H338" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I338" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J338" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K338" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L338" s="19" t="inlineStr">
+        <is>
+          <t>Stań w rozkroku i skieruj przednią stopę na zewnątrz; Ugnij jej kolano, utrzymując tułów pionowo; Wyciągnij ramiona w przeciwnych kierunkach i spójrz nad przednią dłonią; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M338" s="19" t="inlineStr">
+        <is>
+          <t>Opieranie tułowia na przedniej nodze; Zapadanie kolana; Unoszenie barków</t>
+        </is>
+      </c>
+      <c r="N338" s="19" t="inlineStr">
+        <is>
+          <t>Nieco pogłębiaj ugięcie przy stabilnych stopach</t>
+        </is>
+      </c>
+      <c r="O338" s="19" t="inlineStr">
+        <is>
+          <t>Mniejsze ugięcie i dłonie na biodrach</t>
+        </is>
+      </c>
+      <c r="P338" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/warrior-ii-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="19" t="n">
+        <v>338</v>
+      </c>
+      <c r="B339" s="19" t="inlineStr">
+        <is>
+          <t>Wojownik III</t>
+        </is>
+      </c>
+      <c r="C339" s="19" t="inlineStr">
+        <is>
+          <t>Warrior III — Virabhadrasana III</t>
+        </is>
+      </c>
+      <c r="D339" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Tył uda, Przód uda</t>
+        </is>
+      </c>
+      <c r="E339" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Barki, Łydki</t>
+        </is>
+      </c>
+      <c r="F339" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G339" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H339" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I339" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J339" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K339" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L339" s="19" t="inlineStr">
+        <is>
+          <t>Przenieś ciężar na jedną stopę i pochyl długi tułów; Wyciągnij drugą nogę w tył, utrzymując oba biodra skierowane ku podłodze; Sięgnij ramionami przed siebie bez przeprostu kolana podporowego; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M339" s="19" t="inlineStr">
+        <is>
+          <t>Otwieranie miednicy w bok; Zapadanie lędźwi; Blokowanie kolana</t>
+        </is>
+      </c>
+      <c r="N339" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż utrzymanie w poziomie</t>
+        </is>
+      </c>
+      <c r="O339" s="19" t="inlineStr">
+        <is>
+          <t>Oprzyj dłonie o ścianę i unieś nogę niżej</t>
+        </is>
+      </c>
+      <c r="P339" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/warrior-iii-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="19" t="n">
+        <v>339</v>
+      </c>
+      <c r="B340" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja trójkąta</t>
+        </is>
+      </c>
+      <c r="C340" s="19" t="inlineStr">
+        <is>
+          <t>Extended Triangle — Utthita Trikonasana</t>
+        </is>
+      </c>
+      <c r="D340" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="E340" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy, Barki, Przód uda</t>
+        </is>
+      </c>
+      <c r="F340" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G340" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H340" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I340" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J340" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K340" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L340" s="19" t="inlineStr">
+        <is>
+          <t>W szerokim rozkroku skieruj jedną stopę na zewnątrz; Wydłuż tułów nad tą nogą i oprzyj dłoń na goleni, nie na kolanie; Otwórz klatkę i unieś drugą rękę bez skręcania szyi na siłę; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M340" s="19" t="inlineStr">
+        <is>
+          <t>Zapadanie dolnego boku tułowia; Nacisk na kolano; Dążenie dłonią do podłogi kosztem pleców</t>
+        </is>
+      </c>
+      <c r="N340" s="19" t="inlineStr">
+        <is>
+          <t>Zmniejsz podparcie dłonią przy zachowaniu długości boków</t>
+        </is>
+      </c>
+      <c r="O340" s="19" t="inlineStr">
+        <is>
+          <t>Dłoń wyżej na goleni i wzrok w dół</t>
+        </is>
+      </c>
+      <c r="P340" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/extended-triangle-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="19" t="n">
+        <v>340</v>
+      </c>
+      <c r="B341" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja rozciągniętego kąta bocznego</t>
+        </is>
+      </c>
+      <c r="C341" s="19" t="inlineStr">
+        <is>
+          <t>Extended Side Angle — Utthita Parsvakonasana</t>
+        </is>
+      </c>
+      <c r="D341" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki, Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="E341" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Barki, Plecy</t>
+        </is>
+      </c>
+      <c r="F341" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G341" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H341" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I341" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J341" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K341" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L341" s="19" t="inlineStr">
+        <is>
+          <t>Z szerokiego rozkroku zegnij przednie kolano i oprzyj przedramię na udzie; Wydłuż drugi bok od tylnej pięty do ręki sięgającej nad uchem; Otwórz klatkę bez naciskania całym ciężarem na udo; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M341" s="19" t="inlineStr">
+        <is>
+          <t>Zapadanie kolana; Garbienie klatki; Zawieszanie ciężaru na przedramieniu</t>
+        </is>
+      </c>
+      <c r="N341" s="19" t="inlineStr">
+        <is>
+          <t>Sięgnij dolną dłonią niżej bez utraty osi kolana</t>
+        </is>
+      </c>
+      <c r="O341" s="19" t="inlineStr">
+        <is>
+          <t>Mniejsze ugięcie nogi i górna dłoń na biodrze</t>
+        </is>
+      </c>
+      <c r="P341" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/extended-side-angle-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="19" t="n">
+        <v>341</v>
+      </c>
+      <c r="B342" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja półksiężyca w staniu</t>
+        </is>
+      </c>
+      <c r="C342" s="19" t="inlineStr">
+        <is>
+          <t>Half Moon — Ardha Chandrasana</t>
+        </is>
+      </c>
+      <c r="D342" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Przód uda</t>
+        </is>
+      </c>
+      <c r="E342" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Brzuch, Barki, Łydki</t>
+        </is>
+      </c>
+      <c r="F342" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G342" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H342" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I342" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J342" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K342" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L342" s="19" t="inlineStr">
+        <is>
+          <t>Z przeniesienia ciężaru na jedną nogę ustaw dłoń przed stopą; Unieś drugą nogę do tyłu i otwórz miednicę w bok; Wydłuż tułów i unieś wolną rękę, stabilizując kolano podporowe; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M342" s="19" t="inlineStr">
+        <is>
+          <t>Blokowanie kolana; Opadanie tułowia; Wymuszanie spojrzenia w górę</t>
+        </is>
+      </c>
+      <c r="N342" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo odciążaj podpierającą dłoń</t>
+        </is>
+      </c>
+      <c r="O342" s="19" t="inlineStr">
+        <is>
+          <t>Oprzyj plecy i uniesioną piętę o ścianę</t>
+        </is>
+      </c>
+      <c r="P342" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/half-moon-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="19" t="n">
+        <v>342</v>
+      </c>
+      <c r="B343" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja drzewa</t>
+        </is>
+      </c>
+      <c r="C343" s="19" t="inlineStr">
+        <is>
+          <t>Tree — Vrksasana</t>
+        </is>
+      </c>
+      <c r="D343" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Przód uda, Łydki</t>
+        </is>
+      </c>
+      <c r="E343" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="F343" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G343" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H343" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I343" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J343" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K343" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L343" s="19" t="inlineStr">
+        <is>
+          <t>Stań na jednej nodze i przyłóż drugą stopę do łydki lub uda, omijając kolano; Utrzymaj miednicę przodem i spójrz na nieruchomy punkt; Złącz dłonie przed klatką bez wypychania biodra w bok; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M343" s="19" t="inlineStr">
+        <is>
+          <t>Nacisk stopy na staw kolanowy; Skręt miednicy; Przeprost kolana podporowego</t>
+        </is>
+      </c>
+      <c r="N343" s="19" t="inlineStr">
+        <is>
+          <t>Unieś ramiona przy zachowaniu równowagi</t>
+        </is>
+      </c>
+      <c r="O343" s="19" t="inlineStr">
+        <is>
+          <t>Palce uniesionej nogi pozostaw na podłodze</t>
+        </is>
+      </c>
+      <c r="P343" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/tree-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="19" t="n">
+        <v>343</v>
+      </c>
+      <c r="B344" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja orła w staniu</t>
+        </is>
+      </c>
+      <c r="C344" s="19" t="inlineStr">
+        <is>
+          <t>Eagle — Garudasana</t>
+        </is>
+      </c>
+      <c r="D344" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E344" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Plecy, Brzuch, Łydki</t>
+        </is>
+      </c>
+      <c r="F344" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G344" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H344" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I344" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J344" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K344" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L344" s="19" t="inlineStr">
+        <is>
+          <t>Lekko ugnij nogę podporową i skrzyżuj nad nią drugie udo; Skrzyżuj ramiona przed klatką i unieś łokcie w bezbolesnym zakresie; Utrzymuj tułów pionowo, nie wymuszając owinięcia stopy; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M344" s="19" t="inlineStr">
+        <is>
+          <t>Skręcanie bolącego kolana; Zapadanie klatki; Wymuszanie splotu dłoni</t>
+        </is>
+      </c>
+      <c r="N344" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo odciąż stopę pomocniczą</t>
+        </is>
+      </c>
+      <c r="O344" s="19" t="inlineStr">
+        <is>
+          <t>Oprzyj palce wolnej nogi o podłoże i obejmij ramiona dłońmi</t>
+        </is>
+      </c>
+      <c r="P344" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/eagle-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="19" t="n">
+        <v>344</v>
+      </c>
+      <c r="B345" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja krzesła bez podparcia</t>
+        </is>
+      </c>
+      <c r="C345" s="19" t="inlineStr">
+        <is>
+          <t>Chair — Utkatasana</t>
+        </is>
+      </c>
+      <c r="D345" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E345" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Barki, Plecy, Łydki</t>
+        </is>
+      </c>
+      <c r="F345" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G345" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H345" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I345" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J345" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K345" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L345" s="19" t="inlineStr">
+        <is>
+          <t>Stań ze stopami razem lub na szerokość bioder; Cofnij biodra i ugnij kolana jak do siedzenia, nie używając krzesła; Unieś ramiona tylko na tyle, by zachować spokojne ustawienie żeber; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M345" s="19" t="inlineStr">
+        <is>
+          <t>Przeprost pleców przy unoszeniu rąk; Odrywanie pięt; Zapadanie kolan</t>
+        </is>
+      </c>
+      <c r="N345" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo wydłuż utrzymanie</t>
+        </is>
+      </c>
+      <c r="O345" s="19" t="inlineStr">
+        <is>
+          <t>Płytsze ugięcie z dłońmi na biodrach</t>
+        </is>
+      </c>
+      <c r="P345" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/chair-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="19" t="n">
+        <v>345</v>
+      </c>
+      <c r="B346" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja wielbłąda</t>
+        </is>
+      </c>
+      <c r="C346" s="19" t="inlineStr">
+        <is>
+          <t>Camel — Ustrasana</t>
+        </is>
+      </c>
+      <c r="D346" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Pośladki</t>
+        </is>
+      </c>
+      <c r="E346" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder, Przód uda, Klatka piersiowa, Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F346" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G346" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H346" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I346" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J346" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K346" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L346" s="19" t="inlineStr">
+        <is>
+          <t>Uklęknij z biodrami nad kolanami i podeprzyj dłońmi tył miednicy; Unieś mostek, a następnie delikatnie otwórz górę tułowia w tył; Do pięt sięgaj dopiero bez ucisku w lędźwiach i szyi; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M346" s="19" t="inlineStr">
+        <is>
+          <t>Zapadanie lędźwi; Odrzucanie głowy; Cofanie bioder za kolana</t>
+        </is>
+      </c>
+      <c r="N346" s="19" t="inlineStr">
+        <is>
+          <t>Sięgaj do pięt dopiero po opanowaniu podpartej wersji</t>
+        </is>
+      </c>
+      <c r="O346" s="19" t="inlineStr">
+        <is>
+          <t>Dłonie pozostają na miednicy, minimalne odchylenie</t>
+        </is>
+      </c>
+      <c r="P346" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/camel-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="19" t="n">
+        <v>346</v>
+      </c>
+      <c r="B347" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja łuku</t>
+        </is>
+      </c>
+      <c r="C347" s="19" t="inlineStr">
+        <is>
+          <t>Bow — Dhanurasana</t>
+        </is>
+      </c>
+      <c r="D347" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Pośladki, Tył uda</t>
+        </is>
+      </c>
+      <c r="E347" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Zginacze bioder, Klatka piersiowa, Barki</t>
+        </is>
+      </c>
+      <c r="F347" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G347" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H347" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I347" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J347" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K347" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L347" s="19" t="inlineStr">
+        <is>
+          <t>Leżąc na brzuchu, ugnij kolana i chwyć kostki obiema dłońmi; Naciśnij goleniami w tył, unosząc klatkę i ewentualnie uda; Zachowaj oddech i szyję jako przedłużenie pleców; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M347" s="19" t="inlineStr">
+        <is>
+          <t>Rozjeżdżanie kolan; Ciągnięcie stóp samymi rękami; Bolesny ucisk lędźwi</t>
+        </is>
+      </c>
+      <c r="N347" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż łagodne utrzymanie, nie zwiększając wygięcia na siłę</t>
+        </is>
+      </c>
+      <c r="O347" s="19" t="inlineStr">
+        <is>
+          <t>Mniejsze uniesienie, a przy bólu pomiń pozycję</t>
+        </is>
+      </c>
+      <c r="P347" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/bow-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="19" t="n">
+        <v>347</v>
+      </c>
+      <c r="B348" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja łodzi w siadzie</t>
+        </is>
+      </c>
+      <c r="C348" s="19" t="inlineStr">
+        <is>
+          <t>Boat — Paripurna Navasana</t>
+        </is>
+      </c>
+      <c r="D348" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Zginacze bioder</t>
+        </is>
+      </c>
+      <c r="E348" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Plecy</t>
+        </is>
+      </c>
+      <c r="F348" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G348" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H348" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I348" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J348" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K348" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L348" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź na guzach kulszowych i unieś mostek; Odchyl długi tułów, po czym unieś stopy bez opadania na kość krzyżową; Utrzymaj równowagę z rękami przed sobą i stopniowo prostuj kolana; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M348" s="19" t="inlineStr">
+        <is>
+          <t>Zaokrąglanie lędźwi; Wysuwanie brody; Prostowanie nóg kosztem pleców</t>
+        </is>
+      </c>
+      <c r="N348" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo wyprostuj obie nogi</t>
+        </is>
+      </c>
+      <c r="O348" s="19" t="inlineStr">
+        <is>
+          <t>Ugnij kolana i przytrzymaj uda</t>
+        </is>
+      </c>
+      <c r="P348" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/boat-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="19" t="n">
+        <v>348</v>
+      </c>
+      <c r="B349" s="19" t="inlineStr">
+        <is>
+          <t>Skręt mędrca w siadzie na podłodze</t>
+        </is>
+      </c>
+      <c r="C349" s="19" t="inlineStr">
+        <is>
+          <t>Half Lord of the Fishes — Ardha Matsyendrasana</t>
+        </is>
+      </c>
+      <c r="D349" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Brzuch</t>
+        </is>
+      </c>
+      <c r="E349" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Barki</t>
+        </is>
+      </c>
+      <c r="F349" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G349" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H349" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I349" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J349" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K349" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L349" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź i przełóż stopę jednej nogi za przeciwne kolano; Wydłuż kręgosłup na wdechu i łagodnie obróć tułów ku uniesionemu kolanu; Dłoń za plecami tylko podpiera, nie wymusza skrętu; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M349" s="19" t="inlineStr">
+        <is>
+          <t>Szarpanie łokciem o kolano; Zapadanie pleców; Skręt szyją zamiast tułowiem</t>
+        </is>
+      </c>
+      <c r="N349" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż utrzymanie przy równych guzach kulszowych</t>
+        </is>
+      </c>
+      <c r="O349" s="19" t="inlineStr">
+        <is>
+          <t>Pozostaw dolną nogę prostą i obejmij kolano zamiast zapierać łokieć</t>
+        </is>
+      </c>
+      <c r="P349" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/half-lord-of-the-fishes-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="19" t="n">
+        <v>349</v>
+      </c>
+      <c r="B350" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja bramy w klęku</t>
+        </is>
+      </c>
+      <c r="C350" s="19" t="inlineStr">
+        <is>
+          <t>Gate — Parighasana</t>
+        </is>
+      </c>
+      <c r="D350" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="E350" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Barki, Tył uda</t>
+        </is>
+      </c>
+      <c r="F350" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G350" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H350" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I350" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J350" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K350" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L350" s="19" t="inlineStr">
+        <is>
+          <t>Z klęku wyprostuj jedną nogę w bok, pozostawiając drugie biodro nad kolanem; Oprzyj dłoń na wyprostowanej nodze i wydłuż przeciwną rękę nad głową; Wykonaj łagodny skłon boczny bez obracania klatki ku podłodze; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M350" s="19" t="inlineStr">
+        <is>
+          <t>Zgniatanie dolnego boku; Opieranie dłoni na kolanie; Ból kolana klęczącego</t>
+        </is>
+      </c>
+      <c r="N350" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż sięganie ręką bez pogłębiania skłonu na siłę</t>
+        </is>
+      </c>
+      <c r="O350" s="19" t="inlineStr">
+        <is>
+          <t>Mniejszy skłon i dłoń wyżej na udzie</t>
+        </is>
+      </c>
+      <c r="P350" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/gate-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="19" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" s="19" t="inlineStr">
+        <is>
+          <t>Skłon w przód w szerokim rozkroku</t>
+        </is>
+      </c>
+      <c r="C351" s="19" t="inlineStr">
+        <is>
+          <t>Wide-Legged Forward Bend — Prasarita Padottanasana</t>
+        </is>
+      </c>
+      <c r="D351" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="E351" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Plecy, Brzuch</t>
+        </is>
+      </c>
+      <c r="F351" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G351" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H351" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I351" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J351" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K351" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L351" s="19" t="inlineStr">
+        <is>
+          <t>Stań w stabilnym rozkroku i połóż dłonie na biodrach; Pochyl się z bioder, wydłużając plecy i podpierając dłonie na podłodze tylko jeśli sięgasz swobodnie; Wyjdź powoli, bez obciążania głowy; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M351" s="19" t="inlineStr">
+        <is>
+          <t>Przeprost kolan; Dociskanie głowy do podłoża; Zbyt szybkie wstawanie</t>
+        </is>
+      </c>
+      <c r="N351" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo pogłębiaj skłon przy długich plecach</t>
+        </is>
+      </c>
+      <c r="O351" s="19" t="inlineStr">
+        <is>
+          <t>Ugnij kolana i zatrzymaj skłon wyżej z dłońmi na udach</t>
+        </is>
+      </c>
+      <c r="P351" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/wide-legged-forward-bend/</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="19" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" s="19" t="inlineStr">
+        <is>
+          <t>Pozycja szczęśliwego dziecka</t>
+        </is>
+      </c>
+      <c r="C352" s="19" t="inlineStr">
+        <is>
+          <t>Happy Baby — Ananda Balasana</t>
+        </is>
+      </c>
+      <c r="D352" s="19" t="inlineStr">
+        <is>
+          <t>Przywodziciele uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E352" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Plecy</t>
+        </is>
+      </c>
+      <c r="F352" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G352" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H352" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I352" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J352" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K352" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L352" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na plecach i przyciągnij kolana szerzej niż tułów; Chwyć zewnętrzne krawędzie stóp lub łydki, kierując podeszwy ku górze; Pozostaw głowę i kość krzyżową na podłożu, nie ciągnąc nóg na siłę; Oddychaj swobodnie, wyjdź z pozycji przy bólu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M352" s="19" t="inlineStr">
+        <is>
+          <t>Odrywanie głowy; Szarpanie stóp; Ból pachwin</t>
+        </is>
+      </c>
+      <c r="N352" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż spokojne utrzymanie bez mocniejszego ciągnięcia</t>
+        </is>
+      </c>
+      <c r="O352" s="19" t="inlineStr">
+        <is>
+          <t>Chwyć uda zamiast stóp</t>
+        </is>
+      </c>
+      <c r="P352" s="19" t="inlineStr">
+        <is>
+          <t>https://www.yogajournal.com/poses/happy-baby-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="19" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" s="19" t="inlineStr">
+        <is>
+          <t>Przemieszczanie bokiem w przysiadzie na rękach</t>
+        </is>
+      </c>
+      <c r="C353" s="19" t="inlineStr">
+        <is>
+          <t>GMB Monkey</t>
+        </is>
+      </c>
+      <c r="D353" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="E353" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Przód uda, Przywodziciele uda, Plecy</t>
+        </is>
+      </c>
+      <c r="F353" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G353" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H353" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I353" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J353" s="19" t="inlineStr">
+        <is>
+          <t>3 rundy x 30 sek pracy na stronę</t>
+        </is>
+      </c>
+      <c r="K353" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L353" s="19" t="inlineStr">
+        <is>
+          <t>Z przysiadu postaw obie dłonie z jednej strony stóp; Przenieś ciężar na ręce i przenieś stopy bokiem za dłońmi; Pozostań blisko podłoża i ćwicz oba kierunki osobno; Przy bólu nadgarstków lub innych stawów przerwij próbę</t>
+        </is>
+      </c>
+      <c r="M353" s="19" t="inlineStr">
+        <is>
+          <t>Wyrzucanie nóg daleko za siebie; Upadanie na dłonie; Zbyt głęboki bolesny przysiad</t>
+        </is>
+      </c>
+      <c r="N353" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż odcinek ruchu bocznego</t>
+        </is>
+      </c>
+      <c r="O353" s="19" t="inlineStr">
+        <is>
+          <t>Płytszy przysiad i małe przestawienie stóp</t>
+        </is>
+      </c>
+      <c r="P353" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/monkey/</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="19" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" s="19" t="inlineStr">
+        <is>
+          <t>Przemieszczanie żabki z podparciem rąk</t>
+        </is>
+      </c>
+      <c r="C354" s="19" t="inlineStr">
+        <is>
+          <t>GMB Frogger</t>
+        </is>
+      </c>
+      <c r="D354" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="E354" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Przód uda, Plecy, Łydki</t>
+        </is>
+      </c>
+      <c r="F354" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G354" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H354" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I354" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J354" s="19" t="inlineStr">
+        <is>
+          <t>3 rundy x 30 sek pracy</t>
+        </is>
+      </c>
+      <c r="K354" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L354" s="19" t="inlineStr">
+        <is>
+          <t>Z przysiadu sięgnij dłońmi przed siebie; Przenieś ciężar na ręce i unieś biodra, po czym dostaw stopy ku dłoniom; Wyląduj miękko w przysiadzie, nie wykonując wyskoku pionowego; Przy bólu nadgarstków lub innych stawów przerwij próbę</t>
+        </is>
+      </c>
+      <c r="M354" s="19" t="inlineStr">
+        <is>
+          <t>Odbijanie wyłącznie z nóg; Twarde lądowanie; Przeciążenie nadgarstków</t>
+        </is>
+      </c>
+      <c r="N354" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż płynny odcinek przy zachowaniu miękkich lądowań</t>
+        </is>
+      </c>
+      <c r="O354" s="19" t="inlineStr">
+        <is>
+          <t>Mały ruch z płytszego przysiadu</t>
+        </is>
+      </c>
+      <c r="P354" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/frogger/</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="19" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" s="19" t="inlineStr">
+        <is>
+          <t>Przysiad krewetki z chwytem tylnej stopy</t>
+        </is>
+      </c>
+      <c r="C355" s="19" t="inlineStr">
+        <is>
+          <t>Shrimp squat</t>
+        </is>
+      </c>
+      <c r="D355" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E355" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Łydki</t>
+        </is>
+      </c>
+      <c r="F355" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G355" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H355" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I355" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J355" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K355" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L355" s="19" t="inlineStr">
+        <is>
+          <t>Stań na jednej nodze i chwyć stopę drugiej za sobą; Uginaj nogę podporową, prowadząc tylne kolano ku podłodze; Wstań naciskiem całej przedniej stopy bez puszczania tylnej stopy; Przy bólu nadgarstków lub innych stawów przerwij próbę</t>
+        </is>
+      </c>
+      <c r="M355" s="19" t="inlineStr">
+        <is>
+          <t>Opadanie na tylne kolano; Zapadanie kolana podporowego; Odrywanie pięty</t>
+        </is>
+      </c>
+      <c r="N355" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo obniżaj tylne kolano przy zachowaniu kontroli</t>
+        </is>
+      </c>
+      <c r="O355" s="19" t="inlineStr">
+        <is>
+          <t>Płytsze zejście i lekki kontakt wolnej dłoni ze ścianą</t>
+        </is>
+      </c>
+      <c r="P355" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/shrimp-squats/</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="19" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" s="19" t="inlineStr">
+        <is>
+          <t>Przerzut bokiem na obie ręce</t>
+        </is>
+      </c>
+      <c r="C356" s="19" t="inlineStr">
+        <is>
+          <t>Cartwheel</t>
+        </is>
+      </c>
+      <c r="D356" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Triceps</t>
+        </is>
+      </c>
+      <c r="E356" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Pośladki, Przywodziciele uda, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F356" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G356" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H356" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I356" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J356" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K356" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L356" s="19" t="inlineStr">
+        <is>
+          <t>Zapewnij wolny, nieślizgający odcinek podłoża i rozpocznij z wykroku; Postaw kolejno dłoń po stronie nogi prowadzącej i drugą dłoń, przenosząc nogi bokiem; Wyląduj kolejno stopami, zaczynając od niskiej wersji bez pionu; Przy bólu nadgarstków lub innych stawów przerwij próbę</t>
+        </is>
+      </c>
+      <c r="M356" s="19" t="inlineStr">
+        <is>
+          <t>Rzut ciała bez kontroli; Krzyżowanie nóg przy lądowaniu; Próba w ciasnym otoczeniu</t>
+        </is>
+      </c>
+      <c r="N356" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo prostuj nogi i zbliżaj tor do jednej linii</t>
+        </is>
+      </c>
+      <c r="O356" s="19" t="inlineStr">
+        <is>
+          <t>Niskie przejście po łuku, bez unoszenia bioder nad głowę</t>
+        </is>
+      </c>
+      <c r="P356" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/cartwheel/</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="19" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" s="19" t="inlineStr">
+        <is>
+          <t>Most trójpunktowy z sięganiem</t>
+        </is>
+      </c>
+      <c r="C357" s="19" t="inlineStr">
+        <is>
+          <t>Three-point bridge</t>
+        </is>
+      </c>
+      <c r="D357" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Plecy, Barki</t>
+        </is>
+      </c>
+      <c r="E357" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Tył uda, Klatka piersiowa</t>
+        </is>
+      </c>
+      <c r="F357" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G357" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H357" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I357" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J357" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K357" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L357" s="19" t="inlineStr">
+        <is>
+          <t>Z wygodnego przysiadu oprzyj jedną dłoń za biodrem; Naciśnij piętami i unieś biodra, stabilizując bark ręki podporowej; Sięgnij drugą ręką w tył z łagodnym otwarciem klatki, potem wróć; Przy bólu nadgarstków lub innych stawów przerwij próbę</t>
+        </is>
+      </c>
+      <c r="M357" s="19" t="inlineStr">
+        <is>
+          <t>Zapadanie barku podporowego; Skręt wyłącznie w lędźwiach; Ruch przez ból</t>
+        </is>
+      </c>
+      <c r="N357" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż sięganie przy stabilnej dłoni</t>
+        </is>
+      </c>
+      <c r="O357" s="19" t="inlineStr">
+        <is>
+          <t>Podpór na dwóch dłoniach i niższe biodra</t>
+        </is>
+      </c>
+      <c r="P357" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/three-point-bridge/</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="19" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" s="19" t="inlineStr">
+        <is>
+          <t>Podpór żaby na ugiętych ramionach</t>
+        </is>
+      </c>
+      <c r="C358" s="19" t="inlineStr">
+        <is>
+          <t>Crow / frog stand</t>
+        </is>
+      </c>
+      <c r="D358" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="E358" s="19" t="inlineStr">
+        <is>
+          <t>Triceps, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F358" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G358" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H358" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I358" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J358" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K358" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L358" s="19" t="inlineStr">
+        <is>
+          <t>Z przysiadu oprzyj dłonie na szerokość barków i ugnij łokcie; Oprzyj kolana na górze ramion, powoli przenosząc ciężar na dłonie; Unieś stopy tylko przy kontroli, patrząc nieco przed dłonie i zostawiając bezpieczne miejsce przed głową; Przy bólu nadgarstków lub innych stawów przerwij próbę</t>
+        </is>
+      </c>
+      <c r="M358" s="19" t="inlineStr">
+        <is>
+          <t>Wskakiwanie na dłonie; Wstrzymanie oddechu; Zapadanie nadgarstków</t>
+        </is>
+      </c>
+      <c r="N358" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż krótkie udane utrzymania</t>
+        </is>
+      </c>
+      <c r="O358" s="19" t="inlineStr">
+        <is>
+          <t>Palce stóp pozostają na podłodze, bez obciążania głowy</t>
+        </is>
+      </c>
+      <c r="P358" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/crow-pose/</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="19" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" s="19" t="inlineStr">
+        <is>
+          <t>Unoszenie prostej nogi w siadzie z kompresją</t>
+        </is>
+      </c>
+      <c r="C359" s="19" t="inlineStr">
+        <is>
+          <t>Seated single-leg compression raise</t>
+        </is>
+      </c>
+      <c r="D359" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder, Brzuch</t>
+        </is>
+      </c>
+      <c r="E359" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda</t>
+        </is>
+      </c>
+      <c r="F359" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G359" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H359" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I359" s="19" t="inlineStr">
+        <is>
+          <t>Ruch złożony</t>
+        </is>
+      </c>
+      <c r="J359" s="19" t="inlineStr">
+        <is>
+          <t>3 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K359" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L359" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź z jedną nogą prostą, a drugie udo przyciągnij rękami do tułowia; Bez odchylania pleców unieś piętę prostej nogi kilka centymetrów; Opuść kontrolowanie i wykonaj osobną serię na drugą stronę; Przy bólu nadgarstków lub innych stawów przerwij próbę</t>
+        </is>
+      </c>
+      <c r="M359" s="19" t="inlineStr">
+        <is>
+          <t>Odchylanie tułowia; Odbijanie pięty; Zginanie unoszonego kolana</t>
+        </is>
+      </c>
+      <c r="N359" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż zatrzymanie nogi nad podłogą</t>
+        </is>
+      </c>
+      <c r="O359" s="19" t="inlineStr">
+        <is>
+          <t>Mniejsza wysokość unoszenia i krótsza seria</t>
+        </is>
+      </c>
+      <c r="P359" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/l-sit/</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="19" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" s="19" t="inlineStr">
+        <is>
+          <t>Utrzymanie podporu tyłem z ugiętymi nogami</t>
+        </is>
+      </c>
+      <c r="C360" s="19" t="inlineStr">
+        <is>
+          <t>Supine tabletop hold</t>
+        </is>
+      </c>
+      <c r="D360" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Barki, Tył uda</t>
+        </is>
+      </c>
+      <c r="E360" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Triceps, Plecy</t>
+        </is>
+      </c>
+      <c r="F360" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G360" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H360" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I360" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="J360" s="19" t="inlineStr">
+        <is>
+          <t>2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K360" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L360" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź z ugiętymi nogami i oprzyj dłonie za biodrami; Naciśnij stopami oraz dłońmi i unieś biodra do wygodnej wysokości; Utrzymuj otwartą klatkę bez marszu, z szyją w przedłużeniu tułowia; Przy bólu nadgarstków lub innych stawów przerwij próbę</t>
+        </is>
+      </c>
+      <c r="M360" s="19" t="inlineStr">
+        <is>
+          <t>Zapadanie barków; Odrzucanie głowy; Zbyt duży przeprost lędźwi</t>
+        </is>
+      </c>
+      <c r="N360" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż stabilne utrzymanie</t>
+        </is>
+      </c>
+      <c r="O360" s="19" t="inlineStr">
+        <is>
+          <t>Niższe biodra i krótsze utrzymanie</t>
+        </is>
+      </c>
+      <c r="P360" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/three-point-bridge/</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="19" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" s="19" t="inlineStr">
+        <is>
+          <t>Tai chi — zbieranie wiśni w siadzie</t>
+        </is>
+      </c>
+      <c r="C361" s="19" t="inlineStr">
+        <is>
+          <t>Picking Cherries (seated)</t>
+        </is>
+      </c>
+      <c r="D361" s="19" t="inlineStr">
+        <is>
+          <t>Barki</t>
+        </is>
+      </c>
+      <c r="E361" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Brzuch</t>
+        </is>
+      </c>
+      <c r="F361" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G361" s="19" t="inlineStr">
+        <is>
+          <t>Regeneracja</t>
+        </is>
+      </c>
+      <c r="H361" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I361" s="19" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="J361" s="19" t="inlineStr">
+        <is>
+          <t>2 x 8-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K361" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L361" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź na stabilnym krześle bez kółek, stopy oprzyj na podłodze; Sięgaj jedną dłonią po wyobrażoną wiśnię nad głową, potem przed sobą i w bok; Wracaj dłonią bez szarpania i zmieniaj rękę, nie odrywając pośladków od siedziska; Oddychaj naturalnie i wykonuj ruch powoli, bez bólu ani naprężania</t>
+        </is>
+      </c>
+      <c r="M361" s="19" t="inlineStr">
+        <is>
+          <t>Unoszenie barku do ucha; Przechylanie się poza stabilną podstawę</t>
+        </is>
+      </c>
+      <c r="N361" s="19" t="inlineStr">
+        <is>
+          <t>Płynnie łącz kierunki sięgania w bezbolesnym zakresie</t>
+        </is>
+      </c>
+      <c r="O361" s="19" t="inlineStr">
+        <is>
+          <t>Sięgaj niżej i bliżej tułowia</t>
+        </is>
+      </c>
+      <c r="P361" s="19" t="inlineStr">
+        <is>
+          <t>https://www.taichiexercises.co.uk/wp-content/uploads/2020/05/Exercises-Seated.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="19" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" s="19" t="inlineStr">
+        <is>
+          <t>Tai chi — wiosłowanie łodzią w siadzie</t>
+        </is>
+      </c>
+      <c r="C362" s="19" t="inlineStr">
+        <is>
+          <t>Rowing a Boat (seated)</t>
+        </is>
+      </c>
+      <c r="D362" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Brzuch</t>
+        </is>
+      </c>
+      <c r="E362" s="19" t="inlineStr">
+        <is>
+          <t>Barki</t>
+        </is>
+      </c>
+      <c r="F362" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G362" s="19" t="inlineStr">
+        <is>
+          <t>Regeneracja</t>
+        </is>
+      </c>
+      <c r="H362" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I362" s="19" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="J362" s="19" t="inlineStr">
+        <is>
+          <t>2 x 8-10</t>
+        </is>
+      </c>
+      <c r="K362" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L362" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź na stabilnym krześle bez kółek, stopy oprzyj na podłodze; Łagodnie przenoś tułów w przód i w tył z bioder; Dodaj oburącz krążenie ramion jak przy prowadzeniu wioseł po bokach łodzi, utrzymując stopy nieruchomo; Oddychaj naturalnie i wykonuj ruch powoli, bez bólu ani naprężania</t>
+        </is>
+      </c>
+      <c r="M362" s="19" t="inlineStr">
+        <is>
+          <t>Gwałtowne bujanie; Zaokrąglanie samych lędźwi; Utrata kontaktu stóp z podłożem</t>
+        </is>
+      </c>
+      <c r="N362" s="19" t="inlineStr">
+        <is>
+          <t>Łącz ruch ramion i tułowia coraz płynniej</t>
+        </is>
+      </c>
+      <c r="O362" s="19" t="inlineStr">
+        <is>
+          <t>Małe wychylenia z dłońmi bliżej ud</t>
+        </is>
+      </c>
+      <c r="P362" s="19" t="inlineStr">
+        <is>
+          <t>https://www.taichiexercises.co.uk/wp-content/uploads/2020/05/Exercises-Seated.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="19" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" s="19" t="inlineStr">
+        <is>
+          <t>Tai chi — żółw pływający w oceanie w siadzie</t>
+        </is>
+      </c>
+      <c r="C363" s="19" t="inlineStr">
+        <is>
+          <t>Turtle Swims in the Ocean (seated)</t>
+        </is>
+      </c>
+      <c r="D363" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Plecy</t>
+        </is>
+      </c>
+      <c r="E363" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Klatka piersiowa</t>
+        </is>
+      </c>
+      <c r="F363" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G363" s="19" t="inlineStr">
+        <is>
+          <t>Regeneracja</t>
+        </is>
+      </c>
+      <c r="H363" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I363" s="19" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="J363" s="19" t="inlineStr">
+        <is>
+          <t>2 x 8-10</t>
+        </is>
+      </c>
+      <c r="K363" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L363" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź na stabilnym krześle bez kółek, stopy oprzyj na podłodze; Przy łagodnym pochyleniu wykonaj ramionami ruch podobny do pływania żabką; Przy powrocie prowadź ramiona szerokim łukiem jak w stylu motylkowym, bez odrzucania pleców; Zmień kierunek krążenia w kolejnej krótkiej serii; Oddychaj naturalnie i wykonuj ruch powoli, bez bólu ani naprężania</t>
+        </is>
+      </c>
+      <c r="M363" s="19" t="inlineStr">
+        <is>
+          <t>Forsowanie barków za plecy; Szarpanie tułowiem; Zatrzymywanie oddechu</t>
+        </is>
+      </c>
+      <c r="N363" s="19" t="inlineStr">
+        <is>
+          <t>Łącz oba kierunki przy jednakowo spokojnym tempie</t>
+        </is>
+      </c>
+      <c r="O363" s="19" t="inlineStr">
+        <is>
+          <t>Małe łuki ramion bez wychylania tułowia</t>
+        </is>
+      </c>
+      <c r="P363" s="19" t="inlineStr">
+        <is>
+          <t>https://www.taichiexercises.co.uk/wp-content/uploads/2020/05/Exercises-Seated.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="19" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" s="19" t="inlineStr">
+        <is>
+          <t>Tai chi — otwieranie drzwi podeszwą w siadzie</t>
+        </is>
+      </c>
+      <c r="C364" s="19" t="inlineStr">
+        <is>
+          <t>Kick with Sole (seated)</t>
+        </is>
+      </c>
+      <c r="D364" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda</t>
+        </is>
+      </c>
+      <c r="E364" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder, Brzuch, Przód goleni</t>
+        </is>
+      </c>
+      <c r="F364" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G364" s="19" t="inlineStr">
+        <is>
+          <t>Regeneracja</t>
+        </is>
+      </c>
+      <c r="H364" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I364" s="19" t="inlineStr">
+        <is>
+          <t>Flow</t>
+        </is>
+      </c>
+      <c r="J364" s="19" t="inlineStr">
+        <is>
+          <t>2 x 8-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K364" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i kontrolowanie, fazy dynamiczne bez szarpania</t>
+        </is>
+      </c>
+      <c r="L364" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź na stabilnym krześle bez kółek, stopy oprzyj na podłodze; Powoli wyprostuj jedną nogę przed sobą; Skieruj podeszwę w przód jak przy łagodnym otwieraniu drzwi piętą, nie kopiąc gwałtownie; Cofnij stopę na podłogę i zmień nogę; Oddychaj naturalnie i wykonuj ruch powoli, bez bólu ani naprężania</t>
+        </is>
+      </c>
+      <c r="M364" s="19" t="inlineStr">
+        <is>
+          <t>Gwałtowny wyprost kolana; Odchylanie pleców; Unoszenie całego uda wysoko</t>
+        </is>
+      </c>
+      <c r="N364" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż spokojny wyprost bez blokowania kolana</t>
+        </is>
+      </c>
+      <c r="O364" s="19" t="inlineStr">
+        <is>
+          <t>Prostuj kolano tylko częściowo, pięta blisko podłogi</t>
+        </is>
+      </c>
+      <c r="P364" s="19" t="inlineStr">
+        <is>
+          <t>https://www.taichiexercises.co.uk/wp-content/uploads/2020/05/Exercises-Seated.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: release guided training and cloud exercise variants
</commit_message>
<xml_diff>
--- a/tools/source_data/baza_cwiczen_316.xlsx
+++ b/tools/source_data/baza_cwiczen_316.xlsx
@@ -813,6 +813,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="24" customHeight="1" s="39">
       <c r="A8" s="4" t="inlineStr">
         <is>
@@ -964,6 +965,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="24" customHeight="1" s="39">
       <c r="A22" s="4" t="inlineStr">
         <is>
@@ -1163,6 +1165,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40" ht="24" customHeight="1" s="39">
       <c r="A40" s="4" t="inlineStr">
         <is>
@@ -1266,6 +1269,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50" ht="24" customHeight="1" s="39">
       <c r="A50" s="4" t="inlineStr">
         <is>
@@ -1336,6 +1340,7 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58" ht="24" customHeight="1" s="39">
       <c r="A58" s="4" t="inlineStr">
         <is>
@@ -1379,6 +1384,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63" ht="24" customHeight="1" s="39">
       <c r="A63" s="4" t="inlineStr">
         <is>
@@ -1470,6 +1476,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72" ht="24" customHeight="1" s="39">
       <c r="A72" s="4" t="inlineStr">
         <is>
@@ -1681,6 +1688,7 @@
         </is>
       </c>
     </row>
+    <row r="90"/>
     <row r="91" ht="24" customHeight="1" s="39">
       <c r="A91" s="12" t="inlineStr">
         <is>
@@ -1784,6 +1792,7 @@
         </is>
       </c>
     </row>
+    <row r="100"/>
     <row r="101" ht="24" customHeight="1" s="39">
       <c r="A101" s="4" t="inlineStr">
         <is>
@@ -1923,6 +1932,7 @@
         </is>
       </c>
     </row>
+    <row r="113"/>
     <row r="114" ht="24" customHeight="1" s="39">
       <c r="A114" s="4" t="inlineStr">
         <is>
@@ -8435,7 +8445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P364"/>
+  <dimension ref="A1:P370"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.8515625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.00390625" customWidth="1" style="39" min="1" max="1"/>
@@ -37570,6 +37580,486 @@
       <c r="P364" s="19" t="inlineStr">
         <is>
           <t>https://www.taichiexercises.co.uk/wp-content/uploads/2020/05/Exercises-Seated.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="19" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" s="19" t="inlineStr">
+        <is>
+          <t>Przetaczanie miednicy w leżeniu na plecach</t>
+        </is>
+      </c>
+      <c r="C365" s="19" t="inlineStr">
+        <is>
+          <t>Supine pelvic tilt</t>
+        </is>
+      </c>
+      <c r="D365" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E365" s="19" t="inlineStr">
+        <is>
+          <t>Plecy</t>
+        </is>
+      </c>
+      <c r="F365" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G365" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H365" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I365" s="19" t="inlineStr">
+        <is>
+          <t>Kontrola pochylenia miednicy</t>
+        </is>
+      </c>
+      <c r="J365" s="19" t="inlineStr">
+        <is>
+          <t>1 x 3-5</t>
+        </is>
+      </c>
+      <c r="K365" s="19" t="inlineStr">
+        <is>
+          <t>Wolno, około 2 sek w każdą stronę</t>
+        </is>
+      </c>
+      <c r="L365" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na plecach, ugnij kolana i oprzyj stopy o podłogę; Rozluźnij barki i połóż dłonie na miednicy; Łagodnie podwiń miednicę, zmniejszając szczelinę pod lędźwiami; Następnie pochyl miednicę w przeciwną stronę, tworząc tylko niewielką szczelinę; Pośladki pozostają na podłożu, oddychaj swobodnie; Pełne przetoczenie tam i z powrotem to jedno powtórzenie; Przerwij przy bólu, nasileniu objawów lub drętwieniu i skonsultuj dalszy ruch ze specjalistą</t>
+        </is>
+      </c>
+      <c r="M365" s="19" t="inlineStr">
+        <is>
+          <t>Unoszenie bioder jak w moście; Wypychanie brzucha i duży przeprost lędźwi; Zatrzymywanie oddechu</t>
+        </is>
+      </c>
+      <c r="N365" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj 1-2 powtórzenia, jeśli ruch pozostaje swobodny, bez zwiększania wygięcia</t>
+        </is>
+      </c>
+      <c r="O365" s="19" t="inlineStr">
+        <is>
+          <t>Wykonuj bardzo mały ruch miednicy i wracaj do wygodnej pozycji</t>
+        </is>
+      </c>
+      <c r="P365" s="19" t="inlineStr">
+        <is>
+          <t>https://www.cuh.nhs.uk/patient-information/back-mobility-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="19" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" s="19" t="inlineStr">
+        <is>
+          <t>Łagodne napięcie brzucha w leżeniu z normalnym oddechem</t>
+        </is>
+      </c>
+      <c r="C366" s="19" t="inlineStr">
+        <is>
+          <t>Supine abdominal bracing</t>
+        </is>
+      </c>
+      <c r="D366" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E366" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F366" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G366" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H366" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I366" s="19" t="inlineStr">
+        <is>
+          <t>Stabilizacja tułowia bez ruchu kończyn</t>
+        </is>
+      </c>
+      <c r="J366" s="19" t="inlineStr">
+        <is>
+          <t>3 x 5 sek</t>
+        </is>
+      </c>
+      <c r="K366" s="19" t="inlineStr">
+        <is>
+          <t>Spokojny oddech przez całe utrzymanie, odpoczynek po każdym napięciu</t>
+        </is>
+      </c>
+      <c r="L366" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na plecach z ugiętymi kolanami, stopami na podłodze i rękami przy tułowiu; Łagodnie napnij dolną część brzucha, jak przy odsuwaniu go od paska spodni; Nie unoś głowy ani barków, nie poruszaj nogami i nie wyginaj lędźwi; Utrzymuj lekkie napięcie przez 5 sek, swobodnie wdychając i wydychając powietrze; Rozluźnij brzuch całkowicie i odpocznij przed kolejnym napięciem; Przerwij przy bólu, nasileniu objawów lub drętwieniu i skonsultuj dalszy ruch ze specjalistą</t>
+        </is>
+      </c>
+      <c r="M366" s="19" t="inlineStr">
+        <is>
+          <t>Wstrzymywanie oddechu lub parcie; Maksymalne wciąganie brzucha; Unoszenie tułowia jak przy spięciu brzucha</t>
+        </is>
+      </c>
+      <c r="N366" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż lekkie napięcie do 8-10 sek tylko przy swobodnym oddychaniu</t>
+        </is>
+      </c>
+      <c r="O366" s="19" t="inlineStr">
+        <is>
+          <t>Skróć napięcie do 2-3 sek lub zmniejsz jego siłę</t>
+        </is>
+      </c>
+      <c r="P366" s="19" t="inlineStr">
+        <is>
+          <t>https://orthoinfo.aaos.org/en/recovery/spine-conditioning-program/</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="19" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" s="19" t="inlineStr">
+        <is>
+          <t>Kołysanie ugiętych kolan w leżeniu na plecach</t>
+        </is>
+      </c>
+      <c r="C367" s="19" t="inlineStr">
+        <is>
+          <t>Supine bent-knee rolls</t>
+        </is>
+      </c>
+      <c r="D367" s="19" t="inlineStr">
+        <is>
+          <t>Plecy</t>
+        </is>
+      </c>
+      <c r="E367" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Pośladki</t>
+        </is>
+      </c>
+      <c r="F367" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G367" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H367" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I367" s="19" t="inlineStr">
+        <is>
+          <t>Łagodna rotacja tułowia w leżeniu</t>
+        </is>
+      </c>
+      <c r="J367" s="19" t="inlineStr">
+        <is>
+          <t>1 x 3 na stronę</t>
+        </is>
+      </c>
+      <c r="K367" s="19" t="inlineStr">
+        <is>
+          <t>Powolne opuszczenie i powrót, krótka pauza bez dociskania</t>
+        </is>
+      </c>
+      <c r="L367" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na plecach z kolanami ugiętymi i złączonymi, stopy na podłodze; Oprzyj ramiona wygodnie obok tułowia, barki pozostają na podłożu; Przechyl oba kolana razem w wybraną stronę tylko w komfortowym zakresie; Pozwól stopom lekko przetoczyć się na krawędzie, bez unoszenia nóg w powietrze; Powoli wróć do środka, oddychając normalnie; Wyjście w bok i powrót to jedno powtórzenie na tę stronę; Przerwij przy bólu, nasileniu objawów lub drętwieniu i skonsultuj dalszy ruch ze specjalistą</t>
+        </is>
+      </c>
+      <c r="M367" s="19" t="inlineStr">
+        <is>
+          <t>Odrywanie barków; Dociskanie kolan do podłogi ręką; Szybkie przerzucanie nóg</t>
+        </is>
+      </c>
+      <c r="N367" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj 1-2 spokojne powtórzenia na stronę bez pogłębiania skrętu na siłę</t>
+        </is>
+      </c>
+      <c r="O367" s="19" t="inlineStr">
+        <is>
+          <t>Zmniejsz wychylenie kolan i wracaj do środka bez pauzy</t>
+        </is>
+      </c>
+      <c r="P367" s="19" t="inlineStr">
+        <is>
+          <t>https://www.cuh.nhs.uk/patient-information/back-mobility-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="19" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" s="19" t="inlineStr">
+        <is>
+          <t>Otwarta książka — obrót klatki w leżeniu bokiem</t>
+        </is>
+      </c>
+      <c r="C368" s="19" t="inlineStr">
+        <is>
+          <t>Side-lying open book</t>
+        </is>
+      </c>
+      <c r="D368" s="19" t="inlineStr">
+        <is>
+          <t>Plecy</t>
+        </is>
+      </c>
+      <c r="E368" s="19" t="inlineStr">
+        <is>
+          <t>Klatka piersiowa, Brzuch, Barki</t>
+        </is>
+      </c>
+      <c r="F368" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G368" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H368" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I368" s="19" t="inlineStr">
+        <is>
+          <t>Rotacja piersiowa w leżeniu bokiem</t>
+        </is>
+      </c>
+      <c r="J368" s="19" t="inlineStr">
+        <is>
+          <t>1 x 3-5 na stronę</t>
+        </is>
+      </c>
+      <c r="K368" s="19" t="inlineStr">
+        <is>
+          <t>Wolne otwarcie ramienia i kontrolowany powrót</t>
+        </is>
+      </c>
+      <c r="L368" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na boku z biodrami i kolanami ugiętymi, kolana razem na podłodze; Wyciągnij obie ręce przed klatkę, dłoń na dłoni, głowę ułóż wygodnie; Zatocz górnym ramieniem łuk w górę i za siebie, obracając klatkę piersiową; Wzrok może podążać za dłonią, ale nie wymuszaj skrętu szyi; Kolana pozostają razem na podłożu, nie próbuj koniecznie dotknąć tylną dłonią podłogi; Wróć dłonią na dłoń i oddychaj swobodnie, następnie zmień bok; Przerwij przy bólu, nasileniu objawów lub drętwieniu i skonsultuj dalszy ruch ze specjalistą</t>
+        </is>
+      </c>
+      <c r="M368" s="19" t="inlineStr">
+        <is>
+          <t>Odrywanie górnego kolana i przetaczanie całego ciała; Dociskanie ramienia do podłogi; Wymuszanie zakresu barku lub szyi</t>
+        </is>
+      </c>
+      <c r="N368" s="19" t="inlineStr">
+        <is>
+          <t>Zwiększ do 5 swobodnych powtórzeń na stronę, bez ciężaru i dociskania</t>
+        </is>
+      </c>
+      <c r="O368" s="19" t="inlineStr">
+        <is>
+          <t>Otwórz ramię tylko częściowo i pozostaw wzrok przed sobą</t>
+        </is>
+      </c>
+      <c r="P368" s="19" t="inlineStr">
+        <is>
+          <t>https://flipbooks.leedsth.nhs.uk/LN005629.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="19" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" s="19" t="inlineStr">
+        <is>
+          <t>Przyciąganie jednego kolana do klatki w leżeniu</t>
+        </is>
+      </c>
+      <c r="C369" s="19" t="inlineStr">
+        <is>
+          <t>Supine single knee to chest</t>
+        </is>
+      </c>
+      <c r="D369" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Mięsień czworoboczny lędźwi</t>
+        </is>
+      </c>
+      <c r="E369" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki</t>
+        </is>
+      </c>
+      <c r="F369" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G369" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H369" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I369" s="19" t="inlineStr">
+        <is>
+          <t>Zgięcie biodra z łagodnym rozciąganiem pleców</t>
+        </is>
+      </c>
+      <c r="J369" s="19" t="inlineStr">
+        <is>
+          <t>1 x 3 na stronę</t>
+        </is>
+      </c>
+      <c r="K369" s="19" t="inlineStr">
+        <is>
+          <t>Powolne przyciągnięcie, 2-3 sek pauzy i spokojne odłożenie</t>
+        </is>
+      </c>
+      <c r="L369" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na plecach, ugnij oba kolana i oprzyj stopy na podłodze; Unieś jedno kolano ku klatce i obejmij nogę dłońmi, bez mocnego nacisku na kolano; Druga stopa zostaje na podłodze, jej kolano skierowane ku sufitowi; Przybliż udo tylko do łagodnego uczucia rozciągania, głowa i barki zostają na podłożu; Oddychaj normalnie przez krótką pauzę, powoli odstaw stopę; Przyciągnięcie i powrót to jedno powtórzenie na stronę; Przerwij przy bólu, nasileniu objawów lub drętwieniu i skonsultuj dalszy ruch ze specjalistą</t>
+        </is>
+      </c>
+      <c r="M369" s="19" t="inlineStr">
+        <is>
+          <t>Mocne szarpanie nogi; Unoszenie głowy do kolana; Prostowanie drugiej nogi mimo dyskomfortu lędźwi</t>
+        </is>
+      </c>
+      <c r="N369" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj 1-2 powtórzenia na stronę bez silniejszego ciągnięcia</t>
+        </is>
+      </c>
+      <c r="O369" s="19" t="inlineStr">
+        <is>
+          <t>Obejmij udo od tyłu i przyciągnij je mniej, druga stopa nadal na podłodze</t>
+        </is>
+      </c>
+      <c r="P369" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nhsinform.scot/illnesses-and-conditions/muscle-bone-and-joints/neck-and-back-problems-and-conditions/exercises-for-back-pain</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="19" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" s="19" t="inlineStr">
+        <is>
+          <t>Cofanie bioder do ściany bez obciążenia</t>
+        </is>
+      </c>
+      <c r="C370" s="19" t="inlineStr">
+        <is>
+          <t>Bodyweight wall hip hinge</t>
+        </is>
+      </c>
+      <c r="D370" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Tył uda</t>
+        </is>
+      </c>
+      <c r="E370" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Brzuch</t>
+        </is>
+      </c>
+      <c r="F370" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G370" s="19" t="inlineStr">
+        <is>
+          <t>Rozgrzewka</t>
+        </is>
+      </c>
+      <c r="H370" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I370" s="19" t="inlineStr">
+        <is>
+          <t>Zawias biodrowy z kontrolą tułowia</t>
+        </is>
+      </c>
+      <c r="J370" s="19" t="inlineStr">
+        <is>
+          <t>1 x 5</t>
+        </is>
+      </c>
+      <c r="K370" s="19" t="inlineStr">
+        <is>
+          <t>Około 3 sek cofania bioder, lekki dotyk ściany i spokojny powrót</t>
+        </is>
+      </c>
+      <c r="L370" s="19" t="inlineStr">
+        <is>
+          <t>Stań tyłem kilka centymetrów od stabilnej ściany, stopy na szerokość bioder; Lekko ugnij kolana, połóż dłonie w zgięciach bioder; Cofaj biodra do lekkiego dotknięcia ściany pośladkami, pochylając tułów z bioder; Zachowaj wygodne ustawienie kręgosłupa i szyi, stopy cały czas na podłodze; Nie siadaj w przysiad ani nie zaokrąglaj pleców, wróć do stania przez wyprost bioder; Oddychaj swobodnie, bez dodawania ciężaru i bez wypychania lędźwi w przód; Przerwij przy bólu, nasileniu objawów lub drętwieniu i skonsultuj dalszy ruch ze specjalistą</t>
+        </is>
+      </c>
+      <c r="M370" s="19" t="inlineStr">
+        <is>
+          <t>Zaokrąglanie pleców zamiast ruchu bioder; Głęboki przysiad; Uderzanie pośladkami o ścianę lub odchylanie tułowia po powrocie</t>
+        </is>
+      </c>
+      <c r="N370" s="19" t="inlineStr">
+        <is>
+          <t>Odsuń stopy o 2-3 cm od ściany tylko przy zachowaniu kontroli, nadal bez obciążenia</t>
+        </is>
+      </c>
+      <c r="O370" s="19" t="inlineStr">
+        <is>
+          <t>Stań bliżej ściany i skróć cofnięcie bioder</t>
+        </is>
+      </c>
+      <c r="P370" s="19" t="inlineStr">
+        <is>
+          <t>https://www.peakrxtherapy.com/blog/hip-hinging-101</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: expand exercise catalog with partner training; release 1.19.0+34
</commit_message>
<xml_diff>
--- a/tools/source_data/baza_cwiczen_316.xlsx
+++ b/tools/source_data/baza_cwiczen_316.xlsx
@@ -8445,7 +8445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P370"/>
+  <dimension ref="A1:P409"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.8515625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.00390625" customWidth="1" style="39" min="1" max="1"/>
@@ -38060,6 +38060,3126 @@
       <c r="P370" s="19" t="inlineStr">
         <is>
           <t>https://www.peakrxtherapy.com/blog/hip-hinging-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="19" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" s="19" t="inlineStr">
+        <is>
+          <t>Wstawanie z krzesła</t>
+        </is>
+      </c>
+      <c r="C371" s="19" t="inlineStr">
+        <is>
+          <t>Sit to stand</t>
+        </is>
+      </c>
+      <c r="D371" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E371" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="F371" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G371" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H371" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I371" s="19" t="inlineStr">
+        <is>
+          <t>Sit to stand</t>
+        </is>
+      </c>
+      <c r="J371" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K371" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L371" s="19" t="inlineStr">
+        <is>
+          <t>Ustaw stabilne krzesło przy ścianie; Usiądź bliżej krawędzi, stopy płasko; Pochyl tułów z bioder i wstań; Powoli usiądź bez opadania; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M371" s="19" t="inlineStr">
+        <is>
+          <t>Opadanie na siedzisko; Zapadanie kolan do środka</t>
+        </is>
+      </c>
+      <c r="N371" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O371" s="19" t="inlineStr">
+        <is>
+          <t>Wyższe siedzisko i pomoc dłoni</t>
+        </is>
+      </c>
+      <c r="P371" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/live-well/exercise/strength-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="19" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" s="19" t="inlineStr">
+        <is>
+          <t>Odwodzenie prostej nogi w staniu z podparciem</t>
+        </is>
+      </c>
+      <c r="C372" s="19" t="inlineStr">
+        <is>
+          <t>Supported standing hip abduction</t>
+        </is>
+      </c>
+      <c r="D372" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki</t>
+        </is>
+      </c>
+      <c r="E372" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="F372" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G372" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H372" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I372" s="19" t="inlineStr">
+        <is>
+          <t>Supported standing hip abduction</t>
+        </is>
+      </c>
+      <c r="J372" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K372" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L372" s="19" t="inlineStr">
+        <is>
+          <t>Zabezpiecz krzesło przy ścianie, chwyć oparcie; Stań prosto; Unieś nogę w bok bez obrotu miednicy; Spokojnie opuść i zmień stronę; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M372" s="19" t="inlineStr">
+        <is>
+          <t>Przechylanie tułowia; Wymachiwanie nogą</t>
+        </is>
+      </c>
+      <c r="N372" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O372" s="19" t="inlineStr">
+        <is>
+          <t>Mniejszy zakres i obie dłonie na podporze</t>
+        </is>
+      </c>
+      <c r="P372" s="19" t="inlineStr">
+        <is>
+          <t>https://www.uhsussex.nhs.uk/resources/standing-exercises</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="19" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" s="19" t="inlineStr">
+        <is>
+          <t>Prostowanie biodra w staniu z podparciem</t>
+        </is>
+      </c>
+      <c r="C373" s="19" t="inlineStr">
+        <is>
+          <t>Supported standing hip extension</t>
+        </is>
+      </c>
+      <c r="D373" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki</t>
+        </is>
+      </c>
+      <c r="E373" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Brzuch</t>
+        </is>
+      </c>
+      <c r="F373" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G373" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H373" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I373" s="19" t="inlineStr">
+        <is>
+          <t>Supported standing hip extension</t>
+        </is>
+      </c>
+      <c r="J373" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K373" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L373" s="19" t="inlineStr">
+        <is>
+          <t>Zabezpiecz krzesło przed przesuwaniem; Przytrzymaj oparcie; Przesuń prostą nogę nieznacznie za siebie; Wróć bez przeprostu pleców; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M373" s="19" t="inlineStr">
+        <is>
+          <t>Wyginanie lędźwi; Pochylanie tułowia</t>
+        </is>
+      </c>
+      <c r="N373" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O373" s="19" t="inlineStr">
+        <is>
+          <t>Krótszy ruch bez wysokiego unoszenia nogi</t>
+        </is>
+      </c>
+      <c r="P373" s="19" t="inlineStr">
+        <is>
+          <t>https://www.uhsussex.nhs.uk/resources/standing-exercises</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="19" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" s="19" t="inlineStr">
+        <is>
+          <t>Odwodzenie prostej nogi w leżeniu bokiem</t>
+        </is>
+      </c>
+      <c r="C374" s="19" t="inlineStr">
+        <is>
+          <t>Side lying straight leg abduction</t>
+        </is>
+      </c>
+      <c r="D374" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki</t>
+        </is>
+      </c>
+      <c r="E374" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="F374" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G374" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H374" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I374" s="19" t="inlineStr">
+        <is>
+          <t>Side lying straight leg abduction</t>
+        </is>
+      </c>
+      <c r="J374" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K374" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L374" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na boku z podpartą głową; Ugnij dolną nogę; Unieś prostą górną nogę bez obracania bioder; Powoli opuść i zmień bok; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M374" s="19" t="inlineStr">
+        <is>
+          <t>Obracanie palców ku sufitowi; Kołysanie tułowiem</t>
+        </is>
+      </c>
+      <c r="N374" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O374" s="19" t="inlineStr">
+        <is>
+          <t>Niższe uniesienie</t>
+        </is>
+      </c>
+      <c r="P374" s="19" t="inlineStr">
+        <is>
+          <t>https://orthoinfo.aaos.org/en/recovery/hip-conditioning-program</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="19" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" s="19" t="inlineStr">
+        <is>
+          <t>Przywodzenie dolnej nogi w leżeniu bokiem</t>
+        </is>
+      </c>
+      <c r="C375" s="19" t="inlineStr">
+        <is>
+          <t>Side lying lower leg adduction</t>
+        </is>
+      </c>
+      <c r="D375" s="19" t="inlineStr">
+        <is>
+          <t>Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="E375" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="F375" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G375" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H375" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I375" s="19" t="inlineStr">
+        <is>
+          <t>Side lying lower leg adduction</t>
+        </is>
+      </c>
+      <c r="J375" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K375" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L375" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na boku; Przełóż ugiętą górną nogę przed dolną, stopa oparta; Dolną nogę unieś nieznacznie; Opuść i zmień bok; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M375" s="19" t="inlineStr">
+        <is>
+          <t>Przetaczanie na plecy; Szarpanie</t>
+        </is>
+      </c>
+      <c r="N375" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O375" s="19" t="inlineStr">
+        <is>
+          <t>Mały ruch bez bólu pachwiny</t>
+        </is>
+      </c>
+      <c r="P375" s="19" t="inlineStr">
+        <is>
+          <t>https://orthoinfo.aaos.org/en/recovery/hip-conditioning-program</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="19" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" s="19" t="inlineStr">
+        <is>
+          <t>Uginanie nogi z gumą w leżeniu na brzuchu</t>
+        </is>
+      </c>
+      <c r="C376" s="19" t="inlineStr">
+        <is>
+          <t>Prone band hamstring curl</t>
+        </is>
+      </c>
+      <c r="D376" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda</t>
+        </is>
+      </c>
+      <c r="E376" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F376" s="19" t="inlineStr">
+        <is>
+          <t>Gumy oporowe</t>
+        </is>
+      </c>
+      <c r="G376" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H376" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I376" s="19" t="inlineStr">
+        <is>
+          <t>Prone band hamstring curl</t>
+        </is>
+      </c>
+      <c r="J376" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K376" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L376" s="19" t="inlineStr">
+        <is>
+          <t>Zamocuj gumę nisko od strony stóp i zabezpiecz mocowanie przy kostce; Połóż się na brzuchu; Zbliż piętę do pośladka zginając kolano; Powoli wyprostuj bez unoszenia uda; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M376" s="19" t="inlineStr">
+        <is>
+          <t>Wyginanie pleców; Odrywanie uda; Niepewny zaczep</t>
+        </is>
+      </c>
+      <c r="N376" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O376" s="19" t="inlineStr">
+        <is>
+          <t>Słabsza guma i krótszy zakres</t>
+        </is>
+      </c>
+      <c r="P376" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/everyone/exercise-library/131/prone-lying-hamstrings-curl/</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="19" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" s="19" t="inlineStr">
+        <is>
+          <t>Prostowanie kolana z gumą w siadzie</t>
+        </is>
+      </c>
+      <c r="C377" s="19" t="inlineStr">
+        <is>
+          <t>Seated band knee extension</t>
+        </is>
+      </c>
+      <c r="D377" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda</t>
+        </is>
+      </c>
+      <c r="E377" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F377" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło, Gumy oporowe</t>
+        </is>
+      </c>
+      <c r="G377" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H377" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I377" s="19" t="inlineStr">
+        <is>
+          <t>Seated band knee extension</t>
+        </is>
+      </c>
+      <c r="J377" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K377" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L377" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź na stabilnym krześle z podpartym udem; Zabezpiecz gumę przy kostce i nieruchomym zaczepie za sobą; Wyprostuj kolano w wygodnym zakresie; Powoli wróć; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M377" s="19" t="inlineStr">
+        <is>
+          <t>Podrzucanie nogi; Odrywanie uda; Przesuwanie siedziska przez gumę</t>
+        </is>
+      </c>
+      <c r="N377" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O377" s="19" t="inlineStr">
+        <is>
+          <t>Ruch bez gumy</t>
+        </is>
+      </c>
+      <c r="P377" s="19" t="inlineStr">
+        <is>
+          <t>https://musclewiki.com/exercise/band-leg-extension</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="19" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" s="19" t="inlineStr">
+        <is>
+          <t>Wyprost bioder z przeciąganiem gumy między nogami</t>
+        </is>
+      </c>
+      <c r="C378" s="19" t="inlineStr">
+        <is>
+          <t>Band pull through</t>
+        </is>
+      </c>
+      <c r="D378" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Tył uda</t>
+        </is>
+      </c>
+      <c r="E378" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy</t>
+        </is>
+      </c>
+      <c r="F378" s="19" t="inlineStr">
+        <is>
+          <t>Gumy oporowe</t>
+        </is>
+      </c>
+      <c r="G378" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H378" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I378" s="19" t="inlineStr">
+        <is>
+          <t>Band pull through</t>
+        </is>
+      </c>
+      <c r="J378" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K378" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L378" s="19" t="inlineStr">
+        <is>
+          <t>Zabezpiecz niski zaczep za plecami; Stań tyłem i chwyć gumę między nogami; Cofnij biodra przy miękkich kolanach; Wyprostuj biodra do pionu bez odchylenia w tył; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M378" s="19" t="inlineStr">
+        <is>
+          <t>Przysiad zamiast ruchu bioder; Przeprost lędźwi</t>
+        </is>
+      </c>
+      <c r="N378" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O378" s="19" t="inlineStr">
+        <is>
+          <t>Słabsza guma lub cofanie bioder do ściany cw369</t>
+        </is>
+      </c>
+      <c r="P378" s="19" t="inlineStr">
+        <is>
+          <t>https://musclewiki.com/exercise/band-pullthrough</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="19" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" s="19" t="inlineStr">
+        <is>
+          <t>Przywodzenie nogi z gumą w staniu</t>
+        </is>
+      </c>
+      <c r="C379" s="19" t="inlineStr">
+        <is>
+          <t>Standing band hip adduction</t>
+        </is>
+      </c>
+      <c r="D379" s="19" t="inlineStr">
+        <is>
+          <t>Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="E379" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F379" s="19" t="inlineStr">
+        <is>
+          <t>Gumy oporowe, Krzesło</t>
+        </is>
+      </c>
+      <c r="G379" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H379" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I379" s="19" t="inlineStr">
+        <is>
+          <t>Standing band hip adduction</t>
+        </is>
+      </c>
+      <c r="J379" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K379" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L379" s="19" t="inlineStr">
+        <is>
+          <t>Zabezpiecz krzesło i niski zaczep gumy; Stań bokiem, guma przy kostce bliższej zaczepowi; Przyciągnij tę nogę ku środkowi ciała; Powoli odprowadź bez obrotu tułowia; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M379" s="19" t="inlineStr">
+        <is>
+          <t>Szarpanie nogą; Obracanie miednicy</t>
+        </is>
+      </c>
+      <c r="N379" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O379" s="19" t="inlineStr">
+        <is>
+          <t>Słabsza guma i mały zakres</t>
+        </is>
+      </c>
+      <c r="P379" s="19" t="inlineStr">
+        <is>
+          <t>https://library.theprehabguys.com/vimeo-video/standing-hip-adduction-band</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="19" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" s="19" t="inlineStr">
+        <is>
+          <t>Uginanie nóg na ślizgaczach</t>
+        </is>
+      </c>
+      <c r="C380" s="19" t="inlineStr">
+        <is>
+          <t>Sliding leg curl</t>
+        </is>
+      </c>
+      <c r="D380" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E380" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="F380" s="19" t="inlineStr">
+        <is>
+          <t>Ślizgacze</t>
+        </is>
+      </c>
+      <c r="G380" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H380" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I380" s="19" t="inlineStr">
+        <is>
+          <t>Sliding leg curl</t>
+        </is>
+      </c>
+      <c r="J380" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K380" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L380" s="19" t="inlineStr">
+        <is>
+          <t>Sprawdź zgodność ślizgaczy z podłogą i wolny tor ruchu; Połóż się na plecach, pięty na ślizgaczach; Unieś biodra; Powoli odsuń i przyciągnij pięty utrzymując kontrolę miednicy; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M380" s="19" t="inlineStr">
+        <is>
+          <t>Gwałtowny poślizg; Wyginanie pleców; Kontynuowanie mimo skurczu</t>
+        </is>
+      </c>
+      <c r="N380" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O380" s="19" t="inlineStr">
+        <is>
+          <t>Krótki ruch obunóż, bez pełnego wyprostu</t>
+        </is>
+      </c>
+      <c r="P380" s="19" t="inlineStr">
+        <is>
+          <t>https://www.muscleandfitness.com/exercise/workouts/leg-exercises/sliding-leg-curl</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="19" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" s="19" t="inlineStr">
+        <is>
+          <t>Pilates — setka z rytmiczną pracą ramion</t>
+        </is>
+      </c>
+      <c r="C381" s="19" t="inlineStr">
+        <is>
+          <t>Pilates Hundred</t>
+        </is>
+      </c>
+      <c r="D381" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E381" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder</t>
+        </is>
+      </c>
+      <c r="F381" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G381" s="19" t="inlineStr">
+        <is>
+          <t>Wytrzymałość</t>
+        </is>
+      </c>
+      <c r="H381" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I381" s="19" t="inlineStr">
+        <is>
+          <t>Pilates Hundred</t>
+        </is>
+      </c>
+      <c r="J381" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-15 sek</t>
+        </is>
+      </c>
+      <c r="K381" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L381" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na plecach z ugiętymi nogami; Unieś głowę i łopatki tylko przy swobodnej szyi; Wykonuj małe ruchy ramion przy bokach; Oddychaj rytmicznie i odpocznij przed utratą kontroli; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M381" s="19" t="inlineStr">
+        <is>
+          <t>Napinanie szyi; Zatrzymywanie oddechu; Wyginanie pleców</t>
+        </is>
+      </c>
+      <c r="N381" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O381" s="19" t="inlineStr">
+        <is>
+          <t>Głowa i stopy na podłodze, krótsza seria</t>
+        </is>
+      </c>
+      <c r="P381" s="19" t="inlineStr">
+        <is>
+          <t>https://pilatesology.com/pilatesology-encyclopedia-hundred/</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="19" t="n">
+        <v>381</v>
+      </c>
+      <c r="B382" s="19" t="inlineStr">
+        <is>
+          <t>Pilates — krążenia jedną nogą w leżeniu</t>
+        </is>
+      </c>
+      <c r="C382" s="19" t="inlineStr">
+        <is>
+          <t>Pilates single leg circles</t>
+        </is>
+      </c>
+      <c r="D382" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder</t>
+        </is>
+      </c>
+      <c r="E382" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Pośladki</t>
+        </is>
+      </c>
+      <c r="F382" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G382" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H382" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I382" s="19" t="inlineStr">
+        <is>
+          <t>Pilates single leg circles</t>
+        </is>
+      </c>
+      <c r="J382" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K382" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L382" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na plecach, ramiona przy bokach; Unieś jedną nogę; Zataczaj małe koła w obie strony bez ruchu miednicy; Opuść nogę i zmień stronę; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M382" s="19" t="inlineStr">
+        <is>
+          <t>Kołysanie biodrami; Forsowanie pachwiny</t>
+        </is>
+      </c>
+      <c r="N382" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O382" s="19" t="inlineStr">
+        <is>
+          <t>Ugnij kolano drugiej nogi i zmniejsz koła</t>
+        </is>
+      </c>
+      <c r="P382" s="19" t="inlineStr">
+        <is>
+          <t>https://onlinepilatesclasses.com/pilates-exercises/mat-exercises/mat-single-leg-circles</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="19" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" s="19" t="inlineStr">
+        <is>
+          <t>Pilates — naprzemienne wydłużanie nóg</t>
+        </is>
+      </c>
+      <c r="C383" s="19" t="inlineStr">
+        <is>
+          <t>Pilates single leg stretch</t>
+        </is>
+      </c>
+      <c r="D383" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E383" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder</t>
+        </is>
+      </c>
+      <c r="F383" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G383" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H383" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I383" s="19" t="inlineStr">
+        <is>
+          <t>Pilates single leg stretch</t>
+        </is>
+      </c>
+      <c r="J383" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K383" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L383" s="19" t="inlineStr">
+        <is>
+          <t>Połóż się na plecach i unieś głowę z łopatkami; Przybliż jedno ugięte kolano, drugą nogę wydłuż wysoko po skosie; Spokojnie zmieniaj nogi; Utrzymuj tułów bez kołysania i odpoczywaj z głową na macie; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M383" s="19" t="inlineStr">
+        <is>
+          <t>Szarpanie kolanem; Ciągnięcie szyją; Noga zbyt nisko</t>
+        </is>
+      </c>
+      <c r="N383" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O383" s="19" t="inlineStr">
+        <is>
+          <t>Krótszy ruch, noga prostowana wyżej</t>
+        </is>
+      </c>
+      <c r="P383" s="19" t="inlineStr">
+        <is>
+          <t>https://onlinepilatesclasses.com/pilates-exercises/mat-exercises/mat-single-leg-stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="19" t="n">
+        <v>383</v>
+      </c>
+      <c r="B384" s="19" t="inlineStr">
+        <is>
+          <t>Pilates — wydłużanie obu nóg i ramion</t>
+        </is>
+      </c>
+      <c r="C384" s="19" t="inlineStr">
+        <is>
+          <t>Pilates double leg stretch</t>
+        </is>
+      </c>
+      <c r="D384" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E384" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder</t>
+        </is>
+      </c>
+      <c r="F384" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G384" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H384" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I384" s="19" t="inlineStr">
+        <is>
+          <t>Pilates double leg stretch</t>
+        </is>
+      </c>
+      <c r="J384" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K384" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L384" s="19" t="inlineStr">
+        <is>
+          <t>Z leżenia przybliż ugięte nogi do tułowia, głowa i łopatki lekko uniesione; Wydłuż nogi wysoko po skosie i ramiona za głowę; Zatocz ramionami łuk i ugnij nogi; Zachowaj kontrolę pleców bez zatrzymywania oddechu; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M384" s="19" t="inlineStr">
+        <is>
+          <t>Przeprost lędźwi; Napinanie szyi</t>
+        </is>
+      </c>
+      <c r="N384" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O384" s="19" t="inlineStr">
+        <is>
+          <t>Krótszy zasięg, nogi wyżej lub martwy robak cw179</t>
+        </is>
+      </c>
+      <c r="P384" s="19" t="inlineStr">
+        <is>
+          <t>https://onlinepilatesclasses.com/pilates-exercises/mat-exercises/mat-double-leg-stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="19" t="n">
+        <v>384</v>
+      </c>
+      <c r="B385" s="19" t="inlineStr">
+        <is>
+          <t>Pilates — piła w siadzie</t>
+        </is>
+      </c>
+      <c r="C385" s="19" t="inlineStr">
+        <is>
+          <t>Pilates Saw</t>
+        </is>
+      </c>
+      <c r="D385" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E385" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Tył uda</t>
+        </is>
+      </c>
+      <c r="F385" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G385" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H385" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I385" s="19" t="inlineStr">
+        <is>
+          <t>Pilates Saw</t>
+        </is>
+      </c>
+      <c r="J385" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K385" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L385" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź w niewielkim rozkroku, ramiona rozłożone; Obróć tułów i sięgnij do przeciwnej stopy; Wróć do pionu i zmień stronę; Nie przesuwaj bioder ani nie forsuj skłonu; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M385" s="19" t="inlineStr">
+        <is>
+          <t>Ruch bioder; Szarpanie skłonu; Nadmierny skręt szyi</t>
+        </is>
+      </c>
+      <c r="N385" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O385" s="19" t="inlineStr">
+        <is>
+          <t>Ugięte kolana, wyższy siad i mniejszy skręt; przy zaleconym zakazie zgięcia lub rotacji wymaga indywidualnego doboru</t>
+        </is>
+      </c>
+      <c r="P385" s="19" t="inlineStr">
+        <is>
+          <t>https://onlinepilatesclasses.com/pilates-exercises/mat-exercises/mat-saw</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="19" t="n">
+        <v>385</v>
+      </c>
+      <c r="B386" s="19" t="inlineStr">
+        <is>
+          <t>Wysuwanie i cofanie łopatek w klęku podpartym</t>
+        </is>
+      </c>
+      <c r="C386" s="19" t="inlineStr">
+        <is>
+          <t>Quadruped scapular protraction retraction</t>
+        </is>
+      </c>
+      <c r="D386" s="19" t="inlineStr">
+        <is>
+          <t>Mięsień zębaty przedni, Plecy</t>
+        </is>
+      </c>
+      <c r="E386" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F386" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G386" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H386" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I386" s="19" t="inlineStr">
+        <is>
+          <t>Quadruped scapular protraction retraction</t>
+        </is>
+      </c>
+      <c r="J386" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K386" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L386" s="19" t="inlineStr">
+        <is>
+          <t>Ustaw dłonie pod barkami, kolana pod biodrami; Utrzymuj proste łokcie; Pozwól klatce lekko opaść między ramionami; Odepchnij podłoże oddalając łopatki bez ruchu lędźwi; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M386" s="19" t="inlineStr">
+        <is>
+          <t>Zginanie łokci jak w pompce; Zapadanie lędźwi</t>
+        </is>
+      </c>
+      <c r="N386" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O386" s="19" t="inlineStr">
+        <is>
+          <t>Mały ruch lub wykonanie przy ścianie</t>
+        </is>
+      </c>
+      <c r="P386" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/joint-mobility</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="19" t="n">
+        <v>386</v>
+      </c>
+      <c r="B387" s="19" t="inlineStr">
+        <is>
+          <t>Krążenia obręczy barkowej w klęku podpartym</t>
+        </is>
+      </c>
+      <c r="C387" s="19" t="inlineStr">
+        <is>
+          <t>Quadruped shoulder circles</t>
+        </is>
+      </c>
+      <c r="D387" s="19" t="inlineStr">
+        <is>
+          <t>Mięsień zębaty przedni, Plecy</t>
+        </is>
+      </c>
+      <c r="E387" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F387" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G387" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H387" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I387" s="19" t="inlineStr">
+        <is>
+          <t>Quadruped shoulder circles</t>
+        </is>
+      </c>
+      <c r="J387" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K387" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L387" s="19" t="inlineStr">
+        <is>
+          <t>Przyjmij klęk podparty z prostymi ramionami; Połącz małe unoszenie, cofanie, opuszczanie i wysuwanie obręczy barkowej; Wykonaj płynne koło; Zmień kierunek bez kołysania całym tułowiem; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M387" s="19" t="inlineStr">
+        <is>
+          <t>Duży ruch tułowia; Praca mimo bólu nadgarstków</t>
+        </is>
+      </c>
+      <c r="N387" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O387" s="19" t="inlineStr">
+        <is>
+          <t>Osobne wysuwanie i cofanie łopatek cw385</t>
+        </is>
+      </c>
+      <c r="P387" s="19" t="inlineStr">
+        <is>
+          <t>https://gmb.io/joint-mobility</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="19" t="n">
+        <v>387</v>
+      </c>
+      <c r="B388" s="19" t="inlineStr">
+        <is>
+          <t>Cofanie bioder w klęku z nogą wyprostowaną w bok</t>
+        </is>
+      </c>
+      <c r="C388" s="19" t="inlineStr">
+        <is>
+          <t>Straight leg adductor rock back</t>
+        </is>
+      </c>
+      <c r="D388" s="19" t="inlineStr">
+        <is>
+          <t>Przywodziciele uda</t>
+        </is>
+      </c>
+      <c r="E388" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda</t>
+        </is>
+      </c>
+      <c r="F388" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G388" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H388" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I388" s="19" t="inlineStr">
+        <is>
+          <t>Straight leg adductor rock back</t>
+        </is>
+      </c>
+      <c r="J388" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K388" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L388" s="19" t="inlineStr">
+        <is>
+          <t>Przyjmij klęk podparty; Wyprostuj jedną nogę w bok; Cofnij biodra ku pięcie nogi podporowej bez zaokrąglania pleców; Wróć i zmień stronę bez dociskania pachwiny; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M388" s="19" t="inlineStr">
+        <is>
+          <t>Zaokrąglanie pleców; Forsowanie zakresu</t>
+        </is>
+      </c>
+      <c r="N388" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O388" s="19" t="inlineStr">
+        <is>
+          <t>Mniejszy rozkrok i krótszy ruch</t>
+        </is>
+      </c>
+      <c r="P388" s="19" t="inlineStr">
+        <is>
+          <t>https://theprehabguys.com/vimeo-video/quadruped-dynamic-long-adductor-stretch/</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="19" t="n">
+        <v>388</v>
+      </c>
+      <c r="B389" s="19" t="inlineStr">
+        <is>
+          <t>Stanie tandemowe przy podporze</t>
+        </is>
+      </c>
+      <c r="C389" s="19" t="inlineStr">
+        <is>
+          <t>Supported tandem stand</t>
+        </is>
+      </c>
+      <c r="D389" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Pośladki</t>
+        </is>
+      </c>
+      <c r="E389" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Mięśnie stóp</t>
+        </is>
+      </c>
+      <c r="F389" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G389" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H389" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I389" s="19" t="inlineStr">
+        <is>
+          <t>Supported tandem stand</t>
+        </is>
+      </c>
+      <c r="J389" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-15 sek</t>
+        </is>
+      </c>
+      <c r="K389" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L389" s="19" t="inlineStr">
+        <is>
+          <t>Zabezpiecz krzesło przy ścianie i miej oparcie w zasięgu dłoni; Ustaw piętę jednej stopy przed palcami drugiej; Patrz przed siebie i oddychaj; Zamień ustawienie stóp po spokojnym wyjściu z pozycji; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M389" s="19" t="inlineStr">
+        <is>
+          <t>Zamykanie oczu; Brak zabezpieczenia przy chwiejności</t>
+        </is>
+      </c>
+      <c r="N389" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O389" s="19" t="inlineStr">
+        <is>
+          <t>Rozsuń stopy na boki i trzymaj podporę</t>
+        </is>
+      </c>
+      <c r="P389" s="19" t="inlineStr">
+        <is>
+          <t>https://roh.nhs.uk/services-information/therapy/otago-strength-and-balance-exercises</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="19" t="n">
+        <v>389</v>
+      </c>
+      <c r="B390" s="19" t="inlineStr">
+        <is>
+          <t>Chód pięta–palce przy podporze</t>
+        </is>
+      </c>
+      <c r="C390" s="19" t="inlineStr">
+        <is>
+          <t>Heel to toe walk</t>
+        </is>
+      </c>
+      <c r="D390" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Pośladki</t>
+        </is>
+      </c>
+      <c r="E390" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Mięśnie stóp</t>
+        </is>
+      </c>
+      <c r="F390" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G390" s="19" t="inlineStr">
+        <is>
+          <t>Rozgrzewka</t>
+        </is>
+      </c>
+      <c r="H390" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I390" s="19" t="inlineStr">
+        <is>
+          <t>Heel to toe walk</t>
+        </is>
+      </c>
+      <c r="J390" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K390" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L390" s="19" t="inlineStr">
+        <is>
+          <t>Wybierz wolny tor przy stabilnej ścianie; Idź powoli ustawiając piętę przed palcami drugiej stopy; Patrz przed siebie; Zatrzymaj się przed zawróceniem, w razie chwiejności przerwij; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M390" s="19" t="inlineStr">
+        <is>
+          <t>Pośpiech; Patrzenie wyłącznie pod nogi</t>
+        </is>
+      </c>
+      <c r="N390" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O390" s="19" t="inlineStr">
+        <is>
+          <t>Szerszy tor, dotykanie ściany dłonią</t>
+        </is>
+      </c>
+      <c r="P390" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/live-well/exercise/balance-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="19" t="n">
+        <v>390</v>
+      </c>
+      <c r="B391" s="19" t="inlineStr">
+        <is>
+          <t>Zgarnianie ręcznika palcami stopy</t>
+        </is>
+      </c>
+      <c r="C391" s="19" t="inlineStr">
+        <is>
+          <t>Toe towel curls</t>
+        </is>
+      </c>
+      <c r="D391" s="19" t="inlineStr">
+        <is>
+          <t>Mięśnie stóp</t>
+        </is>
+      </c>
+      <c r="E391" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F391" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło, Ręcznik</t>
+        </is>
+      </c>
+      <c r="G391" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H391" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I391" s="19" t="inlineStr">
+        <is>
+          <t>Toe towel curls</t>
+        </is>
+      </c>
+      <c r="J391" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K391" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L391" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź ze stopą na małym ręczniku; Zginając palce przyciągnij materiał pod stopę; Rozluźnij stopę; Powtórz bez przesuwania całej nogi, potem zmień stopę; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M391" s="19" t="inlineStr">
+        <is>
+          <t>Przesuwanie nogi; Mocniejsze zaciskanie przy skurczu</t>
+        </is>
+      </c>
+      <c r="N391" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O391" s="19" t="inlineStr">
+        <is>
+          <t>Cieńszy ręcznik i mniej materiału</t>
+        </is>
+      </c>
+      <c r="P391" s="19" t="inlineStr">
+        <is>
+          <t>https://orthoinfo.aaos.org/recovery/foot-and-ankle-conditioning-program/</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="19" t="n">
+        <v>391</v>
+      </c>
+      <c r="B392" s="19" t="inlineStr">
+        <is>
+          <t>Krótka stopa — aktywacja łuku w siadzie</t>
+        </is>
+      </c>
+      <c r="C392" s="19" t="inlineStr">
+        <is>
+          <t>Seated short foot exercise</t>
+        </is>
+      </c>
+      <c r="D392" s="19" t="inlineStr">
+        <is>
+          <t>Mięśnie stóp</t>
+        </is>
+      </c>
+      <c r="E392" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F392" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G392" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H392" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I392" s="19" t="inlineStr">
+        <is>
+          <t>Seated short foot exercise</t>
+        </is>
+      </c>
+      <c r="J392" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K392" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L392" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź ze stopą płasko; Oprzyj piętę i przodostopie; Delikatnie skróć stopę zbliżając podstawę palucha ku pięcie bez podwijania palców; Rozluźnij po małym napięciu i zmień stopę; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M392" s="19" t="inlineStr">
+        <is>
+          <t>Podwijanie palców; Rolowanie na zewnętrzną krawędź</t>
+        </is>
+      </c>
+      <c r="N392" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O392" s="19" t="inlineStr">
+        <is>
+          <t>Mniejsza siła i krótka pauza</t>
+        </is>
+      </c>
+      <c r="P392" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nhsinform.scot/illnesses-and-conditions/muscle-bone-and-joints/leg-and-foot-problems-and-conditions/exercises-for-foot-conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="19" t="n">
+        <v>392</v>
+      </c>
+      <c r="B393" s="19" t="inlineStr">
+        <is>
+          <t>Ruch stopy na zewnątrz przeciw gumie</t>
+        </is>
+      </c>
+      <c r="C393" s="19" t="inlineStr">
+        <is>
+          <t>Banded ankle eversion</t>
+        </is>
+      </c>
+      <c r="D393" s="19" t="inlineStr">
+        <is>
+          <t>Mięśnie strzałkowe</t>
+        </is>
+      </c>
+      <c r="E393" s="19" t="inlineStr">
+        <is>
+          <t>Mięśnie stóp</t>
+        </is>
+      </c>
+      <c r="F393" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło, Gumy oporowe</t>
+        </is>
+      </c>
+      <c r="G393" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H393" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I393" s="19" t="inlineStr">
+        <is>
+          <t>Banded ankle eversion</t>
+        </is>
+      </c>
+      <c r="J393" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K393" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L393" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź z podpartą nogą; Zabezpiecz gumę na przodostopiu tak, by opór przeciwdziałał ruchowi na zewnątrz; Utrzymując kolano nieruchomo odchyl przodostopie na zewnątrz; Powoli wróć bez wymuszania zakresu; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu</t>
+        </is>
+      </c>
+      <c r="M393" s="19" t="inlineStr">
+        <is>
+          <t>Obracanie całej nogi w biodrze; Guma zsuwająca się ze stopy</t>
+        </is>
+      </c>
+      <c r="N393" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O393" s="19" t="inlineStr">
+        <is>
+          <t>Mały ruch bez gumy</t>
+        </is>
+      </c>
+      <c r="P393" s="19" t="inlineStr">
+        <is>
+          <t>https://www.leicspart.nhs.uk/wp-content/uploads/2022/07/474-ankle-exercises.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="19" t="n">
+        <v>393</v>
+      </c>
+      <c r="B394" s="19" t="inlineStr">
+        <is>
+          <t>Deska z dotknięciem dłoni — w parach</t>
+        </is>
+      </c>
+      <c r="C394" s="19" t="inlineStr">
+        <is>
+          <t>Partner plank hand tap</t>
+        </is>
+      </c>
+      <c r="D394" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Mięsień zębaty przedni</t>
+        </is>
+      </c>
+      <c r="E394" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Pośladki</t>
+        </is>
+      </c>
+      <c r="F394" s="19" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="G394" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H394" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I394" s="19" t="inlineStr">
+        <is>
+          <t>Partner plank hand tap</t>
+        </is>
+      </c>
+      <c r="J394" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-15 sek</t>
+        </is>
+      </c>
+      <c r="K394" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L394" s="19" t="inlineStr">
+        <is>
+          <t>A: ustaw podpór naprzeciw partnera, dłonie pod barkami; B: ustaw taki sam podpór w odległości lekkiego kontaktu dłoni; Oboje naprzemiennie dotknijcie dłoni partnera i odłóżcie ją; Utrzymujcie nieruchome biodra, kontakt bez uderzania; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M394" s="19" t="inlineStr">
+        <is>
+          <t>Obracanie bioder; Sięganie za daleko; Próby przewracania partnera</t>
+        </is>
+      </c>
+      <c r="N394" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O394" s="19" t="inlineStr">
+        <is>
+          <t>Podpór na kolanach; warianty po opanowaniu: pompka przed kontaktem lub gąsienica do podporu</t>
+        </is>
+      </c>
+      <c r="P394" s="19" t="inlineStr">
+        <is>
+          <t>https://www.healthline.com/health/fitness-exercise/partner-workouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="19" t="n">
+        <v>394</v>
+      </c>
+      <c r="B395" s="19" t="inlineStr">
+        <is>
+          <t>Przysiad plecami do siebie — w parach</t>
+        </is>
+      </c>
+      <c r="C395" s="19" t="inlineStr">
+        <is>
+          <t>Back to back partner squat</t>
+        </is>
+      </c>
+      <c r="D395" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E395" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="F395" s="19" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="G395" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H395" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I395" s="19" t="inlineStr">
+        <is>
+          <t>Back to back partner squat</t>
+        </is>
+      </c>
+      <c r="J395" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K395" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L395" s="19" t="inlineStr">
+        <is>
+          <t>A: oprzyj plecy o partnera i ustal równy nacisk; B: przyjmij stabilne ustawienie stóp i potwierdź gotowość; Oboje na sygnał wykonajcie płytki przysiad; Wróćcie razem do stania, nie odchodźcie nagle; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M395" s="19" t="inlineStr">
+        <is>
+          <t>Nierówne tempo; Zbyt duża różnica masy lub wzrostu; Nagłe odejście</t>
+        </is>
+      </c>
+      <c r="N395" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O395" s="19" t="inlineStr">
+        <is>
+          <t>Mały zakres; wariant: krótkie utrzymanie półprzysiadu; przy niedopasowaniu wykonujcie niezależne przysiady naprzeciw siebie</t>
+        </is>
+      </c>
+      <c r="P395" s="19" t="inlineStr">
+        <is>
+          <t>https://www.mobilesport.ch/aktuell/kraeftigen-oberschenkel-vorne-ruecken-an-ruecken/</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="19" t="n">
+        <v>395</v>
+      </c>
+      <c r="B396" s="19" t="inlineStr">
+        <is>
+          <t>Lustro ruchowe — w parach</t>
+        </is>
+      </c>
+      <c r="C396" s="19" t="inlineStr">
+        <is>
+          <t>Partner movement mirror</t>
+        </is>
+      </c>
+      <c r="D396" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E396" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F396" s="19" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="G396" s="19" t="inlineStr">
+        <is>
+          <t>Rozgrzewka</t>
+        </is>
+      </c>
+      <c r="H396" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I396" s="19" t="inlineStr">
+        <is>
+          <t>Partner movement mirror</t>
+        </is>
+      </c>
+      <c r="J396" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-15 sek</t>
+        </is>
+      </c>
+      <c r="K396" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L396" s="19" t="inlineStr">
+        <is>
+          <t>A: prowadź powolne kroki i płytkie przysiady bez pozycji walki; B: odwzorowuj ruch z zachowaniem odstępu; Pozostańcie w wyznaczonej wolnej strefie; Zmieńcie prowadzącego na ustalony sygnał; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M396" s="19" t="inlineStr">
+        <is>
+          <t>Nagłe trudne ruchy; Cofanie poza wolną strefę</t>
+        </is>
+      </c>
+      <c r="N396" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O396" s="19" t="inlineStr">
+        <is>
+          <t>Tylko kroki boczne w marszu</t>
+        </is>
+      </c>
+      <c r="P396" s="19" t="inlineStr">
+        <is>
+          <t>https://www.westernracquet.com/blog/fun-partner-workouts-to-try</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="19" t="n">
+        <v>396</v>
+      </c>
+      <c r="B397" s="19" t="inlineStr">
+        <is>
+          <t>Przemieszczanie na gest — w parach</t>
+        </is>
+      </c>
+      <c r="C397" s="19" t="inlineStr">
+        <is>
+          <t>Partner wave direction drill</t>
+        </is>
+      </c>
+      <c r="D397" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E397" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F397" s="19" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="G397" s="19" t="inlineStr">
+        <is>
+          <t>Rozgrzewka</t>
+        </is>
+      </c>
+      <c r="H397" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I397" s="19" t="inlineStr">
+        <is>
+          <t>Partner wave direction drill</t>
+        </is>
+      </c>
+      <c r="J397" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-15 sek</t>
+        </is>
+      </c>
+      <c r="K397" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L397" s="19" t="inlineStr">
+        <is>
+          <t>A: pokazuj wcześniej uzgodnione kierunki; B: odpowiadaj krótkimi krokami i wracaj do środka; Wyznaczcie strefę hamowania bez przeszkód; Zmieniajcie role, na początku bez szybkiego biegu tyłem; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M397" s="19" t="inlineStr">
+        <is>
+          <t>Sygnały zbyt szybkie; Brak miejsca na hamowanie</t>
+        </is>
+      </c>
+      <c r="N397" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O397" s="19" t="inlineStr">
+        <is>
+          <t>Tylko lewo i prawo w marszu</t>
+        </is>
+      </c>
+      <c r="P397" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nsca.com/education/articles/kinetic-select/5-reaction-drills-to-build-quickness/</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="19" t="n">
+        <v>397</v>
+      </c>
+      <c r="B398" s="19" t="inlineStr">
+        <is>
+          <t>Chwyt piłki przed drugim odbiciem — w parach</t>
+        </is>
+      </c>
+      <c r="C398" s="19" t="inlineStr">
+        <is>
+          <t>Partner ball drop catch</t>
+        </is>
+      </c>
+      <c r="D398" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E398" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F398" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka</t>
+        </is>
+      </c>
+      <c r="G398" s="19" t="inlineStr">
+        <is>
+          <t>Rozgrzewka</t>
+        </is>
+      </c>
+      <c r="H398" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I398" s="19" t="inlineStr">
+        <is>
+          <t>Partner ball drop catch</t>
+        </is>
+      </c>
+      <c r="J398" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K398" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L398" s="19" t="inlineStr">
+        <is>
+          <t>A: upuszczaj małą odbijającą piłkę w wolnej strefie; B: reaguj i łap przed drugim odbiciem; Ustalcie dystans bez ryzyka zderzenia; Nie rzucaj się na podłogę, nieudaną próbę odpuść; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M398" s="19" t="inlineStr">
+        <is>
+          <t>Wbieganie na partnera; Nurkowanie za piłką</t>
+        </is>
+      </c>
+      <c r="N398" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O398" s="19" t="inlineStr">
+        <is>
+          <t>Mniejsza odległość i zapowiedź upuszczenia</t>
+        </is>
+      </c>
+      <c r="P398" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nsca.com/education/articles/kinetic-select/5-reaction-drills-to-build-quickness/</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="19" t="n">
+        <v>398</v>
+      </c>
+      <c r="B399" s="19" t="inlineStr">
+        <is>
+          <t>Krok boczny z chwytem piłki — w parach</t>
+        </is>
+      </c>
+      <c r="C399" s="19" t="inlineStr">
+        <is>
+          <t>Partner shuffle reaction catch</t>
+        </is>
+      </c>
+      <c r="D399" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E399" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F399" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka</t>
+        </is>
+      </c>
+      <c r="G399" s="19" t="inlineStr">
+        <is>
+          <t>Rozgrzewka</t>
+        </is>
+      </c>
+      <c r="H399" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I399" s="19" t="inlineStr">
+        <is>
+          <t>Partner shuffle reaction catch</t>
+        </is>
+      </c>
+      <c r="J399" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K399" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L399" s="19" t="inlineStr">
+        <is>
+          <t>A: łagodnie podaj miękką piłkę na lewo lub prawo B; B: przesuń się krokiem dostawnym, złap i odeślij; Utrzymujcie bezpieczny dystans i wolny tor; Po serii zamieńcie role; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M399" s="19" t="inlineStr">
+        <is>
+          <t>Podania poza zasięg; Krzyżowanie nóg w pośpiechu</t>
+        </is>
+      </c>
+      <c r="N399" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O399" s="19" t="inlineStr">
+        <is>
+          <t>Zapowiedziana strona i krótki dystans</t>
+        </is>
+      </c>
+      <c r="P399" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nsca.com/education/articles/kinetic-select/5-reaction-drills-to-build-quickness/</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="19" t="n">
+        <v>399</v>
+      </c>
+      <c r="B400" s="19" t="inlineStr">
+        <is>
+          <t>Podania na jednej nodze — w parach</t>
+        </is>
+      </c>
+      <c r="C400" s="19" t="inlineStr">
+        <is>
+          <t>Partner single leg ball toss</t>
+        </is>
+      </c>
+      <c r="D400" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Łydki</t>
+        </is>
+      </c>
+      <c r="E400" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Przedramiona, Mięśnie stóp</t>
+        </is>
+      </c>
+      <c r="F400" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka</t>
+        </is>
+      </c>
+      <c r="G400" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H400" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I400" s="19" t="inlineStr">
+        <is>
+          <t>Partner single leg ball toss</t>
+        </is>
+      </c>
+      <c r="J400" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-15 sek</t>
+        </is>
+      </c>
+      <c r="K400" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L400" s="19" t="inlineStr">
+        <is>
+          <t>A: stań stabilnie na jednej nodze z lekką miękką piłką; B: przyjmij takie samo ustawienie i pokaż gotowe dłonie; Wymieniajcie łagodne podania w zasięg dłoni; Zmieńcie nogi, odstaw stopę przed utratą równowagi; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M400" s="19" t="inlineStr">
+        <is>
+          <t>Ciężka piłka; Ratowanie równowagi za wszelką cenę</t>
+        </is>
+      </c>
+      <c r="N400" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O400" s="19" t="inlineStr">
+        <is>
+          <t>Palce drugiej stopy na podłodze</t>
+        </is>
+      </c>
+      <c r="P400" s="19" t="inlineStr">
+        <is>
+          <t>https://www.silversneakers.com/blog/partner-workout-total-body-strength-exercises-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="19" t="n">
+        <v>400</v>
+      </c>
+      <c r="B401" s="19" t="inlineStr">
+        <is>
+          <t>Podania sprzed klatki — w parach</t>
+        </is>
+      </c>
+      <c r="C401" s="19" t="inlineStr">
+        <is>
+          <t>Partner chest pass</t>
+        </is>
+      </c>
+      <c r="D401" s="19" t="inlineStr">
+        <is>
+          <t>Klatka piersiowa, Triceps</t>
+        </is>
+      </c>
+      <c r="E401" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Brzuch, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F401" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka</t>
+        </is>
+      </c>
+      <c r="G401" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H401" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I401" s="19" t="inlineStr">
+        <is>
+          <t>Partner chest pass</t>
+        </is>
+      </c>
+      <c r="J401" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K401" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L401" s="19" t="inlineStr">
+        <is>
+          <t>A: trzymaj miękką lekką piłkę przy klatce; B: pokaż gotowe dłonie; A podaje oburącz, B amortyzuje chwyt uginając ramiona i odsyła; Nie rzucajcie w twarz, zaczynajcie od łagodnych podań; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M401" s="19" t="inlineStr">
+        <is>
+          <t>Podanie bez gotowości odbierającego; Sztywne łokcie przy chwycie</t>
+        </is>
+      </c>
+      <c r="N401" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O401" s="19" t="inlineStr">
+        <is>
+          <t>Lżejsza piłka i krótszy dystans</t>
+        </is>
+      </c>
+      <c r="P401" s="19" t="inlineStr">
+        <is>
+          <t>https://www.healthline.com/health/fitness-exercise/partner-workouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="19" t="n">
+        <v>401</v>
+      </c>
+      <c r="B402" s="19" t="inlineStr">
+        <is>
+          <t>Wykrok z podaniem piłki — w parach</t>
+        </is>
+      </c>
+      <c r="C402" s="19" t="inlineStr">
+        <is>
+          <t>Partner lunge chest pass</t>
+        </is>
+      </c>
+      <c r="D402" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E402" s="19" t="inlineStr">
+        <is>
+          <t>Klatka piersiowa, Triceps, Brzuch</t>
+        </is>
+      </c>
+      <c r="F402" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka</t>
+        </is>
+      </c>
+      <c r="G402" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H402" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I402" s="19" t="inlineStr">
+        <is>
+          <t>Partner lunge chest pass</t>
+        </is>
+      </c>
+      <c r="J402" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K402" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L402" s="19" t="inlineStr">
+        <is>
+          <t>A: wykonaj kontrolowany wykrok i podaj lekką piłkę; B: odbierz stojąc stabilnie; Poczekajcie aż A wróci do pozycji; Teraz B wykonuje wykrok i podaje, zachowajcie odstęp bez wchodzenia na siebie; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M402" s="19" t="inlineStr">
+        <is>
+          <t>Jednoczesne wchodzenie na siebie; Podanie przed stabilizacją</t>
+        </is>
+      </c>
+      <c r="N402" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O402" s="19" t="inlineStr">
+        <is>
+          <t>Sam krok lub płytki wykrok</t>
+        </is>
+      </c>
+      <c r="P402" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/everyone/exercise-library/264/medicine-ball-lunge-to-chest-pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="19" t="n">
+        <v>402</v>
+      </c>
+      <c r="B403" s="19" t="inlineStr">
+        <is>
+          <t>Krok dostawny z podaniami — w parach</t>
+        </is>
+      </c>
+      <c r="C403" s="19" t="inlineStr">
+        <is>
+          <t>Partner side shuffle ball toss</t>
+        </is>
+      </c>
+      <c r="D403" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E403" s="19" t="inlineStr">
+        <is>
+          <t>Łydki, Klatka piersiowa, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F403" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka</t>
+        </is>
+      </c>
+      <c r="G403" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H403" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I403" s="19" t="inlineStr">
+        <is>
+          <t>Partner side shuffle ball toss</t>
+        </is>
+      </c>
+      <c r="J403" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-15 sek</t>
+        </is>
+      </c>
+      <c r="K403" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L403" s="19" t="inlineStr">
+        <is>
+          <t>A: rozpocznij spokojny krok dostawny z lekką piłką; B: przemieszczaj się równolegle naprzeciw; Wymieniajcie łagodne podania przed klatkę; Zwolnijcie przed wspólną zmianą kierunku; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M403" s="19" t="inlineStr">
+        <is>
+          <t>Rzuty za plecy; Rozbieganie partnerów; Nagłe zmiany kierunku</t>
+        </is>
+      </c>
+      <c r="N403" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O403" s="19" t="inlineStr">
+        <is>
+          <t>Zatrzymujcie się na każde podanie</t>
+        </is>
+      </c>
+      <c r="P403" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/pros/expert-articles/6194/6-calorie-blasting-partner-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="19" t="n">
+        <v>403</v>
+      </c>
+      <c r="B404" s="19" t="inlineStr">
+        <is>
+          <t>Przysiad z przekazaniem piłki — w parach</t>
+        </is>
+      </c>
+      <c r="C404" s="19" t="inlineStr">
+        <is>
+          <t>Partner squat ball handoff</t>
+        </is>
+      </c>
+      <c r="D404" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E404" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Barki</t>
+        </is>
+      </c>
+      <c r="F404" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka</t>
+        </is>
+      </c>
+      <c r="G404" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H404" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I404" s="19" t="inlineStr">
+        <is>
+          <t>Partner squat ball handoff</t>
+        </is>
+      </c>
+      <c r="J404" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K404" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L404" s="19" t="inlineStr">
+        <is>
+          <t>A: trzymaj lekką piłkę przy klatce; B: stań naprzeciw w zasięgu przekazania; Oboje wykonajcie przysiad i wróćcie do stania; A przekazuje piłkę do dłoni B bez rzutu i puszcza po potwierdzeniu chwytu; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M404" s="19" t="inlineStr">
+        <is>
+          <t>Puszczanie zbyt wcześnie; Piłka daleko od tułowia</t>
+        </is>
+      </c>
+      <c r="N404" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O404" s="19" t="inlineStr">
+        <is>
+          <t>Płytki przysiad lub wstawanie ze stabilnych krzeseł</t>
+        </is>
+      </c>
+      <c r="P404" s="19" t="inlineStr">
+        <is>
+          <t>https://www.silversneakers.com/blog/partner-workout-total-body-strength-exercises-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="19" t="n">
+        <v>404</v>
+      </c>
+      <c r="B405" s="19" t="inlineStr">
+        <is>
+          <t>Przekazywanie piłki w siadzie plecami do siebie — w parach</t>
+        </is>
+      </c>
+      <c r="C405" s="19" t="inlineStr">
+        <is>
+          <t>Seated back to back partner ball pass</t>
+        </is>
+      </c>
+      <c r="D405" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E405" s="19" t="inlineStr">
+        <is>
+          <t>Plecy, Barki</t>
+        </is>
+      </c>
+      <c r="F405" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka</t>
+        </is>
+      </c>
+      <c r="G405" s="19" t="inlineStr">
+        <is>
+          <t>Mobilność</t>
+        </is>
+      </c>
+      <c r="H405" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I405" s="19" t="inlineStr">
+        <is>
+          <t>Seated back to back partner ball pass</t>
+        </is>
+      </c>
+      <c r="J405" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K405" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L405" s="19" t="inlineStr">
+        <is>
+          <t>A: usiądź stabilnie z ugiętymi kolanami i piłką; B: usiądź plecami do A; Obróćcie tułowia i przekażcie piłkę z rąk do rąk, potem na drugą stronę; Zmieńcie kierunek, nie szarpcie, przy ograniczeniu skrętów wybierzcie zwykłe podania; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M405" s="19" t="inlineStr">
+        <is>
+          <t>Forsowanie skrętu; Szarpanie piłki; Przesuwanie bioder</t>
+        </is>
+      </c>
+      <c r="N405" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O405" s="19" t="inlineStr">
+        <is>
+          <t>Lekka piłka i mały skręt; wariant stojący w półprzysiadzie tylko bez dyskomfortu</t>
+        </is>
+      </c>
+      <c r="P405" s="19" t="inlineStr">
+        <is>
+          <t>https://www.goldsgym.com/blog/partner-workout</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="19" t="n">
+        <v>405</v>
+      </c>
+      <c r="B406" s="19" t="inlineStr">
+        <is>
+          <t>Wiosłowanie gumą z oporem partnera — w parach</t>
+        </is>
+      </c>
+      <c r="C406" s="19" t="inlineStr">
+        <is>
+          <t>Partner anchored band row</t>
+        </is>
+      </c>
+      <c r="D406" s="19" t="inlineStr">
+        <is>
+          <t>Plecy</t>
+        </is>
+      </c>
+      <c r="E406" s="19" t="inlineStr">
+        <is>
+          <t>Biceps, Przedramiona, Brzuch</t>
+        </is>
+      </c>
+      <c r="F406" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Gumy oporowe</t>
+        </is>
+      </c>
+      <c r="G406" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H406" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I406" s="19" t="inlineStr">
+        <is>
+          <t>Partner anchored band row</t>
+        </is>
+      </c>
+      <c r="J406" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K406" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L406" s="19" t="inlineStr">
+        <is>
+          <t>A: stań stabilnie i trzymaj pewnie środek gumy przed sobą; B: chwyć uchwyty, przyjmij stabilny wykrok i przyciągnij łokcie ku tyłowi; B powoli prostuje ramiona, A utrzymuje stały opór; Zmieniajcie role dopiero po rozluźnieniu gumy; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M406" s="19" t="inlineStr">
+        <is>
+          <t>Odchylanie tułowia; Szarpanie; Nagłe puszczanie gumy</t>
+        </is>
+      </c>
+      <c r="N406" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O406" s="19" t="inlineStr">
+        <is>
+          <t>Słabsza guma; przy niepewnym chwycie użyj właściwego nieruchomego zaczepu</t>
+        </is>
+      </c>
+      <c r="P406" s="19" t="inlineStr">
+        <is>
+          <t>https://www.healthline.com/health/fitness-exercise/partner-workouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="19" t="n">
+        <v>406</v>
+      </c>
+      <c r="B407" s="19" t="inlineStr">
+        <is>
+          <t>Wyciskanie gumy z partnerem za plecami — w parach</t>
+        </is>
+      </c>
+      <c r="C407" s="19" t="inlineStr">
+        <is>
+          <t>Partner anchored band chest press</t>
+        </is>
+      </c>
+      <c r="D407" s="19" t="inlineStr">
+        <is>
+          <t>Klatka piersiowa, Triceps</t>
+        </is>
+      </c>
+      <c r="E407" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F407" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Gumy oporowe</t>
+        </is>
+      </c>
+      <c r="G407" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H407" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I407" s="19" t="inlineStr">
+        <is>
+          <t>Partner anchored band chest press</t>
+        </is>
+      </c>
+      <c r="J407" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6</t>
+        </is>
+      </c>
+      <c r="K407" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L407" s="19" t="inlineStr">
+        <is>
+          <t>A: stabilizuj gumę za plecami B, poza linią twarzy; B: trzymaj uchwyty z gumą poniżej pach i przyjmij wykrok; B wypycha uchwyty przed klatkę i powoli cofa; A nie zmienia nagle oporu, zmiana ról po rozluźnieniu; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M407" s="19" t="inlineStr">
+        <is>
+          <t>Guma przy szyi; Wyginanie pleców; Utrata chwytu</t>
+        </is>
+      </c>
+      <c r="N407" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O407" s="19" t="inlineStr">
+        <is>
+          <t>Słabsza guma lub nieruchomy zaczep zamiast partnera</t>
+        </is>
+      </c>
+      <c r="P407" s="19" t="inlineStr">
+        <is>
+          <t>https://www.healthline.com/health/fitness-exercise/partner-workouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="19" t="n">
+        <v>407</v>
+      </c>
+      <c r="B408" s="19" t="inlineStr">
+        <is>
+          <t>Ruch po przekątnej z gumą — w parach</t>
+        </is>
+      </c>
+      <c r="C408" s="19" t="inlineStr">
+        <is>
+          <t>Partner band woodchop</t>
+        </is>
+      </c>
+      <c r="D408" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E408" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Pośladki</t>
+        </is>
+      </c>
+      <c r="F408" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Gumy oporowe</t>
+        </is>
+      </c>
+      <c r="G408" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H408" s="19" t="inlineStr">
+        <is>
+          <t>Średni</t>
+        </is>
+      </c>
+      <c r="I408" s="19" t="inlineStr">
+        <is>
+          <t>Partner band woodchop</t>
+        </is>
+      </c>
+      <c r="J408" s="19" t="inlineStr">
+        <is>
+          <t>1 x 4-6 na stronę</t>
+        </is>
+      </c>
+      <c r="K408" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L408" s="19" t="inlineStr">
+        <is>
+          <t>A: stabilizuj gumę z boku B poniżej barków; B: chwyć drugi koniec i prowadź ramiona po krótkiej przekątnej z kontrolowanym obrotem; Wróć spokojnie bez skręcania kolan; Zmieńcie stronę i role po rozluźnieniu, nie kierujcie gumy na twarz; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M408" s="19" t="inlineStr">
+        <is>
+          <t>Szarpanie; Skręt kolan przy nieruchomych stopach; Kierowanie gumy w twarz</t>
+        </is>
+      </c>
+      <c r="N408" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O408" s="19" t="inlineStr">
+        <is>
+          <t>Słaba guma, mała przekątna poniżej barków</t>
+        </is>
+      </c>
+      <c r="P408" s="19" t="inlineStr">
+        <is>
+          <t>https://www.healthline.com/health/fitness-exercise/partner-workouts</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="19" t="n">
+        <v>408</v>
+      </c>
+      <c r="B409" s="19" t="inlineStr">
+        <is>
+          <t>Chód w półprzysiadzie ze wspólną piłką — w parach</t>
+        </is>
+      </c>
+      <c r="C409" s="19" t="inlineStr">
+        <is>
+          <t>Partner stability ball squat walk</t>
+        </is>
+      </c>
+      <c r="D409" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E409" s="19" t="inlineStr">
+        <is>
+          <t>Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F409" s="19" t="inlineStr">
+        <is>
+          <t>Partner, Piłka gimnastyczna</t>
+        </is>
+      </c>
+      <c r="G409" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H409" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I409" s="19" t="inlineStr">
+        <is>
+          <t>Partner stability ball squat walk</t>
+        </is>
+      </c>
+      <c r="J409" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-15 sek</t>
+        </is>
+      </c>
+      <c r="K409" s="19" t="inlineStr">
+        <is>
+          <t>Spokojnie i kontrolowanie, odpocznij po próbie</t>
+        </is>
+      </c>
+      <c r="L409" s="19" t="inlineStr">
+        <is>
+          <t>A: oprzyj jedną dłoń o dużą piłkę gimnastyczną na wysokości barku; B: stań naprzeciw i oprzyj dłoń z drugiej strony; Przy lekkim wspólnym nacisku przejdźcie do płytkiego półprzysiadu i kroków bocznych; Zmieńcie ręce i kierunek, nie opierajcie ciężaru ciała na piłce; Przerwij przy bólu, drętwieniu, zawrotach głowy lub nietypowej duszności; nie wstrzymuj oddechu; Ustalcie komendę STOP; kończcie zadanie razem bez nagłego puszczania oporu; Dobierzcie trudność do słabszego partnera; po serii zamieńcie role A i B</t>
+        </is>
+      </c>
+      <c r="M409" s="19" t="inlineStr">
+        <is>
+          <t>Siłowe przepychanie piłki; Oparcie całego ciężaru; Nierówne tempo</t>
+        </is>
+      </c>
+      <c r="N409" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę ruchu; dopiero potem dodaj 1-2 powtórzenia bez bólu</t>
+        </is>
+      </c>
+      <c r="O409" s="19" t="inlineStr">
+        <is>
+          <t>Wyższa pozycja i pozostanie w miejscu</t>
+        </is>
+      </c>
+      <c r="P409" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/pros/expert-articles/6194/6-calorie-blasting-partner-exercises/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add EZ bar and stationary bike catalog; release 1.20.0+36
</commit_message>
<xml_diff>
--- a/tools/source_data/baza_cwiczen_316.xlsx
+++ b/tools/source_data/baza_cwiczen_316.xlsx
@@ -8445,7 +8445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P409"/>
+  <dimension ref="A1:P413"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.8515625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.00390625" customWidth="1" style="39" min="1" max="1"/>
@@ -41180,6 +41180,326 @@
       <c r="P409" s="19" t="inlineStr">
         <is>
           <t>https://www.acefitness.org/resources/pros/expert-articles/6194/6-calorie-blasting-partner-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="19" t="n">
+        <v>409</v>
+      </c>
+      <c r="B410" s="19" t="inlineStr">
+        <is>
+          <t>Uginanie ramion z gryfem łamanym EZ stojąc</t>
+        </is>
+      </c>
+      <c r="C410" s="19" t="inlineStr">
+        <is>
+          <t>Standing EZ bar curl</t>
+        </is>
+      </c>
+      <c r="D410" s="19" t="inlineStr">
+        <is>
+          <t>Biceps</t>
+        </is>
+      </c>
+      <c r="E410" s="19" t="inlineStr">
+        <is>
+          <t>Mięsień ramienny, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F410" s="19" t="inlineStr">
+        <is>
+          <t>Gryf łamany EZ</t>
+        </is>
+      </c>
+      <c r="G410" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H410" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I410" s="19" t="inlineStr">
+        <is>
+          <t>Zginanie łokci</t>
+        </is>
+      </c>
+      <c r="J410" s="19" t="inlineStr">
+        <is>
+          <t>2 x 10-15</t>
+        </is>
+      </c>
+      <c r="K410" s="19" t="inlineStr">
+        <is>
+          <t>Unoszenie 1-2 s, opuszczanie 2-3 s bez szarpania</t>
+        </is>
+      </c>
+      <c r="L410" s="19" t="inlineStr">
+        <is>
+          <t>Stań stabilnie, stopy na szerokość bioder, kolana miękkie; Chwyć ukośne odcinki gryfu symetrycznie podchwytem, dłonie ku górze, nadgarstki w linii przedramion; Utrzymuj łokcie blisko boków i tułów nieruchomo; Ugnij łokcie unosząc gryf bez wysuwania ramion; Opuść powoli do wygodnego wyprostu bez blokowania łokci; Oddychaj swobodnie: wydech przy unoszeniu, wdech przy opuszczaniu; Przerwij przy bólu łokci, nadgarstków lub barków, drętwieniu albo zawrotach głowy; Zapisuj łączną masę gryfu i talerzy w kg, nie ciężar na rękę; Zabezpiecz talerze zaciskami, dobierz lekki ciężar do kontroli ruchu i zostaw około 3 powtórzeń w zapasie</t>
+        </is>
+      </c>
+      <c r="M410" s="19" t="inlineStr">
+        <is>
+          <t>Bujanie tułowiem i odchylanie pleców; Wysuwanie łokci; Załamywanie nadgarstków; Zrzucanie ciężaru</t>
+        </is>
+      </c>
+      <c r="N410" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw osiągnij 15 kontrolowanych powtórzeń bez bólu i z zapasem; potem dodaj najmniejszy dostępny ciężar i wróć do 10 powtórzeń</t>
+        </is>
+      </c>
+      <c r="O410" s="19" t="inlineStr">
+        <is>
+          <t>Lżejszy gryf lub mniej talerzy i krótszy bezbolesny zakres; jeśli sam gryf jest za ciężki, wybierz lżejszy wariant z innym sprzętem</t>
+        </is>
+      </c>
+      <c r="P410" s="19" t="inlineStr">
+        <is>
+          <t>https://www.muscleandstrength.com/exercises/ez-bar-curl.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="19" t="n">
+        <v>410</v>
+      </c>
+      <c r="B411" s="19" t="inlineStr">
+        <is>
+          <t>Uginanie ramion z gryfem łamanym EZ nachwytem stojąc</t>
+        </is>
+      </c>
+      <c r="C411" s="19" t="inlineStr">
+        <is>
+          <t>Standing reverse grip EZ bar curl</t>
+        </is>
+      </c>
+      <c r="D411" s="19" t="inlineStr">
+        <is>
+          <t>Przedramiona, Mięsień ramienny</t>
+        </is>
+      </c>
+      <c r="E411" s="19" t="inlineStr">
+        <is>
+          <t>Biceps</t>
+        </is>
+      </c>
+      <c r="F411" s="19" t="inlineStr">
+        <is>
+          <t>Gryf łamany EZ</t>
+        </is>
+      </c>
+      <c r="G411" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H411" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I411" s="19" t="inlineStr">
+        <is>
+          <t>Zginanie łokci</t>
+        </is>
+      </c>
+      <c r="J411" s="19" t="inlineStr">
+        <is>
+          <t>2 x 10-15</t>
+        </is>
+      </c>
+      <c r="K411" s="19" t="inlineStr">
+        <is>
+          <t>Unoszenie 1-2 s, opuszczanie 2-3 s bez szarpania</t>
+        </is>
+      </c>
+      <c r="L411" s="19" t="inlineStr">
+        <is>
+          <t>Stań stabilnie, stopy na szerokość bioder, tułów wyprostowany; Chwyć ukośne odcinki gryfu symetrycznie nachwytem, dłonie ku dołowi; Utrzymaj nadgarstki w linii przedramion i łokcie przy bokach; Ugnij łokcie bez wymachu i podnoszenia barków; Opuść gryf powoli, nie pozwalaj nadgarstkom opaść; Oddychaj swobodnie: wydech przy unoszeniu, wdech przy opuszczaniu; Przerwij przy bólu łokci, nadgarstków lub barków, drętwieniu albo zawrotach głowy; Zapisuj łączną masę gryfu i talerzy w kg, nie ciężar na rękę; Zabezpiecz talerze zaciskami, dobierz lekki ciężar do kontroli ruchu i zostaw około 3 powtórzeń w zapasie</t>
+        </is>
+      </c>
+      <c r="M411" s="19" t="inlineStr">
+        <is>
+          <t>Podchwyt zamiast nachwytu; Kołysanie tułowiem; Opadanie nadgarstków; Ciężar wymuszający skrócenie ruchu</t>
+        </is>
+      </c>
+      <c r="N411" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw osiągnij 15 kontrolowanych powtórzeń bez bólu i z zapasem; potem dodaj najmniejszy dostępny ciężar i wróć do 10 powtórzeń</t>
+        </is>
+      </c>
+      <c r="O411" s="19" t="inlineStr">
+        <is>
+          <t>Lżejszy gryf lub mniej talerzy i krótszy bezbolesny zakres; jeśli sam gryf jest za ciężki, wybierz lżejszy wariant z innym sprzętem</t>
+        </is>
+      </c>
+      <c r="P411" s="19" t="inlineStr">
+        <is>
+          <t>https://www.muscleandstrength.com/exercises/ez-bar-reverse-grip-barbell-curl.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="19" t="n">
+        <v>411</v>
+      </c>
+      <c r="B412" s="19" t="inlineStr">
+        <is>
+          <t>Prostowanie ramion z gryfem łamanym EZ w leżeniu na ławce płaskiej</t>
+        </is>
+      </c>
+      <c r="C412" s="19" t="inlineStr">
+        <is>
+          <t>Lying EZ bar triceps extension on flat bench</t>
+        </is>
+      </c>
+      <c r="D412" s="19" t="inlineStr">
+        <is>
+          <t>Triceps</t>
+        </is>
+      </c>
+      <c r="E412" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F412" s="19" t="inlineStr">
+        <is>
+          <t>Gryf łamany EZ, Ławeczka</t>
+        </is>
+      </c>
+      <c r="G412" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H412" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I412" s="19" t="inlineStr">
+        <is>
+          <t>Prostowanie łokci</t>
+        </is>
+      </c>
+      <c r="J412" s="19" t="inlineStr">
+        <is>
+          <t>2 x 10-15</t>
+        </is>
+      </c>
+      <c r="K412" s="19" t="inlineStr">
+        <is>
+          <t>Unoszenie 1-2 s, opuszczanie 2-3 s bez szarpania</t>
+        </is>
+      </c>
+      <c r="L412" s="19" t="inlineStr">
+        <is>
+          <t>Zablokuj stabilną ławkę w ustawieniu płaskim i oprzyj stopy na podłodze; Chwyć wewnętrzne ukośne odcinki gryfu symetrycznie nachwytem z kciukiem wokół gryfu; Połóż się z podpartą głową, plecami i pośladkami, ustaw gryf nad górą klatki; Utrzymuj ramiona niemal nieruchomo i łokcie skierowane w górę bez rozpychania; Zginając łokcie opuść gryf kontrolowanie za linię czoła, bez kontaktu z głową; Wyprostuj łokcie bez gwałtownego blokowania, nie zmieniaj ruchu w wyciskanie; Użyj ciężaru, który samodzielnie bezpiecznie ustawisz i odłożysz, w razie trudności poproś o pomoc przy podaniu i odebraniu; Oddychaj swobodnie: wydech przy unoszeniu, wdech przy opuszczaniu; Przerwij przy bólu łokci, nadgarstków lub barków, drętwieniu albo zawrotach głowy; Zapisuj łączną masę gryfu i talerzy w kg, nie ciężar na rękę; Zabezpiecz talerze zaciskami, dobierz lekki ciężar do kontroli ruchu i zostaw około 3 powtórzeń w zapasie</t>
+        </is>
+      </c>
+      <c r="M412" s="19" t="inlineStr">
+        <is>
+          <t>Opuszczanie gryfu na twarz; Rozchodzenie łokci; Ruch barkami zamiast łokci; Wyginanie pleców; Zbyt ciężki gryf bez bezpiecznego odłożenia</t>
+        </is>
+      </c>
+      <c r="N412" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw osiągnij 15 kontrolowanych powtórzeń bez bólu i z zapasem; potem dodaj najmniejszy dostępny ciężar i wróć do 10 powtórzeń</t>
+        </is>
+      </c>
+      <c r="O412" s="19" t="inlineStr">
+        <is>
+          <t>Lżejszy gryf lub mniej talerzy i krótszy bezbolesny zakres; jeśli sam gryf jest za ciężki, wybierz lżejszy wariant z innym sprzętem</t>
+        </is>
+      </c>
+      <c r="P412" s="19" t="inlineStr">
+        <is>
+          <t>https://www.endomondo.com/exercise/ez-bar-lying-triceps-extension</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="19" t="n">
+        <v>412</v>
+      </c>
+      <c r="B413" s="19" t="inlineStr">
+        <is>
+          <t>Spokojna jazda na rowerze stacjonarnym</t>
+        </is>
+      </c>
+      <c r="C413" s="19" t="inlineStr">
+        <is>
+          <t>Easy stationary cycling</t>
+        </is>
+      </c>
+      <c r="D413" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E413" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Łydki</t>
+        </is>
+      </c>
+      <c r="F413" s="19" t="inlineStr">
+        <is>
+          <t>Rower stacjonarny</t>
+        </is>
+      </c>
+      <c r="G413" s="19" t="inlineStr">
+        <is>
+          <t>Cardio</t>
+        </is>
+      </c>
+      <c r="H413" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I413" s="19" t="inlineStr">
+        <is>
+          <t>Pedałowanie</t>
+        </is>
+      </c>
+      <c r="J413" s="19" t="inlineStr">
+        <is>
+          <t>1 x 10-20 min łącznie z łagodnym początkiem i zakończeniem</t>
+        </is>
+      </c>
+      <c r="K413" s="19" t="inlineStr">
+        <is>
+          <t>Płynnie, spokojne tempo rozmowy, bez sprintów</t>
+        </is>
+      </c>
+      <c r="L413" s="19" t="inlineStr">
+        <is>
+          <t>Sprawdź stabilność roweru i blokadę regulacji; Ustaw siodełko tak, aby kolano pozostało lekko ugięte przy najdalszym położeniu pedału, biodra nie kołysały się; Ustaw kierownicę w wygodnym zasięgu, rozluźnij barki i lekko oprzyj dłonie; Zacznij od kilku minut bardzo lekkiego pedałowania z małym oporem; Pedałuj płynnie w siadzie, kolana prowadź zgodnie z kierunkiem stóp; Dobierz tempo i opór tak, by swobodnie rozmawiać pełnymi zdaniami, bez zadyszki; Oddychaj swobodnie, zakończ kilkoma minutami coraz lżejszej jazdy i zatrzymaj pedały przed zejściem; Przerwij przy bólu kolan, bólu w klatce, zawrotach głowy lub nietypowej duszności</t>
+        </is>
+      </c>
+      <c r="M413" s="19" t="inlineStr">
+        <is>
+          <t>Zbyt niskie siodełko; Blokowanie kolan lub kołysanie bioder; Wysoki opór i zadyszka zamiast spokojnej jazdy; Wstrzymywanie oddechu; Zsiadanie przy obracających się pedałach</t>
+        </is>
+      </c>
+      <c r="N413" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw stopniowo wydłużaj komfortową jazdę o kilka minut; dopiero później nieznacznie zwiększ opór, nadal zachowując swobodną rozmowę</t>
+        </is>
+      </c>
+      <c r="O413" s="19" t="inlineStr">
+        <is>
+          <t>Krótsza jazda, mniejszy opór i spokojniejsze tempo; zrób przerwę przed pogorszeniem techniki</t>
+        </is>
+      </c>
+      <c r="P413" s="19" t="inlineStr">
+        <is>
+          <t>https://www.arthritis.org/health-wellness/healthy-living/physical-activity/other-activities/benefits-of-stationary-biking</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add owner equipment exercises; release 1.23.0+39
Preserve the 412-row raw catalog prefix and user history; add explicit gear alternatives and six scoped corrections. Align Apple Health ORM constraints with migration 0008 without changing the database schema.
</commit_message>
<xml_diff>
--- a/tools/source_data/baza_cwiczen_316.xlsx
+++ b/tools/source_data/baza_cwiczen_316.xlsx
@@ -8445,7 +8445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P413"/>
+  <dimension ref="A1:P425"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.8515625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.00390625" customWidth="1" style="39" min="1" max="1"/>
@@ -41500,6 +41500,966 @@
       <c r="P413" s="19" t="inlineStr">
         <is>
           <t>https://www.arthritis.org/health-wellness/healthy-living/physical-activity/other-activities/benefits-of-stationary-biking</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="19" t="n">
+        <v>413</v>
+      </c>
+      <c r="B414" s="19" t="inlineStr">
+        <is>
+          <t>Wejście bokiem na step</t>
+        </is>
+      </c>
+      <c r="C414" s="19" t="inlineStr">
+        <is>
+          <t>Lateral step-up</t>
+        </is>
+      </c>
+      <c r="D414" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E414" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Łydki</t>
+        </is>
+      </c>
+      <c r="F414" s="19" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="G414" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H414" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I414" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J414" s="19" t="inlineStr">
+        <is>
+          <t>2 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K414" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L414" s="19" t="inlineStr">
+        <is>
+          <t>Sprawdź stabilność i blokadę podstawy stepu na nieśliskim podłożu; Wysokość stepu właściciela jest niezmierzona, deklarowane 150 kg nie jest zweryfikowaną nośnością; Wybierz niskie ustawienie pozwalające zachować kontrolę, bez narzucania wysokości; Stań bokiem przy stepie, bliższą stopę ustaw w całości na platformie; Kolano prowadź w kierunku palców; Unieś tułów pracą nogi na stepie, bez wybicia z podłogi; Dostaw drugą stopę i zejdź powoli w tej samej kolejności; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M414" s="19" t="inlineStr">
+        <is>
+          <t>Kolano zapadające do środka; Odbijanie nogą z podłogi; Zeskakiwanie</t>
+        </is>
+      </c>
+      <c r="N414" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw dodaj kontrolowane powtórzenia z niezmienioną wysokością</t>
+        </is>
+      </c>
+      <c r="O414" s="19" t="inlineStr">
+        <is>
+          <t>Niższe ustawienie i mniej powtórzeń, z odpoczynkiem przed utratą kontroli</t>
+        </is>
+      </c>
+      <c r="P414" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/pros/expert-articles/6369/back-to-the-basics-how-to-create-innovative-fitness-programs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="19" t="n">
+        <v>414</v>
+      </c>
+      <c r="B415" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowane zejście ze stepu</t>
+        </is>
+      </c>
+      <c r="C415" s="19" t="inlineStr">
+        <is>
+          <t>Controlled step-down</t>
+        </is>
+      </c>
+      <c r="D415" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E415" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="F415" s="19" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="G415" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H415" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I415" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J415" s="19" t="inlineStr">
+        <is>
+          <t>2 x 6-10 na stronę</t>
+        </is>
+      </c>
+      <c r="K415" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L415" s="19" t="inlineStr">
+        <is>
+          <t>Sprawdź stabilność i blokadę podstawy stepu na nieśliskim podłożu; Wysokość stepu właściciela jest niezmierzona, deklarowane 150 kg nie jest zweryfikowaną nośnością; Wybierz niskie ustawienie pozwalające zachować kontrolę, bez narzucania wysokości; Stań stabilnie na stepie z całą stopą nogi podporowej na platformie; Powoli ugnij biodro i kolano nogi podporowej, opuszczając drugą piętę do lekkiego dotknięcia podłogi przed stepem; Zachowaj miednicę poziomo i kolano w linii stopy; Po dotknięciu piętą spokojnie przenieś ciężar na podłogę i zakończ zejście; Następnie wejdź ponownie na step, ustaw się stabilnie i rozpocznij kolejne kontrolowane zejście; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M415" s="19" t="inlineStr">
+        <is>
+          <t>Spadanie na podłogę; Zapadanie kolana; Przechylanie miednicy; Gwałtowne odbicie zamiast spokojnego zejścia i ponownego ustawienia</t>
+        </is>
+      </c>
+      <c r="N415" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż kontrolowaną fazę opuszczania lub dodaj powtórzenia, nie skoki</t>
+        </is>
+      </c>
+      <c r="O415" s="19" t="inlineStr">
+        <is>
+          <t>Niższy step i krótszy kontrolowany zakres</t>
+        </is>
+      </c>
+      <c r="P415" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/pros/expert-articles/5901/effective-exercises-to-target-the-glutes/</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="19" t="n">
+        <v>415</v>
+      </c>
+      <c r="B416" s="19" t="inlineStr">
+        <is>
+          <t>Pompki z dłońmi na stepie</t>
+        </is>
+      </c>
+      <c r="C416" s="19" t="inlineStr">
+        <is>
+          <t>Hands-elevated step push-up</t>
+        </is>
+      </c>
+      <c r="D416" s="19" t="inlineStr">
+        <is>
+          <t>Klatka piersiowa</t>
+        </is>
+      </c>
+      <c r="E416" s="19" t="inlineStr">
+        <is>
+          <t>Triceps, Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F416" s="19" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="G416" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H416" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I416" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J416" s="19" t="inlineStr">
+        <is>
+          <t>2 x 6-10</t>
+        </is>
+      </c>
+      <c r="K416" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L416" s="19" t="inlineStr">
+        <is>
+          <t>Sprawdź stabilność i blokadę podstawy stepu na nieśliskim podłożu; Wysokość stepu właściciela jest niezmierzona, deklarowane 150 kg nie jest zweryfikowaną nośnością; Wybierz niskie ustawienie pozwalające zachować kontrolę, bez narzucania wysokości; Oprzyj dłonie stabilnie na platformie stepu nieco szerzej niż barki, stopy na podłodze; Utrzymaj tułów i biodra w jednej linii; Ugnij łokcie ukośnie w tył i zbliż klatkę do stepu; Odepchnij się bez zapadania lędźwi; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M416" s="19" t="inlineStr">
+        <is>
+          <t>Ślizgający się step; Zapadanie bioder; Łokcie szeroko na boki; Stopy zamiast dłoni na stepie</t>
+        </is>
+      </c>
+      <c r="N416" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj poprawne powtórzenia; później wybierz trudniejszą pompkę na podłodze jako osobny wariant</t>
+        </is>
+      </c>
+      <c r="O416" s="19" t="inlineStr">
+        <is>
+          <t>Mniej powtórzeń; łatwiejszy wariant z dłońmi na wyższej, stabilnej podporze</t>
+        </is>
+      </c>
+      <c r="P416" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/pros/expert-articles/5808/strength-and-cardio-circuit-for-beginning-clients/</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="19" t="n">
+        <v>416</v>
+      </c>
+      <c r="B417" s="19" t="inlineStr">
+        <is>
+          <t>Spięcia brzucha na ławce głową w dół</t>
+        </is>
+      </c>
+      <c r="C417" s="19" t="inlineStr">
+        <is>
+          <t>Decline bench crunch</t>
+        </is>
+      </c>
+      <c r="D417" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="E417" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F417" s="19" t="inlineStr">
+        <is>
+          <t>Ławka do brzuszków</t>
+        </is>
+      </c>
+      <c r="G417" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H417" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I417" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J417" s="19" t="inlineStr">
+        <is>
+          <t>2 x 6-10</t>
+        </is>
+      </c>
+      <c r="K417" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L417" s="19" t="inlineStr">
+        <is>
+          <t>Sprawdź stabilność ławki do brzuszków, blokadę skosu i pewne zabezpieczenie nóg; Zacznij od łagodnego skosu głową w dół, bez dodatkowego ciężaru; Połóż się z podpartymi plecami i lekko ugiętymi kolanami; Skrzyżuj ręce na klatce; Z wydechem unieś tylko głowę i łopatki, zbliżając żebra do miednicy; Powoli odłóż łopatki, nie przechodź do pełnego siadu; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M417" s="19" t="inlineStr">
+        <is>
+          <t>Ciągnięcie głowy rękami; Zamach; Pełny siad zamiast spięcia; Wstrzymywanie oddechu</t>
+        </is>
+      </c>
+      <c r="N417" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj kontrolowane powtórzenia i krótką pauzę w spięciu, bez dokładania ciężaru</t>
+        </is>
+      </c>
+      <c r="O417" s="19" t="inlineStr">
+        <is>
+          <t>Mniejszy skos lub krótszy zakres; jeśli pozycja głową w dół jest źle tolerowana, wybierz spięcia na podłodze</t>
+        </is>
+      </c>
+      <c r="P417" s="19" t="inlineStr">
+        <is>
+          <t>https://exrx.net/WeightExercises/RectusAbdominis/BWInclineCrunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="19" t="n">
+        <v>417</v>
+      </c>
+      <c r="B418" s="19" t="inlineStr">
+        <is>
+          <t>Pełne brzuszki na ławce głową w dół</t>
+        </is>
+      </c>
+      <c r="C418" s="19" t="inlineStr">
+        <is>
+          <t>Decline bench sit-up</t>
+        </is>
+      </c>
+      <c r="D418" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder, Brzuch</t>
+        </is>
+      </c>
+      <c r="E418" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F418" s="19" t="inlineStr">
+        <is>
+          <t>Ławka do brzuszków</t>
+        </is>
+      </c>
+      <c r="G418" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H418" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I418" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J418" s="19" t="inlineStr">
+        <is>
+          <t>2 x 6-10</t>
+        </is>
+      </c>
+      <c r="K418" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L418" s="19" t="inlineStr">
+        <is>
+          <t>Sprawdź stabilność ławki do brzuszków, blokadę skosu i pewne zabezpieczenie nóg; Zacznij od łagodnego skosu głową w dół, bez dodatkowego ciężaru; Połóż plecy na ławce, ręce skrzyżuj na klatce; Najpierw zbliż żebra do miednicy, potem zegnij biodra i unieś tułów do siadu w wygodnym zakresie; Opuszczaj tułów powoli aż plecy znów będą podparte; Nie szarp nogami o blokadę; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M418" s="19" t="inlineStr">
+        <is>
+          <t>Zamach ramion; Gwałtowne odchylanie głowy; Zrzucanie tułowia; Zbyt duży skos</t>
+        </is>
+      </c>
+      <c r="N418" s="19" t="inlineStr">
+        <is>
+          <t>Zwiększ liczbę płynnych powtórzeń, nie obciążenie ani głębokość skosu za wszelką cenę</t>
+        </is>
+      </c>
+      <c r="O418" s="19" t="inlineStr">
+        <is>
+          <t>Mniejszy skos i mniej powtórzeń; wybierz samo spięcie brzucha, jeśli pełny siad traci kontrolę</t>
+        </is>
+      </c>
+      <c r="P418" s="19" t="inlineStr">
+        <is>
+          <t>https://exrx.net/WeightExercises/HipFlexors/WtDeclineSitup</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="19" t="n">
+        <v>418</v>
+      </c>
+      <c r="B419" s="19" t="inlineStr">
+        <is>
+          <t>Wyciskanie hantli na ławce głową w dół</t>
+        </is>
+      </c>
+      <c r="C419" s="19" t="inlineStr">
+        <is>
+          <t>Dumbbell decline bench press</t>
+        </is>
+      </c>
+      <c r="D419" s="19" t="inlineStr">
+        <is>
+          <t>Klatka piersiowa</t>
+        </is>
+      </c>
+      <c r="E419" s="19" t="inlineStr">
+        <is>
+          <t>Triceps, Barki</t>
+        </is>
+      </c>
+      <c r="F419" s="19" t="inlineStr">
+        <is>
+          <t>Ławka ujemna do wyciskania, Hantle</t>
+        </is>
+      </c>
+      <c r="G419" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H419" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I419" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J419" s="19" t="inlineStr">
+        <is>
+          <t>2 x 6-10</t>
+        </is>
+      </c>
+      <c r="K419" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L419" s="19" t="inlineStr">
+        <is>
+          <t>Wymagana jest osobno potwierdzona ławka ujemna przeznaczona do wyciskania z obciążeniem; Ławka właściciela do brzuszków ma niezweryfikowaną nośność do hantli: sama deklaracja przydatności nie wystarcza, nie wykonuj na niej tego ruchu bez potwierdzenia producenta; Sprawdź limit łącznej masy ciała i hantli, stabilność, blokadę skosu oraz zabezpieczenie nóg; Ustal bezpieczne podanie i odebranie lekkich hantli, w razie potrzeby z asekuracją; Połóż się z podpartą głową, plecami i pośladkami; Prowadź hantle po bokach klatki, nadgarstki nad łokciami; Wyciskaj płynnie nad klatkę i opuszczaj bez odbicia; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M419" s="19" t="inlineStr">
+        <is>
+          <t>Użycie niezweryfikowanej ławki do brzuszków; Brak bezpiecznego odłożenia; Zrzucanie hantli; Nadmierny skos; Wstrzymywanie oddechu</t>
+        </is>
+      </c>
+      <c r="N419" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw popraw kontrolę i powtórzenia; dopiero na zweryfikowanym sprzęcie rozważ najmniejszy przyrost obciążenia</t>
+        </is>
+      </c>
+      <c r="O419" s="19" t="inlineStr">
+        <is>
+          <t>Lżejsze hantle i mniejszy zatwierdzony skos; bez właściwej ławki wybierz inne ćwiczenie</t>
+        </is>
+      </c>
+      <c r="P419" s="19" t="inlineStr">
+        <is>
+          <t>https://exrx.net/WeightExercises/PectoralSternal/DBDeclineBenchPress</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="19" t="n">
+        <v>419</v>
+      </c>
+      <c r="B420" s="19" t="inlineStr">
+        <is>
+          <t>Stanie obunóż na poduszce równoważnej</t>
+        </is>
+      </c>
+      <c r="C420" s="19" t="inlineStr">
+        <is>
+          <t>Double-leg balance cushion stand</t>
+        </is>
+      </c>
+      <c r="D420" s="19" t="inlineStr">
+        <is>
+          <t>Mięśnie stóp, Łydki</t>
+        </is>
+      </c>
+      <c r="E420" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F420" s="19" t="inlineStr">
+        <is>
+          <t>Poduszka równoważna</t>
+        </is>
+      </c>
+      <c r="G420" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H420" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I420" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J420" s="19" t="inlineStr">
+        <is>
+          <t>2 x 15-30 sek</t>
+        </is>
+      </c>
+      <c r="K420" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L420" s="19" t="inlineStr">
+        <is>
+          <t>Połóż poduszkę na nieśliskiej podłodze obok stabilnego podparcia awaryjnego; Wejdź ostrożnie i ustaw obie stopy na poduszce; Utrzymuj miękkie kolana, wzrok na nieruchomym punkcie i spokojny oddech; Zejdź przed utratą równowagi; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M420" s="19" t="inlineStr">
+        <is>
+          <t>Zamykanie oczu na początku; Blokowanie kolan; Ustawienie przy przeszkodach; Kontynuowanie mimo utraty równowagi</t>
+        </is>
+      </c>
+      <c r="N420" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo wydłuż spokojne stanie z otwartymi oczami</t>
+        </is>
+      </c>
+      <c r="O420" s="19" t="inlineStr">
+        <is>
+          <t>Krótsze próby lub stanie na stabilnej podłodze</t>
+        </is>
+      </c>
+      <c r="P420" s="19" t="inlineStr">
+        <is>
+          <t>https://www.togu.de/en/blog/pelvic-floor-training-with-the-dynair-ballkissen</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="19" t="n">
+        <v>420</v>
+      </c>
+      <c r="B421" s="19" t="inlineStr">
+        <is>
+          <t>Stanie jednonóż na poduszce równoważnej</t>
+        </is>
+      </c>
+      <c r="C421" s="19" t="inlineStr">
+        <is>
+          <t>Single-leg balance cushion stand</t>
+        </is>
+      </c>
+      <c r="D421" s="19" t="inlineStr">
+        <is>
+          <t>Mięśnie stóp, Łydki</t>
+        </is>
+      </c>
+      <c r="E421" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F421" s="19" t="inlineStr">
+        <is>
+          <t>Poduszka równoważna</t>
+        </is>
+      </c>
+      <c r="G421" s="19" t="inlineStr">
+        <is>
+          <t>Izometria</t>
+        </is>
+      </c>
+      <c r="H421" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I421" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J421" s="19" t="inlineStr">
+        <is>
+          <t>2 x 15-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K421" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L421" s="19" t="inlineStr">
+        <is>
+          <t>Ustaw poduszkę na nieśliskiej podłodze blisko stabilnego podparcia awaryjnego; Ustaw stopę podporową na środku i lekko ugnij kolano; Ostrożnie unieś drugą stopę, utrzymuj miednicę poziomo i patrz przed siebie; Odstaw stopę natychmiast przy utracie kontroli; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M421" s="19" t="inlineStr">
+        <is>
+          <t>Zapadanie kolana; Przechylanie miednicy; Zamykanie oczu; Ryzyko upadku przy zbyt długiej próbie</t>
+        </is>
+      </c>
+      <c r="N421" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż krótkie stabilne próby z otwartymi oczami, bez dodawania ciężaru</t>
+        </is>
+      </c>
+      <c r="O421" s="19" t="inlineStr">
+        <is>
+          <t>Stanie obunóż na poduszce lub jednonóż na stabilnej podłodze</t>
+        </is>
+      </c>
+      <c r="P421" s="19" t="inlineStr">
+        <is>
+          <t>https://www.togu.de/en/blog/pelvic-floor-training-with-the-dynair-ballkissen</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="19" t="n">
+        <v>421</v>
+      </c>
+      <c r="B422" s="19" t="inlineStr">
+        <is>
+          <t>Rolowanie łydki</t>
+        </is>
+      </c>
+      <c r="C422" s="19" t="inlineStr">
+        <is>
+          <t>Calf foam rolling</t>
+        </is>
+      </c>
+      <c r="D422" s="19" t="inlineStr">
+        <is>
+          <t>Łydki</t>
+        </is>
+      </c>
+      <c r="E422" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F422" s="19" t="inlineStr">
+        <is>
+          <t>Roller</t>
+        </is>
+      </c>
+      <c r="G422" s="19" t="inlineStr">
+        <is>
+          <t>Regeneracja</t>
+        </is>
+      </c>
+      <c r="H422" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I422" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J422" s="19" t="inlineStr">
+        <is>
+          <t>2 x 15-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K422" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L422" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź na podłodze, roller umieść pod miękką częścią łydki, drugą stopę i dłonie oprzyj dla kontroli nacisku; Powoli przesuwaj łydkę po rollerze na krótkim odcinku; Omijaj dół podkolanowy, kostki i ścięgno Achillesa; Nacisk ma być łagodny i tolerowany, nie walcz z bólem; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M422" s="19" t="inlineStr">
+        <is>
+          <t>Nacisk na staw lub ścięgno; Szybkie ruchy; Silny ból; Wstrzymywanie oddechu</t>
+        </is>
+      </c>
+      <c r="N422" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż łagodne rolowanie do komfortowego czasu, nie zwiększaj nacisku przez ból</t>
+        </is>
+      </c>
+      <c r="O422" s="19" t="inlineStr">
+        <is>
+          <t>Więcej ciężaru na stopie i dłoniach, krótszy odcinek i czas</t>
+        </is>
+      </c>
+      <c r="P422" s="19" t="inlineStr">
+        <is>
+          <t>https://contentcdn.eacefitness.com/certifiednews/images/article/pdfs/MyofascialRelease.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="19" t="n">
+        <v>422</v>
+      </c>
+      <c r="B423" s="19" t="inlineStr">
+        <is>
+          <t>Rolowanie przedniej części uda</t>
+        </is>
+      </c>
+      <c r="C423" s="19" t="inlineStr">
+        <is>
+          <t>Quadriceps foam rolling</t>
+        </is>
+      </c>
+      <c r="D423" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda</t>
+        </is>
+      </c>
+      <c r="E423" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F423" s="19" t="inlineStr">
+        <is>
+          <t>Roller</t>
+        </is>
+      </c>
+      <c r="G423" s="19" t="inlineStr">
+        <is>
+          <t>Regeneracja</t>
+        </is>
+      </c>
+      <c r="H423" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I423" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J423" s="19" t="inlineStr">
+        <is>
+          <t>2 x 15-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K423" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L423" s="19" t="inlineStr">
+        <is>
+          <t>Połóż przód uda na rollerze i podeprzyj tułów na przedramionach; Drugą nogą reguluj nacisk; Powoli przesuwaj miękką część uda po rollerze, bez dociskania pachwiny i rzepki; Utrzymuj spokojny oddech i łagodny nacisk; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M423" s="19" t="inlineStr">
+        <is>
+          <t>Rolowanie po kolanie; Zbyt silny nacisk; Zapadanie lędźwi; Szybkie przejazdy</t>
+        </is>
+      </c>
+      <c r="N423" s="19" t="inlineStr">
+        <is>
+          <t>Stopniowo wydłuż komfortowy czas, bez forsowania nacisku</t>
+        </is>
+      </c>
+      <c r="O423" s="19" t="inlineStr">
+        <is>
+          <t>Odciąż nogę podporową, skróć zakres i czas</t>
+        </is>
+      </c>
+      <c r="P423" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/about-ace/our-efforts/blog/7786/foam-rollers-should-you-use-them/</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="19" t="n">
+        <v>423</v>
+      </c>
+      <c r="B424" s="19" t="inlineStr">
+        <is>
+          <t>Rolowanie pośladka</t>
+        </is>
+      </c>
+      <c r="C424" s="19" t="inlineStr">
+        <is>
+          <t>Glute foam rolling</t>
+        </is>
+      </c>
+      <c r="D424" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki</t>
+        </is>
+      </c>
+      <c r="E424" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F424" s="19" t="inlineStr">
+        <is>
+          <t>Roller</t>
+        </is>
+      </c>
+      <c r="G424" s="19" t="inlineStr">
+        <is>
+          <t>Regeneracja</t>
+        </is>
+      </c>
+      <c r="H424" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I424" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J424" s="19" t="inlineStr">
+        <is>
+          <t>2 x 15-30 sek na stronę</t>
+        </is>
+      </c>
+      <c r="K424" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L424" s="19" t="inlineStr">
+        <is>
+          <t>Usiądź na rollerze z dłońmi i stopami opartymi stabilnie; Lekko przenieś nacisk na jeden pośladek, drugą stopą reguluj obciążenie; Wykonuj małe powolne przesunięcia po miękkiej części pośladka; Omijaj kości i przerwij przy promieniowaniu lub drętwieniu; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M424" s="19" t="inlineStr">
+        <is>
+          <t>Ucisk kości; Silny ból; Szybkie kołysanie; Ignorowanie drętwienia</t>
+        </is>
+      </c>
+      <c r="N424" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż łagodne kontrolowane rolowanie, bez wymuszania większego nacisku</t>
+        </is>
+      </c>
+      <c r="O424" s="19" t="inlineStr">
+        <is>
+          <t>Więcej podparcia na stopach i dłoniach oraz krótszy czas</t>
+        </is>
+      </c>
+      <c r="P424" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/pros/expert-articles/5895/recover-faster-and-more-effectively-with-these-foam-roller-moves/</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="19" t="n">
+        <v>424</v>
+      </c>
+      <c r="B425" s="19" t="inlineStr">
+        <is>
+          <t>Chód z sandbagiem objętym przed tułowiem</t>
+        </is>
+      </c>
+      <c r="C425" s="19" t="inlineStr">
+        <is>
+          <t>Bear-hug sandbag carry</t>
+        </is>
+      </c>
+      <c r="D425" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Plecy</t>
+        </is>
+      </c>
+      <c r="E425" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki, Przód uda, Przedramiona</t>
+        </is>
+      </c>
+      <c r="F425" s="19" t="inlineStr">
+        <is>
+          <t>Sandbag</t>
+        </is>
+      </c>
+      <c r="G425" s="19" t="inlineStr">
+        <is>
+          <t>Wytrzymałość</t>
+        </is>
+      </c>
+      <c r="H425" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I425" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J425" s="19" t="inlineStr">
+        <is>
+          <t>2 x 15-30 sek</t>
+        </is>
+      </c>
+      <c r="K425" s="19" t="inlineStr">
+        <is>
+          <t>Wolno i płynnie, bez odbicia</t>
+        </is>
+      </c>
+      <c r="L425" s="19" t="inlineStr">
+        <is>
+          <t>Sprawdź zamknięcia worka i wolną płaską trasę bez przeszkód; Dobierz masę pozwalającą bezpiecznie podnieść, objąć i odłożyć worek, bez szarpania; Obejmij worek przed tułowiem, blisko klatki, nie zaciskaj szyi; Idź małymi spokojnymi krokami z wyprostowanym tułowiem i swobodnym oddechem; Odłóż worek kontrolowanie pracą bioder i kolan; Worek właściciela pozostaje operacyjnie przy 20 kg, to nie uniwersalny cel: jeśli za ciężki, nie wykonuj ruchu; Oddychaj swobodnie; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M425" s="19" t="inlineStr">
+        <is>
+          <t>Odchylanie tułowia w tył; Zasłonięta trasa; Wstrzymywanie oddechu; Zrzucanie worka; Schody lub step z workiem</t>
+        </is>
+      </c>
+      <c r="N425" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw wydłuż krótki odcinek lub czas przy tej samej komfortowej masie; nie dokładaj obciążenia</t>
+        </is>
+      </c>
+      <c r="O425" s="19" t="inlineStr">
+        <is>
+          <t>Krótszy odcinek lub lżejszy worek, jeśli dostępny; gdy posiadany worek jest za ciężki, wybierz inny ruch</t>
+        </is>
+      </c>
+      <c r="P425" s="19" t="inlineStr">
+        <is>
+          <t>https://ultimatesandbagtraining.com/best-secret-great-ultimate-sandbag-workouts/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add seven basic bodyweight catalog movements
</commit_message>
<xml_diff>
--- a/tools/source_data/baza_cwiczen_316.xlsx
+++ b/tools/source_data/baza_cwiczen_316.xlsx
@@ -8445,7 +8445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P425"/>
+  <dimension ref="A1:P432"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.8515625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.00390625" customWidth="1" style="39" min="1" max="1"/>
@@ -42460,6 +42460,566 @@
       <c r="P425" s="19" t="inlineStr">
         <is>
           <t>https://ultimatesandbagtraining.com/best-secret-great-ultimate-sandbag-workouts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="19" t="n">
+        <v>425</v>
+      </c>
+      <c r="B426" s="19" t="inlineStr">
+        <is>
+          <t>Pompki od ściany</t>
+        </is>
+      </c>
+      <c r="C426" s="19" t="inlineStr">
+        <is>
+          <t>Wall push-up</t>
+        </is>
+      </c>
+      <c r="D426" s="19" t="inlineStr">
+        <is>
+          <t>Klatka piersiowa</t>
+        </is>
+      </c>
+      <c r="E426" s="19" t="inlineStr">
+        <is>
+          <t>Triceps, Barki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F426" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G426" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H426" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I426" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J426" s="19" t="inlineStr">
+        <is>
+          <t>1-2 x 5-8</t>
+        </is>
+      </c>
+      <c r="K426" s="19" t="inlineStr">
+        <is>
+          <t>Około 2 sek ruchu w każdą stronę, bez zamachu</t>
+        </is>
+      </c>
+      <c r="L426" s="19" t="inlineStr">
+        <is>
+          <t>Stań twarzą do stabilnej ściany mniej więcej na odległość ramion, na nieśliskiej podłodze; Oprzyj dłonie na wysokości klatki, palce skieruj w górę; Utrzymaj tułów i biodra w jednej linii, stopy pozostają na podłodze; Powoli zegnij łokcie blisko boków i przybliż klatkę do ściany w wygodnym zakresie; Odepchnij się płynnie do pozycji wyjściowej; Oddychaj swobodnie; Zakończ serię przed utratą kontroli; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M426" s="19" t="inlineStr">
+        <is>
+          <t>Ślizgające się dłonie lub stopy; Zapadanie bioder; Wysuwanie samej głowy; Gwałtowne odbicie</t>
+        </is>
+      </c>
+      <c r="N426" s="19" t="inlineStr">
+        <is>
+          <t>Najpierw dodaj płynne powtórzenia, potem odsuń stopy nieznacznie dalej przy zachowanej stabilności</t>
+        </is>
+      </c>
+      <c r="O426" s="19" t="inlineStr">
+        <is>
+          <t>Stań bliżej ściany i zmniejsz zakres oraz liczbę powtórzeń</t>
+        </is>
+      </c>
+      <c r="P426" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/live-well/exercise/strength-and-flexibility-exercises/strength-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="19" t="n">
+        <v>426</v>
+      </c>
+      <c r="B427" s="19" t="inlineStr">
+        <is>
+          <t>Przysiad bez obciążenia</t>
+        </is>
+      </c>
+      <c r="C427" s="19" t="inlineStr">
+        <is>
+          <t>Bodyweight squat</t>
+        </is>
+      </c>
+      <c r="D427" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E427" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch</t>
+        </is>
+      </c>
+      <c r="F427" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G427" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H427" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I427" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J427" s="19" t="inlineStr">
+        <is>
+          <t>1-2 x 5-8</t>
+        </is>
+      </c>
+      <c r="K427" s="19" t="inlineStr">
+        <is>
+          <t>Około 2 sek ruchu w każdą stronę, bez zamachu</t>
+        </is>
+      </c>
+      <c r="L427" s="19" t="inlineStr">
+        <is>
+          <t>Stań stabilnie ze stopami nieco szerzej niż biodra, palce lekko na zewnątrz; Ręce wysuń przed siebie bez opierania ich na sprzęcie; Cofnij biodra i powoli ugnij biodra oraz kolana, prowadząc kolana zgodnie z kierunkiem stóp; Zejdź tylko tak nisko, by całe stopy pozostały oparte, a plecy zachowały kontrolowaną pozycję; Naciśnij stopami podłoże i wyprostuj biodra oraz kolana bez szarpania; Oddychaj swobodnie; Zakończ serię przed utratą kontroli; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M427" s="19" t="inlineStr">
+        <is>
+          <t>Odrywanie pięt; Zapadanie kolan; Wymuszanie głębokości; Opadanie tułowia bez kontroli</t>
+        </is>
+      </c>
+      <c r="N427" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj powtórzenia lub stopniowo większy kontrolowany zakres bez obciążenia</t>
+        </is>
+      </c>
+      <c r="O427" s="19" t="inlineStr">
+        <is>
+          <t>Płytszy przysiad i mniej powtórzeń, bez wymuszania zejścia do równoległości</t>
+        </is>
+      </c>
+      <c r="P427" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/everyone/exercise-library/135/bodyweight-squat/</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="19" t="n">
+        <v>427</v>
+      </c>
+      <c r="B428" s="19" t="inlineStr">
+        <is>
+          <t>Zakroki bez obciążenia</t>
+        </is>
+      </c>
+      <c r="C428" s="19" t="inlineStr">
+        <is>
+          <t>Bodyweight reverse lunge</t>
+        </is>
+      </c>
+      <c r="D428" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki</t>
+        </is>
+      </c>
+      <c r="E428" s="19" t="inlineStr">
+        <is>
+          <t>Tył uda, Brzuch</t>
+        </is>
+      </c>
+      <c r="F428" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G428" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H428" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I428" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J428" s="19" t="inlineStr">
+        <is>
+          <t>1-2 x 5-8 na stronę</t>
+        </is>
+      </c>
+      <c r="K428" s="19" t="inlineStr">
+        <is>
+          <t>Około 2 sek ruchu w każdą stronę, bez zamachu</t>
+        </is>
+      </c>
+      <c r="L428" s="19" t="inlineStr">
+        <is>
+          <t>Stań ze stopami na szerokość bioder i wolnym miejscem za sobą, bez ciężaru w dłoniach; Cofnij jedną stopę i oprzyj jej przodostopie, zachowując odstęp między stopami na boki; Powoli ugnij obie nogi, przednie kolano prowadź w kierunku palców; Tylne kolano pozostaje nad podłogą przez cały ruch, nie klękaj; Naciśnij całą przednią stopą podłoże i wróć do stania bez odbicia; Wykonaj krótką serię na jedną stronę, potem zmień nogę; Oddychaj swobodnie; Zakończ serię przed utratą kontroli; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M428" s="19" t="inlineStr">
+        <is>
+          <t>Stopy na jednej wąskiej linii; Opadanie kolana na podłogę; Zapadanie przedniego kolana; Zamach tułowiem</t>
+        </is>
+      </c>
+      <c r="N428" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj kontrolowane powtórzenia na stronę lub nieco zwiększ komfortowy zakres</t>
+        </is>
+      </c>
+      <c r="O428" s="19" t="inlineStr">
+        <is>
+          <t>Krótszy krok i płytsze ugięcie; jeśli nie utrzymujesz równowagi bez podparcia, wybierz inne ćwiczenie</t>
+        </is>
+      </c>
+      <c r="P428" s="19" t="inlineStr">
+        <is>
+          <t>https://www.acefitness.org/resources/everyone/exercise-library/319/reverse-lunge/</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="19" t="n">
+        <v>428</v>
+      </c>
+      <c r="B429" s="19" t="inlineStr">
+        <is>
+          <t>Marsz w miejscu</t>
+        </is>
+      </c>
+      <c r="C429" s="19" t="inlineStr">
+        <is>
+          <t>March in place</t>
+        </is>
+      </c>
+      <c r="D429" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder, Łydki</t>
+        </is>
+      </c>
+      <c r="E429" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Pośladki, Brzuch</t>
+        </is>
+      </c>
+      <c r="F429" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G429" s="19" t="inlineStr">
+        <is>
+          <t>Rozgrzewka</t>
+        </is>
+      </c>
+      <c r="H429" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I429" s="19" t="inlineStr">
+        <is>
+          <t>Marsz naprzemienny</t>
+        </is>
+      </c>
+      <c r="J429" s="19" t="inlineStr">
+        <is>
+          <t>1-2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K429" s="19" t="inlineStr">
+        <is>
+          <t>Spokojny równy rytm, bez podskoków</t>
+        </is>
+      </c>
+      <c r="L429" s="19" t="inlineStr">
+        <is>
+          <t>Stań na równym nieśliskim podłożu z wolnym miejscem wokół; Naprzemiennie unoś stopę niewysoko i odkładaj ją cicho pod biodrem; Zachowaj wyprostowany tułów, wzrok przed sobą i spokojny oddech; Poruszaj swobodnie lekko ugiętymi ramionami w rytmie kroków; Pozostawaj w miejscu, bez podskoków i bez wymuszania wysokiego unoszenia kolan; Oddychaj swobodnie; Zakończ serię przed utratą kontroli; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M429" s="19" t="inlineStr">
+        <is>
+          <t>Podskakiwanie; Głośne tupanie; Odchylanie tułowia; Zbyt szybki rytm utrudniający swobodną rozmowę</t>
+        </is>
+      </c>
+      <c r="N429" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż krótki odcinek marszu przy rytmie pozwalającym swobodnie rozmawiać</t>
+        </is>
+      </c>
+      <c r="O429" s="19" t="inlineStr">
+        <is>
+          <t>Niższe unoszenie stóp, wolniejszy rytm i krótszy czas z przerwą</t>
+        </is>
+      </c>
+      <c r="P429" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/live-well/exercise/how-to-warm-up-before-exercising/</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="19" t="n">
+        <v>429</v>
+      </c>
+      <c r="B430" s="19" t="inlineStr">
+        <is>
+          <t>Marsz w siadzie</t>
+        </is>
+      </c>
+      <c r="C430" s="19" t="inlineStr">
+        <is>
+          <t>Seated march</t>
+        </is>
+      </c>
+      <c r="D430" s="19" t="inlineStr">
+        <is>
+          <t>Zginacze bioder</t>
+        </is>
+      </c>
+      <c r="E430" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda, Brzuch</t>
+        </is>
+      </c>
+      <c r="F430" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G430" s="19" t="inlineStr">
+        <is>
+          <t>Rozgrzewka</t>
+        </is>
+      </c>
+      <c r="H430" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I430" s="19" t="inlineStr">
+        <is>
+          <t>Marsz naprzemienny</t>
+        </is>
+      </c>
+      <c r="J430" s="19" t="inlineStr">
+        <is>
+          <t>1-2 x 20-30 sek</t>
+        </is>
+      </c>
+      <c r="K430" s="19" t="inlineStr">
+        <is>
+          <t>Spokojny równy rytm, bez podskoków</t>
+        </is>
+      </c>
+      <c r="L430" s="19" t="inlineStr">
+        <is>
+          <t>Wybierz stabilne krzesło bez kółek na nieśliskim podłożu, ze stopami opartymi płasko na podłodze; Usiądź prosto bez opierania pleców, chwyć lekko boki siedziska dla stabilności; Unieś jedną stopę niewysoko z ugiętym kolanem bez odchylania tułowia; Odstaw stopę łagodnie i powtórz drugą nogą; Kontynuuj naprzemiennie w spokojnym rytmie, bez szarpania krzesłem; Oddychaj swobodnie; Zakończ serię przed utratą kontroli; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M430" s="19" t="inlineStr">
+        <is>
+          <t>Odchylanie pleców; Wymuszanie wysokiego kolana; Tupanie; Kołysanie krzesłem</t>
+        </is>
+      </c>
+      <c r="N430" s="19" t="inlineStr">
+        <is>
+          <t>Wydłuż czas spokojnej naprzemiennej pracy bez przyspieszania</t>
+        </is>
+      </c>
+      <c r="O430" s="19" t="inlineStr">
+        <is>
+          <t>Unoś stopę minimalnie, skróć czas i odpocznij między próbami</t>
+        </is>
+      </c>
+      <c r="P430" s="19" t="inlineStr">
+        <is>
+          <t>https://www.nhs.uk/live-well/exercise/strength-and-flexibility-exercises/sitting-exercises/</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="19" t="n">
+        <v>430</v>
+      </c>
+      <c r="B431" s="19" t="inlineStr">
+        <is>
+          <t>Prostowanie kolana w siadzie bez gumy</t>
+        </is>
+      </c>
+      <c r="C431" s="19" t="inlineStr">
+        <is>
+          <t>Seated knee extension</t>
+        </is>
+      </c>
+      <c r="D431" s="19" t="inlineStr">
+        <is>
+          <t>Przód uda</t>
+        </is>
+      </c>
+      <c r="E431" s="19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F431" s="19" t="inlineStr">
+        <is>
+          <t>Krzesło</t>
+        </is>
+      </c>
+      <c r="G431" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H431" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I431" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J431" s="19" t="inlineStr">
+        <is>
+          <t>1-2 x 5-8 na stronę</t>
+        </is>
+      </c>
+      <c r="K431" s="19" t="inlineStr">
+        <is>
+          <t>Około 2 sek ruchu w każdą stronę, bez zamachu</t>
+        </is>
+      </c>
+      <c r="L431" s="19" t="inlineStr">
+        <is>
+          <t>Wybierz stabilne krzesło bez kółek na nieśliskim podłożu, ze stopami opartymi płasko na podłodze; Usiądź prosto, dłonie połóż swobodnie na udach bez podpierania ciężaru ciała; Trzymaj udo na siedzisku i powoli prostuj jedno kolano, unosząc stopę przed siebie, palce łagodnie przyciągnij ku goleni; Zatrzymaj ruch w wygodnym zakresie bez gwałtownego blokowania kolana; Powoli zegnij kolano i odstaw stopę; Po krótkiej serii zmień nogę, nie używaj gumy ani ciężarka; Oddychaj swobodnie; Zakończ serię przed utratą kontroli; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M431" s="19" t="inlineStr">
+        <is>
+          <t>Kopnięcie z zamachu; Odchylanie tułowia; Odrywanie uda; Wciskanie kolana na siłę w przeprost</t>
+        </is>
+      </c>
+      <c r="N431" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj kontrolowane powtórzenia lub krótką spokojną pauzę przy wyproście bez dodatkowego obciążenia</t>
+        </is>
+      </c>
+      <c r="O431" s="19" t="inlineStr">
+        <is>
+          <t>Mniejszy wygodny zakres i mniej powtórzeń na stronę</t>
+        </is>
+      </c>
+      <c r="P431" s="19" t="inlineStr">
+        <is>
+          <t>https://www.opalreturntowork.nhs.uk/exercises/seated-knee-extension/</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="19" t="n">
+        <v>431</v>
+      </c>
+      <c r="B432" s="19" t="inlineStr">
+        <is>
+          <t>Odwodzenie ugiętej nogi w bok w klęku podpartym bez gumy</t>
+        </is>
+      </c>
+      <c r="C432" s="19" t="inlineStr">
+        <is>
+          <t>Bodyweight fire hydrant</t>
+        </is>
+      </c>
+      <c r="D432" s="19" t="inlineStr">
+        <is>
+          <t>Pośladki</t>
+        </is>
+      </c>
+      <c r="E432" s="19" t="inlineStr">
+        <is>
+          <t>Brzuch, Barki</t>
+        </is>
+      </c>
+      <c r="F432" s="19" t="inlineStr">
+        <is>
+          <t>Masa własna</t>
+        </is>
+      </c>
+      <c r="G432" s="19" t="inlineStr">
+        <is>
+          <t>Siła</t>
+        </is>
+      </c>
+      <c r="H432" s="19" t="inlineStr">
+        <is>
+          <t>Początkujący</t>
+        </is>
+      </c>
+      <c r="I432" s="19" t="inlineStr">
+        <is>
+          <t>Kontrolowany ruch</t>
+        </is>
+      </c>
+      <c r="J432" s="19" t="inlineStr">
+        <is>
+          <t>1-2 x 5-8 na stronę</t>
+        </is>
+      </c>
+      <c r="K432" s="19" t="inlineStr">
+        <is>
+          <t>Około 2 sek ruchu w każdą stronę, bez zamachu</t>
+        </is>
+      </c>
+      <c r="L432" s="19" t="inlineStr">
+        <is>
+          <t>Ustaw dłonie pod barkami i kolana pod biodrami na równym wygodnym podłożu, bez gumy; Utrzymaj plecy spokojnie, brzuch lekko napięty i wzrok w dół; Zachowując ugięcie kolana około kąta prostego, unieś jedną nogę w bok małym ruchem w biodrze; Nie obracaj miednicy ani tułowia i nie unoś kolana wyżej niż około 45 stopni, mniejszy zakres jest wystarczający; Powoli odstaw kolano pod biodro i po krótkiej serii zmień stronę; Mata może zwiększyć komfort, ale nie jest wymagana; Oddychaj swobodnie; Zakończ serię przed utratą kontroli; Przerwij przy bólu, drętwieniu lub zawrotach głowy</t>
+        </is>
+      </c>
+      <c r="M432" s="19" t="inlineStr">
+        <is>
+          <t>Obracanie miednicy; Zapadanie lędźwi; Prostowanie kolana zamiast odwodzenia biodra; Wymuszanie wysokości</t>
+        </is>
+      </c>
+      <c r="N432" s="19" t="inlineStr">
+        <is>
+          <t>Dodaj płynne powtórzenia lub krótką pauzę przy zachowaniu nieruchomej miednicy</t>
+        </is>
+      </c>
+      <c r="O432" s="19" t="inlineStr">
+        <is>
+          <t>Zmniejsz zakres i liczbę powtórzeń; jeśli podpór lub klęk jest niewygodny, wybierz inne ćwiczenie</t>
+        </is>
+      </c>
+      <c r="P432" s="19" t="inlineStr">
+        <is>
+          <t>https://sportsrehab.ucsf.edu/sites/g/files/tkssra10961/files/doc/Core_Strengthening_Basics_Protocol_Nov2025.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>